<commit_message>
Ajouter le prêt d'honneur IQPH au classeur de financement
Initiative Québec Prêt d'Honneur, inséré au rang 5 : territoire pilote de
l'agglomération de Québec, phase croissance admissible, prêt sans intérêt,
sans garantie et sans mise de fonds. Montant non publié par l'organisme, la
fourchette est inférée de son objectif public et signalée comme telle.

Le script de vérification localise désormais les lignes de total par leur
libellé plutôt que par un numéro codé en dur, qui devenait faux dès qu'un
programme était inséré.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UvYqHAWmt8Vm4vpbKQ1Pmv
</commit_message>
<xml_diff>
--- a/financement/Financement_Lasclay_2026.xlsx
+++ b/financement/Financement_Lasclay_2026.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan priorisé'!$A$4:$P$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan priorisé'!$A$4:$P$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -574,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P47"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1001,48 +1001,48 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Allonger les périodes d'emploi</t>
+          <t>Prêt d'honneur IQPH</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Services Québec (MESS)</t>
+          <t>Initiative Québec Prêt d'Honneur</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Québec (Capitale-Nationale)</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
+          <t>Prêt SANS INTÉRÊT ni garantie</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>3000</v>
+        <v>15000</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>13000</v>
+        <v>30000</v>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>50 % du salaire</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Ouvert — dépôt en continu</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>Via un conseiller aux entreprises Services Québec</t>
+          <t>Envoi des documents à candidature@iqph.org</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
@@ -1052,22 +1052,22 @@
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>50 % du salaire brut, maximum 6 500 $ par emploi par année. Le projet doit être récurrent et allonger la saison de travail.</t>
+          <t>Territoire pilote : agglomération de Québec — rempli. Phases admissibles : démarrage, CROISSANCE et repreneuriat. Prêt sans intérêt, sans frais de dossier et sans garantie personnelle. Sélection à deux niveaux : qualités entrepreneuriales et projet, puis productivité, innovation, commercialisation et développement durable. Montant fixé au cas par cas par le comité d'approbation — non publié.</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>Taillé pour la saisonnalité hivernale de Lasclay. Le développement de la gamme été et plein air EST le projet de diversification que le programme finance.</t>
+          <t>Aucune mise de fonds et zéro intérêt : c'est le seul financement de la liste qui attaque directement les 53 074 $ d'intérêts. Organisme en phase pilote (objectif : 48 entreprises sur 6 ans) qui cherche des dossiers vitrines — la notoriété de Lasclay joue pour. DEUX RÉSERVES : le prêt vise à renforcer les fonds propres pour lever du financement institutionnel, or ils sont à -254 035 $, ce qui est autant l'argument que le risque devant le comité ; et l'accompagnement par un mentor est obligatoire pendant toute la durée du contrat. À CLARIFIER AVEC EUX : le prêt est-il consenti à l'entreprise ou à l'entrepreneur personnellement ?</t>
         </is>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/allonger-periodes-emploi</t>
+          <t>https://www.iqph.org/</t>
         </is>
       </c>
     </row>
@@ -1077,12 +1077,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Mesure de formation de la main-d'œuvre</t>
+          <t>Allonger les périodes d'emploi</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Services Québec</t>
+          <t>Services Québec (MESS)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
+          <t>Subvention salariale</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -1101,14 +1101,14 @@
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Variable</t>
+          <t>50 % du salaire</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>Via le même conseiller</t>
+          <t>Via un conseiller aux entreprises Services Québec</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
@@ -1133,17 +1133,17 @@
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>Couvre les frais de formateur et les salaires des employés pendant la formation, y compris pour la transformation numérique.</t>
+          <t>50 % du salaire brut, maximum 6 500 $ par emploi par année. Le projet doit être récurrent et allonger la saison de travail.</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>Équipe réduite à environ 2 personnes après le virage : la montée en compétences des restants tient les opérations.</t>
+          <t>Taillé pour la saisonnalité hivernale de Lasclay. Le développement de la gamme été et plein air EST le projet de diversification que le programme finance.</t>
         </is>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/former-main-oeuvre/developper-competences</t>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/allonger-periodes-emploi</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Concertation pour l'emploi (GRH)</t>
+          <t>Mesure de formation de la main-d'œuvre</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1180,7 +1180,7 @@
         <v>2000</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
@@ -1209,17 +1209,17 @@
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>Honoraires professionnels : diagnostic RH, mandat de consultation, coaching de gestion, accompagnement en gestion du changement.</t>
+          <t>Couvre les frais de formateur et les salaires des employés pendant la formation, y compris pour la transformation numérique.</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>Le virage manufacturier 2025-2026, avec mises à pied et redéfinition des rôles, est une gestion du changement documentée.</t>
+          <t>Équipe réduite à environ 2 personnes après le virage : la montée en compétences des restants tient les opérations.</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/obtenir-conseils</t>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/former-main-oeuvre/developper-competences</t>
         </is>
       </c>
     </row>
@@ -1229,22 +1229,22 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>PARI — Programme emploi jeunesse</t>
+          <t>Concertation pour l'emploi (GRH)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Conseil national de recherches Canada</t>
+          <t>Services Québec</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
+          <t>Subvention</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1253,24 +1253,24 @@
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Part du salaire</t>
+          <t>Variable</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>À déposer avec le dossier PARI principal</t>
+          <t>Via le même conseiller</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
@@ -1285,17 +1285,17 @@
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>Diplômé postsecondaire de 15 à 30 ans, 6 à 12 mois, minimum 30 h/semaine. Volets R-D, génie, multimédia ou étude de marché.</t>
+          <t>Honoraires professionnels : diagnostic RH, mandat de consultation, coaching de gestion, accompagnement en gestion du changement.</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>Le volet étude de marché couvre exactement le travail d'expansion américaine par régions réceptives.</t>
+          <t>Le virage manufacturier 2025-2026, avec mises à pied et redéfinition des rôles, est une gestion du changement documentée.</t>
         </is>
       </c>
       <c r="P12" s="9" t="inlineStr">
         <is>
-          <t>https://nrc.canada.ca/fr/soutien-linnovation-technologique/largent-pari-cnrc-embaucher-jeunes-diplomes</t>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/obtenir-conseils</t>
         </is>
       </c>
     </row>
@@ -1305,12 +1305,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Stages pratiques PSPE (Magnet, CTIC, TECHNATION, BioTalent)</t>
+          <t>PARI — Programme emploi jeunesse</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>ESDC via partenaires sectoriels</t>
+          <t>Conseil national de recherches Canada</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1329,29 +1329,29 @@
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>15000</v>
+        <v>30000</v>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Salaire avancé, remboursé après</t>
+          <t>Part du salaire</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Ouvert par trimestre scolaire</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>Premier arrivé, premier servi</t>
+          <t>À déposer avec le dossier PARI principal</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>FY27 T2</t>
+          <t>FY27 T1</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
@@ -1361,17 +1361,17 @@
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>5 000 $ par stage d'étudiant postsecondaire. Postes à composante numérique ou technologique priorisés.</t>
+          <t>Diplômé postsecondaire de 15 à 30 ans, 6 à 12 mois, minimum 30 h/semaine. Volets R-D, génie, multimédia ou étude de marché.</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>Un poste en commerce électronique, automatisation ou données qualifie sans forcer. Déposer chez UN SEUL partenaire : c'est la même enveloppe fédérale.</t>
+          <t>Le volet étude de marché couvre exactement le travail d'expansion américaine par régions réceptives.</t>
         </is>
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>https://swpprogram.ca/fr/</t>
+          <t>https://nrc.canada.ca/fr/soutien-linnovation-technologique/largent-pari-cnrc-embaucher-jeunes-diplomes</t>
         </is>
       </c>
     </row>
@@ -1381,12 +1381,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Emplois d'été Canada</t>
+          <t>Stages pratiques PSPE (Magnet, CTIC, TECHNATION, BioTalent)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Emploi et Développement social Canada</t>
+          <t>ESDC via partenaires sectoriels</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1405,24 +1405,24 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>50 % du salaire minimum</t>
+          <t>Salaire avancé, remboursé après</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Fermé — rouvre vers novembre 2026</t>
+          <t>Ouvert par trimestre scolaire</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>Date limite attendue ~11 décembre 2026 pour l'été 2027</t>
+          <t>Premier arrivé, premier servi</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
@@ -1437,17 +1437,17 @@
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>Secteur privé : jusqu'à 50 % du salaire minimum en vigueur. Jeunes de 15 à 30 ans, postes à temps plein.</t>
+          <t>5 000 $ par stage d'étudiant postsecondaire. Postes à composante numérique ou technologique priorisés.</t>
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>Renfort d'atelier ou d'expédition pour la production estivale, en amont de la saison hivernale.</t>
+          <t>Un poste en commerce électronique, automatisation ou données qualifie sans forcer. Déposer chez UN SEUL partenaire : c'est la même enveloppe fédérale.</t>
         </is>
       </c>
       <c r="P14" s="9" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/emploi-developpement-social/services/financement/emplois-ete-canada.html</t>
+          <t>https://swpprogram.ca/fr/</t>
         </is>
       </c>
     </row>
@@ -1457,12 +1457,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Riipen — Level UP</t>
+          <t>Emplois d'été Canada</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Riipen</t>
+          <t>Emploi et Développement social Canada</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
+          <t>Subvention salariale</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1481,24 +1481,24 @@
         </is>
       </c>
       <c r="G15" s="7" t="n">
-        <v>1400</v>
+        <v>3000</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>4200</v>
+        <v>8000</v>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Aucune</t>
+          <t>50 % du salaire minimum</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Fermé — rouvre vers novembre 2026</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>Par semestre universitaire</t>
+          <t>Date limite attendue ~11 décembre 2026 pour l'été 2027</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
@@ -1513,17 +1513,17 @@
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>1 400 $ par étudiant. Projets de 60 heures sur 2 à 8 semaines, encadrés par un enseignant.</t>
+          <t>Secteur privé : jusqu'à 50 % du salaire minimum en vigueur. Jeunes de 15 à 30 ans, postes à temps plein.</t>
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
         <is>
-          <t>Format parfait pour des mandats bornés : localisation des fiches produits pour les marchés américains, refonte du guide de plantation, analyse de saisonnalité.</t>
+          <t>Renfort d'atelier ou d'expédition pour la production estivale, en amont de la saison hivernale.</t>
         </is>
       </c>
       <c r="P15" s="9" t="inlineStr">
         <is>
-          <t>https://fr.riipen.com/levelup/employers</t>
+          <t>https://www.canada.ca/fr/emploi-developpement-social/services/financement/emplois-ete-canada.html</t>
         </is>
       </c>
     </row>
@@ -1533,17 +1533,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Mitacs Accélération</t>
+          <t>Riipen — Level UP</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Mitacs + MEIE</t>
+          <t>Riipen</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Fédéral et Québec</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1557,49 +1557,49 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>7500</v>
+        <v>1400</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>30000</v>
+        <v>4200</v>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Environ 50 %</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>Via un conseiller Mitacs en développement des affaires</t>
+          <t>Par semestre universitaire</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>FY27 T3</t>
+          <t>FY27 T2</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>Stagiaires universitaires, postdoctoraux et chercheurs intégrés à un projet d'innovation en entreprise. Financement partagé MEIE, entreprise, fédéral.</t>
+          <t>1 400 $ par étudiant. Projets de 60 heures sur 2 à 8 semaines, encadrés par un enseignant.</t>
         </is>
       </c>
       <c r="O16" s="8" t="inlineStr">
         <is>
-          <t>Le meilleur véhicule pour faire caractériser la fibre en laboratoire : conductivité thermique du produit fini, tenue à la compression, comportement à l'humidité.</t>
+          <t>Format parfait pour des mandats bornés : localisation des fiches produits pour les marchés américains, refonte du guide de plantation, analyse de saisonnalité.</t>
         </is>
       </c>
       <c r="P16" s="9" t="inlineStr">
         <is>
-          <t>https://www.mitacs.ca/fr-ca/</t>
+          <t>https://fr.riipen.com/levelup/employers</t>
         </is>
       </c>
     </row>
@@ -1609,22 +1609,22 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>grand V — accompagnement technologique</t>
+          <t>Mitacs Accélération</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>Mitacs + MEIE</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Fédéral et Québec</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Service (sans dette)</t>
+          <t>Subvention</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1633,14 +1633,14 @@
         </is>
       </c>
       <c r="G17" s="7" t="n">
-        <v>0</v>
+        <v>7500</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Aucune</t>
+          <t>Environ 50 %</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>En continu</t>
+          <t>Via un conseiller Mitacs en développement des affaires</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
@@ -1660,22 +1660,22 @@
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>Jusqu'à 100 heures d'experts en innovation. Séparable du volet financement, qui lui est hors de portée.</t>
+          <t>Stagiaires universitaires, postdoctoraux et chercheurs intégrés à un projet d'innovation en entreprise. Financement partagé MEIE, entreprise, fédéral.</t>
         </is>
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>Couvre le prototypage d'équipements sur mesure et la valorisation des résidus. Demander SANS le prêt de 250 000 $.</t>
+          <t>Le meilleur véhicule pour faire caractériser la fibre en laboratoire : conductivité thermique du produit fini, tenue à la compression, comportement à l'humidité.</t>
         </is>
       </c>
       <c r="P17" s="9" t="inlineStr">
         <is>
-          <t>https://grandv.investquebec.com/</t>
+          <t>https://www.mitacs.ca/fr-ca/</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Fonds Écoleader — Biodiversité</t>
+          <t>grand V — accompagnement technologique</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>FAQDD / MELCCFP</t>
+          <t>Investissement Québec</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -1700,33 +1700,33 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Contribution non remboursable</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+          <t>Service (sans dette)</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Environ 25 %</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Modalités non publiées</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>Annoncé pour le printemps 2026, en retard — relancer chaque mois au 418 692-5888</t>
+          <t>En continu</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
@@ -1736,22 +1736,22 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>Enveloppe de 5,7 M$, 2026-2028, Plan nature 2030. Entreprises de toutes tailles. Paie des experts pour intégrer la biodiversité.</t>
+          <t>Jusqu'à 100 heures d'experts en innovation. Séparable du volet financement, qui lui est hors de portée.</t>
         </is>
       </c>
       <c r="O18" s="8" t="inlineStr">
         <is>
-          <t>Fit exceptionnel : la thèse d'affaires entière de Lasclay est de rendre l'asclépiade viable pour restaurer l'habitat du monarque.</t>
+          <t>Couvre le prototypage d'équipements sur mesure et la valorisation des résidus. Demander SANS le prêt de 250 000 $.</t>
         </is>
       </c>
       <c r="P18" s="9" t="inlineStr">
         <is>
-          <t>https://faqdd.qc.ca/programmes/fonds-ecoleader-biodiversite/</t>
+          <t>https://grandv.investquebec.com/</t>
         </is>
       </c>
     </row>
@@ -1761,53 +1761,53 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>CanExport PME</t>
+          <t>Fonds Écoleader — Biodiversité</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Affaires mondiales Canada</t>
+          <t>FAQDD / MELCCFP</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
+          <t>Contribution non remboursable</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
         <v>10000</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>50 %</t>
+          <t>Environ 25 %</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Ouvert jusqu'au 31 août 2026, 12 h</t>
+          <t>Modalités non publiées</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>Rouvre vers le 4 février 2027 pour l'exercice 2027-28</t>
+          <t>Annoncé pour le printemps 2026, en retard — relancer chaque mois au 418 692-5888</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>FY27 T2</t>
+          <t>FY27 T3</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
@@ -1817,17 +1817,17 @@
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>Enveloppe É.-U. de 3,1 M$ ENTIÈREMENT ALLOUÉE. Cible les marchés où l'entreprise a peu ou pas d'activités. 50 % des coûts, projet de 20 k$ à 100 k$.</t>
+          <t>Enveloppe de 5,7 M$, 2026-2028, Plan nature 2030. Entreprises de toutes tailles. Paie des experts pour intégrer la biodiversité.</t>
         </is>
       </c>
       <c r="O19" s="8" t="inlineStr">
         <is>
-          <t>Viser la France, la Belgique et les pays nordiques, où le récit du monarque se transpose. Pas les États-Unis. Bâtir le dossier d'ici février plutôt que d'improviser en 26 jours.</t>
+          <t>Fit exceptionnel : la thèse d'affaires entière de Lasclay est de rendre l'asclépiade viable pour restaurer l'habitat du monarque.</t>
         </is>
       </c>
       <c r="P19" s="9" t="inlineStr">
         <is>
-          <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/soutien-financier-expansion-commerciale-international/canexport-pme/nouveau-2026-2027.html</t>
+          <t>https://faqdd.qc.ca/programmes/fonds-ecoleader-biodiversite/</t>
         </is>
       </c>
     </row>
@@ -1837,12 +1837,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>CERI — Expansion des entreprises et productivité</t>
+          <t>CanExport PME</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Développement économique Canada</t>
+          <t>Affaires mondiales Canada</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -1852,19 +1852,19 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Contribution remboursable à 0 %</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>25000</v>
+        <v>10000</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>250000</v>
+        <v>50000</v>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
@@ -1873,37 +1873,37 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Ouvert jusqu'au 31 août 2026, 12 h</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>En continu</t>
+          <t>Rouvre vers le 4 février 2027 pour l'exercice 2027-28</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>FY27 T4</t>
+          <t>FY27 T2</t>
         </is>
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>Aucun seuil de revenus, contrairement à l'IRRT. Secteurs admissibles : manufacturier, transformation alimentaire, TIC, sciences de la vie. Commerce de détail EXPLICITEMENT EXCLU.</t>
+          <t>Enveloppe É.-U. de 3,1 M$ ENTIÈREMENT ALLOUÉE. Cible les marchés où l'entreprise a peu ou pas d'activités. 50 % des coûts, projet de 20 k$ à 100 k$.</t>
         </is>
       </c>
       <c r="O20" s="8" t="inlineStr">
         <is>
-          <t>Le dossier doit se présenter comme manufacturier — atelier de Limoilou, transformation de l'isolant, code d'activité — et non comme du commerce en ligne. 0 % d'intérêt, remboursements 2 ans après la fin.</t>
+          <t>Viser la France, la Belgique et les pays nordiques, où le récit du monarque se transpose. Pas les États-Unis. Bâtir le dossier d'ici février plutôt que d'improviser en 26 jours.</t>
         </is>
       </c>
       <c r="P20" s="9" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/developpement-economique-regions-quebec/financement-services/expansion-des-entreprises-et-productivite.html</t>
+          <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/soutien-financier-expansion-commerciale-international/canexport-pme/nouveau-2026-2027.html</t>
         </is>
       </c>
     </row>
@@ -1913,22 +1913,22 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Capitale-Innovation</t>
+          <t>CERI — Expansion des entreprises et productivité</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Ville de Québec</t>
+          <t>Développement économique Canada</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Contribution non remboursable</t>
+          <t>Contribution remboursable à 0 %</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
@@ -1937,29 +1937,29 @@
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>50000</v>
+        <v>25000</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>500000</v>
+        <v>250000</v>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>50 %, puis 60 % au-delà de 250 k$</t>
+          <t>50 %</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Volet ouvert (page à jour le 8 juillet 2026)</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>Enveloppe Vision Québec 2030 possiblement fermée depuis le 31 mars 2026 — à faire trancher</t>
+          <t>En continu</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>FY28 T3</t>
+          <t>FY27 T4</t>
         </is>
       </c>
       <c r="M21" s="5" t="inlineStr">
@@ -1969,17 +1969,17 @@
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
-          <t>Secteur « Manufacturier, matériaux, transformation industrielle » explicitement admissible. Siège dans l'agglomération de Québec : rempli (1286 av. de la Ronde).</t>
+          <t>Aucun seuil de revenus, contrairement à l'IRRT. Secteurs admissibles : manufacturier, transformation alimentaire, TIC, sciences de la vie. Commerce de détail EXPLICITEMENT EXCLU.</t>
         </is>
       </c>
       <c r="O21" s="8" t="inlineStr">
         <is>
-          <t>Le plus gros non remboursable accessible localement. Exige la preuve de détention de la PI. Cumul de toute aide publique plafonné à 70 %.</t>
+          <t>Le dossier doit se présenter comme manufacturier — atelier de Limoilou, transformation de l'isolant, code d'activité — et non comme du commerce en ligne. 0 % d'intérêt, remboursements 2 ans après la fin.</t>
         </is>
       </c>
       <c r="P21" s="9" t="inlineStr">
         <is>
-          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/innovation/capitale-innovation.aspx</t>
+          <t>https://www.canada.ca/fr/developpement-economique-regions-quebec/financement-services/expansion-des-entreprises-et-productivite.html</t>
         </is>
       </c>
     </row>
@@ -1989,27 +1989,27 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Programme Innovation — Volet 1</t>
+          <t>Capitale-Innovation</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>MEIE</t>
+          <t>Ville de Québec</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Municipal</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
-        </is>
-      </c>
-      <c r="F22" s="11" t="inlineStr">
-        <is>
-          <t>Reporté</t>
+          <t>Contribution non remboursable</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -2020,22 +2020,22 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>25 % en argent</t>
+          <t>50 %, puis 60 % au-delà de 250 k$</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>N'accepte pas les demandes</t>
+          <t>Volet ouvert (page à jour le 8 juillet 2026)</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>Surveiller la réouverture</t>
+          <t>Enveloppe Vision Québec 2030 possiblement fermée depuis le 31 mars 2026 — à faire trancher</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>FY28 T3</t>
         </is>
       </c>
       <c r="M22" s="5" t="inlineStr">
@@ -2045,17 +2045,17 @@
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
-          <t>Jusqu'à 500 000 $ par entreprise. Contribution privée EN ARGENT d'au moins 25 % des dépenses admissibles.</t>
+          <t>Secteur « Manufacturier, matériaux, transformation industrielle » explicitement admissible. Siège dans l'agglomération de Québec : rempli (1286 av. de la Ronde).</t>
         </is>
       </c>
       <c r="O22" s="8" t="inlineStr">
         <is>
-          <t>ABSENT du répertoire Innoveici : c'est un angle mort du premier tri. Pendant provincial de Capitale-Innovation, à surveiller activement.</t>
+          <t>Le plus gros non remboursable accessible localement. Exige la preuve de détention de la PI. Cumul de toute aide publique plafonné à 70 %.</t>
         </is>
       </c>
       <c r="P22" s="9" t="inlineStr">
         <is>
-          <t>https://www.economie.gouv.qc.ca/bibliotheques/programmes/aide-financiere/programme-innovation</t>
+          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/innovation/capitale-innovation.aspx</t>
         </is>
       </c>
     </row>
@@ -2065,12 +2065,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>ESSOR — Volet 1 (études préalables)</t>
+          <t>Programme Innovation — Volet 1</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>MEIE</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -2083,55 +2083,55 @@
           <t>Subvention</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>5000</v>
+        <v>50000</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>50000</v>
+        <v>500000</v>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Variable</t>
+          <t>25 % en argent</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>N'accepte pas les demandes</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>Dépôt en continu</t>
+          <t>Surveiller la réouverture</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>FY28 T3</t>
+          <t>FY28</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Élevé</t>
         </is>
       </c>
       <c r="N23" s="8" t="inlineStr">
         <is>
-          <t>Études de faisabilité, diagnostic numérique, plan numérique. Entreprises de tous secteurs.</t>
+          <t>Jusqu'à 500 000 $ par entreprise. Contribution privée EN ARGENT d'au moins 25 % des dépenses admissibles.</t>
         </is>
       </c>
       <c r="O23" s="8" t="inlineStr">
         <is>
-          <t>Porte d'entrée à faible risque avant tout projet d'équipement financé par ESSOR volet 2.</t>
+          <t>ABSENT du répertoire Innoveici : c'est un angle mort du premier tri. Pendant provincial de Capitale-Innovation, à surveiller activement.</t>
         </is>
       </c>
       <c r="P23" s="9" t="inlineStr">
         <is>
-          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-la-concretisation-de-projets-dinvestissement</t>
+          <t>https://www.economie.gouv.qc.ca/bibliotheques/programmes/aide-financiere/programme-innovation</t>
         </is>
       </c>
     </row>
@@ -2141,34 +2141,34 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Bons d'accompagnement à la croissance</t>
+          <t>ESSOR — Volet 1 (études préalables)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Ville de Québec</t>
+          <t>Investissement Québec</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Contribution</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
         <v>5000</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
@@ -2177,37 +2177,37 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Ouvert, dépôt en continu</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>Aucune date de tombée</t>
+          <t>Dépôt en continu</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>FY27 T4</t>
+          <t>FY28 T3</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
-          <t>Exclut explicitement les commerces opérant UNIQUEMENT en ligne.</t>
+          <t>Études de faisabilité, diagnostic numérique, plan numérique. Entreprises de tous secteurs.</t>
         </is>
       </c>
       <c r="O24" s="8" t="inlineStr">
         <is>
-          <t>L'atelier de Limoilou et la transformation de l'isolant sortent Lasclay de l'exclusion, mais il faut l'énoncer clairement dans la demande.</t>
+          <t>Porte d'entrée à faible risque avant tout projet d'équipement financé par ESSOR volet 2.</t>
         </is>
       </c>
       <c r="P24" s="9" t="inlineStr">
         <is>
-          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/productivite/bons-accompagnement.aspx</t>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-la-concretisation-de-projets-dinvestissement</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Prêts aux entreprises</t>
+          <t>Bons d'accompagnement à la croissance</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Prêt</t>
+          <t>Contribution</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
@@ -2241,49 +2241,49 @@
         </is>
       </c>
       <c r="G25" s="7" t="n">
-        <v>25000</v>
+        <v>5000</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>150000</v>
+        <v>20000</v>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Capacité de crédit</t>
+          <t>Variable</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Ouvert, dépôt en continu</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>En continu</t>
+          <t>Aucune date de tombée</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>FY28 T1</t>
+          <t>FY27 T4</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="N25" s="8" t="inlineStr">
         <is>
-          <t>Quatre volets : démarrage, amélioration et transformation, croissance et expansion, relève.</t>
+          <t>Exclut explicitement les commerces opérant UNIQUEMENT en ligne.</t>
         </is>
       </c>
       <c r="O25" s="8" t="inlineStr">
         <is>
-          <t>Le volet « amélioration et transformation » colle au virage manufacturier. La capacité de crédit reste à démontrer avec un avoir négatif.</t>
+          <t>L'atelier de Limoilou et la transformation de l'isolant sortent Lasclay de l'exclusion, mais il faut l'énoncer clairement dans la demande.</t>
         </is>
       </c>
       <c r="P25" s="9" t="inlineStr">
         <is>
-          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/autres/prets-aux-entreprises/index.aspx</t>
+          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/productivite/bons-accompagnement.aspx</t>
         </is>
       </c>
     </row>
@@ -2293,53 +2293,53 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Primo-adoptants</t>
+          <t>Prêts aux entreprises</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>MEIE</t>
+          <t>Ville de Québec</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Municipal</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Subvention (versée au partenaire)</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
+          <t>Prêt</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="H26" s="7" t="n">
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>20 % en espèces</t>
+          <t>Capacité de crédit</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Appel de projets</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>Surveiller les appels</t>
+          <t>En continu</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>FY28 T3</t>
+          <t>FY28 T1</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
@@ -2349,17 +2349,17 @@
       </c>
       <c r="N26" s="8" t="inlineStr">
         <is>
-          <t>Lasclay serait le primo-adoptant, pas le bénéficiaire. La contribution du gouvernement va à la startup ; le primo-adoptant met 20 % en espèces.</t>
+          <t>Quatre volets : démarrage, amélioration et transformation, croissance et expansion, relève.</t>
         </is>
       </c>
       <c r="O26" s="8" t="inlineStr">
         <is>
-          <t>Manière peu coûteuse de faire tester sur la fibre des équipements d'automatisation ou de vision par ordinateur pour le contrôle qualité.</t>
+          <t>Le volet « amélioration et transformation » colle au virage manufacturier. La capacité de crédit reste à démontrer avec un avoir négatif.</t>
         </is>
       </c>
       <c r="P26" s="9" t="inlineStr">
         <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/liste-partielle-aide-financiere/appels-projets-innovation/appel-primo-adoptants</t>
+          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/autres/prets-aux-entreprises/index.aspx</t>
         </is>
       </c>
     </row>
@@ -2369,53 +2369,53 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Accès aux talents</t>
+          <t>Primo-adoptants</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Produits naturels Canada</t>
+          <t>MEIE</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+          <t>Subvention (versée au partenaire)</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>75000</v>
+        <v>0</v>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>60 % du salaire</t>
+          <t>20 % en espèces</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Appel de projets</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>Demande à tout moment</t>
+          <t>Surveiller les appels</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>FY28 T1</t>
+          <t>FY28 T3</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
@@ -2425,17 +2425,17 @@
       </c>
       <c r="N27" s="8" t="inlineStr">
         <is>
-          <t>40 % du salaire d'un nouvel employé, maximum 75 000 $. Exige d'être membre de la grappe de l'innovation en produits naturels.</t>
+          <t>Lasclay serait le primo-adoptant, pas le bénéficiaire. La contribution du gouvernement va à la startup ; le primo-adoptant met 20 % en espèces.</t>
         </is>
       </c>
       <c r="O27" s="8" t="inlineStr">
         <is>
-          <t>La définition de PNC — bioproduits et durabilité — couvre l'asclépiade. La collaboration cosmétique autour de l'huile de graine est le candidat naturel.</t>
+          <t>Manière peu coûteuse de faire tester sur la fibre des équipements d'automatisation ou de vision par ordinateur pour le contrôle qualité.</t>
         </is>
       </c>
       <c r="P27" s="9" t="inlineStr">
         <is>
-          <t>https://www.naturalproductscanada.com/fr/programmes/programme-daccess-aux-talents/</t>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/liste-partielle-aide-financiere/appels-projets-innovation/appel-primo-adoptants</t>
         </is>
       </c>
     </row>
@@ -2445,38 +2445,38 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Contrat d'intégration au travail</t>
+          <t>Accès aux talents</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Services Québec</t>
+          <t>Produits naturels Canada</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="G28" s="7" t="n">
-        <v>3000</v>
+        <v>20000</v>
       </c>
       <c r="H28" s="7" t="n">
-        <v>20000</v>
+        <v>75000</v>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Part du salaire</t>
+          <t>60 % du salaire</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -2486,32 +2486,32 @@
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>En continu</t>
+          <t>Demande à tout moment</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>FY28 T1</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="N28" s="8" t="inlineStr">
         <is>
-          <t>Soutien au salaire pour compenser un écart de productivité, plus couverture de l'adaptation du poste.</t>
+          <t>40 % du salaire d'un nouvel employé, maximum 75 000 $. Exige d'être membre de la grappe de l'innovation en produits naturels.</t>
         </is>
       </c>
       <c r="O28" s="8" t="inlineStr">
         <is>
-          <t>Pertinent pour l'assemblage, l'emballage de semences et l'expédition, où les tâches se découpent bien.</t>
+          <t>La définition de PNC — bioproduits et durabilité — couvre l'asclépiade. La collaboration cosmétique autour de l'huile de graine est le candidat naturel.</t>
         </is>
       </c>
       <c r="P28" s="9" t="inlineStr">
         <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/recruter/contrat-integration-travail</t>
+          <t>https://www.naturalproductscanada.com/fr/programmes/programme-daccess-aux-talents/</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Pratiques RH (FCCQ) et RH éclair! (FCEI)</t>
+          <t>Contrat d'intégration au travail</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>FCCQ / FCEI</t>
+          <t>Services Québec</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Québec et fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Service gratuit</t>
+          <t>Subvention salariale</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -2545,19 +2545,19 @@
         </is>
       </c>
       <c r="G29" s="7" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Aucune</t>
+          <t>Part du salaire</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>FY27 T1</t>
+          <t>FY28</t>
         </is>
       </c>
       <c r="M29" s="5" t="inlineStr">
@@ -2577,17 +2577,17 @@
       </c>
       <c r="N29" s="8" t="inlineStr">
         <is>
-          <t>Accès gratuit à des conseils RH et juridiques, à une bibliothèque de modèles et de politiques.</t>
+          <t>Soutien au salaire pour compenser un écart de productivité, plus couverture de l'adaptation du poste.</t>
         </is>
       </c>
       <c r="O29" s="8" t="inlineStr">
         <is>
-          <t>Zéro dollar en jeu, mais utile pour sécuriser les contrats et les politiques après une réduction d'effectifs.</t>
+          <t>Pertinent pour l'assemblage, l'emballage de semences et l'expédition, où les tâches se découpent bien.</t>
         </is>
       </c>
       <c r="P29" s="9" t="inlineStr">
         <is>
-          <t>https://pratiquesrh.com/</t>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/recruter/contrat-integration-travail</t>
         </is>
       </c>
     </row>
@@ -2597,22 +2597,22 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>ICI on recycle +</t>
+          <t>Pratiques RH (FCCQ) et RH éclair! (FCEI)</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Recyc-Québec</t>
+          <t>FCCQ / FCEI</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Québec et fédéral</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Attestation (clé d'accès)</t>
+          <t>Service gratuit</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -2621,14 +2621,14 @@
         </is>
       </c>
       <c r="G30" s="7" t="n">
-        <v>-350</v>
+        <v>0</v>
       </c>
       <c r="H30" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>350 $ de frais d'inscription</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>FY27 T1</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
@@ -2653,17 +2653,17 @@
       </c>
       <c r="N30" s="8" t="inlineStr">
         <is>
-          <t>N'octroie pas d'aide. Écocondition OBLIGATOIRE, au niveau « Mise en œuvre », pour le versement final de plusieurs aides de Recyc-Québec.</t>
+          <t>Accès gratuit à des conseils RH et juridiques, à une bibliothèque de modèles et de politiques.</t>
         </is>
       </c>
       <c r="O30" s="8" t="inlineStr">
         <is>
-          <t>C'est une clé, pas une source. Environ 350 $ pour déverrouiller les enveloppes de Recyc-Québec et crédibiliser les appels d'offres corporatifs.</t>
+          <t>Zéro dollar en jeu, mais utile pour sécuriser les contrats et les politiques après une réduction d'effectifs.</t>
         </is>
       </c>
       <c r="P30" s="9" t="inlineStr">
         <is>
-          <t>https://www.recyc-quebec.gouv.qc.ca/entreprises-organismes/performer/programme-ici-on-recycle-plus/</t>
+          <t>https://pratiquesrh.com/</t>
         </is>
       </c>
     </row>
@@ -2673,73 +2673,73 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Validation de principe</t>
+          <t>ICI on recycle +</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Produits naturels Canada</t>
+          <t>Recyc-Québec</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Financement remboursable</t>
-        </is>
-      </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+          <t>Attestation (clé d'accès)</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="G31" s="7" t="n">
-        <v>50000</v>
+        <v>-350</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>250000</v>
+        <v>0</v>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>60 %</t>
+          <t>350 $ de frais d'inscription</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>Demande à tout moment</t>
+          <t>En continu</t>
         </is>
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>FY28 T4</t>
+          <t>FY28</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="N31" s="8" t="inlineStr">
         <is>
-          <t>40 % des coûts, maximum 250 000 $. PNC cherche un potentiel de 10 à 15 M$ de revenus annuels — un cran au-dessus de la trajectoire de Lasclay.</t>
+          <t>N'octroie pas d'aide. Écocondition OBLIGATOIRE, au niveau « Mise en œuvre », pour le versement final de plusieurs aides de Recyc-Québec.</t>
         </is>
       </c>
       <c r="O31" s="8" t="inlineStr">
         <is>
-          <t>Réserve sérieuse sur le critère de potentiel de revenus. À tenter seulement si le volet cosmétique prend de l'ampleur.</t>
+          <t>C'est une clé, pas une source. Environ 350 $ pour déverrouiller les enveloppes de Recyc-Québec et crédibiliser les appels d'offres corporatifs.</t>
         </is>
       </c>
       <c r="P31" s="9" t="inlineStr">
         <is>
-          <t>https://www.naturalproductscanada.com/fr/programmes/programme-validation-de-principe/</t>
+          <t>https://www.recyc-quebec.gouv.qc.ca/entreprises-organismes/performer/programme-ici-on-recycle-plus/</t>
         </is>
       </c>
     </row>
@@ -2749,53 +2749,53 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Panorama</t>
+          <t>Validation de principe</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>Produits naturels Canada</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Prêt</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>Reporté</t>
+          <t>Financement remboursable</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="G32" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H32" s="7" t="n">
         <v>250000</v>
       </c>
-      <c r="H32" s="7" t="n">
-        <v>1000000</v>
-      </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Capacité de crédit</t>
+          <t>60 %</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>Après retour à la rentabilité</t>
+          <t>Demande à tout moment</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>FY28 T4</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
@@ -2805,17 +2805,17 @@
       </c>
       <c r="N32" s="8" t="inlineStr">
         <is>
-          <t>Prêt de fonds de roulement export, moratoire de capital de 24 mois, SANS sûreté ni caution corporative ou personnelle. EXCLUT les États-Unis.</t>
+          <t>40 % des coûts, maximum 250 000 $. PNC cherche un potentiel de 10 à 15 M$ de revenus annuels — un cran au-dessus de la trajectoire de Lasclay.</t>
         </is>
       </c>
       <c r="O32" s="8" t="inlineStr">
         <is>
-          <t>Structure rare et attrayante, mais hors de portée avec un avoir de -254 035 $ et 584 320 $ de dette portant intérêt.</t>
+          <t>Réserve sérieuse sur le critère de potentiel de revenus. À tenter seulement si le volet cosmétique prend de l'ampleur.</t>
         </is>
       </c>
       <c r="P32" s="9" t="inlineStr">
         <is>
-          <t>https://exportation.investquebec.com/solutions</t>
+          <t>https://www.naturalproductscanada.com/fr/programmes/programme-validation-de-principe/</t>
         </is>
       </c>
     </row>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>ESSOR — Volet 2 (productivité et expansion)</t>
+          <t>Panorama</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Contribution remboursable ou garantie</t>
+          <t>Prêt</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
@@ -2849,10 +2849,10 @@
         </is>
       </c>
       <c r="G33" s="7" t="n">
-        <v>50000</v>
+        <v>250000</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>500000</v>
+        <v>1000000</v>
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
@@ -2861,17 +2861,17 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>Après un exercice FY2027 positif</t>
+          <t>Après retour à la rentabilité</t>
         </is>
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>FY28 T1</t>
+          <t>FY28</t>
         </is>
       </c>
       <c r="M33" s="5" t="inlineStr">
@@ -2881,17 +2881,17 @@
       </c>
       <c r="N33" s="8" t="inlineStr">
         <is>
-          <t>Exige de démontrer un potentiel de hausse de rentabilité ou de masse salariale. Honoraires de gestion d'au moins 0,5 % du montant accordé.</t>
+          <t>Prêt de fonds de roulement export, moratoire de capital de 24 mois, SANS sûreté ni caution corporative ou personnelle. EXCLUT les États-Unis.</t>
         </is>
       </c>
       <c r="O33" s="8" t="inlineStr">
         <is>
-          <t>Le raisonnement reste juste, il est prématuré d'un ou deux exercices. Rouvrir le dossier sur des états financiers montrant un redressement.</t>
+          <t>Structure rare et attrayante, mais hors de portée avec un avoir de -254 035 $ et 584 320 $ de dette portant intérêt.</t>
         </is>
       </c>
       <c r="P33" s="9" t="inlineStr">
         <is>
-          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/essor-volet-2</t>
+          <t>https://exportation.investquebec.com/solutions</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>grand V — financement</t>
+          <t>ESSOR — Volet 2 (productivité et expansion)</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Prêt à terme</t>
+          <t>Contribution remboursable ou garantie</t>
         </is>
       </c>
       <c r="F34" s="11" t="inlineStr">
@@ -2925,10 +2925,10 @@
         </is>
       </c>
       <c r="G34" s="7" t="n">
-        <v>250000</v>
+        <v>50000</v>
       </c>
       <c r="H34" s="7" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
@@ -2957,17 +2957,17 @@
       </c>
       <c r="N34" s="8" t="inlineStr">
         <is>
-          <t>Prêt MINIMUM de 250 000 $, moratoire de capital jusqu'à 48 mois. Devant -254 035 $ de capitaux propres et 584 320 $ de dette, l'analyse de crédit bloque.</t>
+          <t>Exige de démontrer un potentiel de hausse de rentabilité ou de masse salariale. Honoraires de gestion d'au moins 0,5 % du montant accordé.</t>
         </is>
       </c>
       <c r="O34" s="8" t="inlineStr">
         <is>
-          <t>C'était le levier identifié pour remplacer Merchant Growth et Shopify Capital. Il reste le bon levier, mais pas avant un redressement.</t>
+          <t>Le raisonnement reste juste, il est prématuré d'un ou deux exercices. Rouvrir le dossier sur des états financiers montrant un redressement.</t>
         </is>
       </c>
       <c r="P34" s="9" t="inlineStr">
         <is>
-          <t>https://grandv.investquebec.com/</t>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/essor-volet-2</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>ESSOR — Volet 4 (internationalisation)</t>
+          <t>grand V — financement</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Prêt ou garantie</t>
+          <t>Prêt à terme</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
@@ -3001,10 +3001,10 @@
         </is>
       </c>
       <c r="G35" s="7" t="n">
-        <v>50000</v>
+        <v>250000</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>500000</v>
+        <v>1000000</v>
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
@@ -3013,17 +3013,17 @@
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>Si le développement É.-U. passe par de la distribution locale</t>
+          <t>Après un exercice FY2027 positif</t>
         </is>
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>FY28 T4</t>
+          <t>FY28 T1</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
@@ -3033,17 +3033,17 @@
       </c>
       <c r="N35" s="8" t="inlineStr">
         <is>
-          <t>Vise les stratégies d'internationalisation complexes : entités, entrepôts, chaînes d'approvisionnement à l'étranger.</t>
+          <t>Prêt MINIMUM de 250 000 $, moratoire de capital jusqu'à 48 mois. Devant -254 035 $ de capitaux propres et 584 320 $ de dette, l'analyse de crédit bloque.</t>
         </is>
       </c>
       <c r="O35" s="8" t="inlineStr">
         <is>
-          <t>Ne se justifie pas tant que les États-Unis sont servis par expédition directe depuis Québec.</t>
+          <t>C'était le levier identifié pour remplacer Merchant Growth et Shopify Capital. Il reste le bon levier, mais pas avant un redressement.</t>
         </is>
       </c>
       <c r="P35" s="9" t="inlineStr">
         <is>
-          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-linternationalisation-des-entreprises</t>
+          <t>https://grandv.investquebec.com/</t>
         </is>
       </c>
     </row>
@@ -3053,12 +3053,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Fonds économie circulaire</t>
+          <t>ESSOR — Volet 4 (internationalisation)</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Fondaction</t>
+          <t>Investissement Québec</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -3068,23 +3068,23 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Capital (dilution)</t>
-        </is>
-      </c>
-      <c r="F36" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+          <t>Prêt ou garantie</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
         </is>
       </c>
       <c r="G36" s="7" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="H36" s="7" t="n">
         <v>500000</v>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>Dilution du capital</t>
+          <t>Capacité de crédit</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
@@ -3094,12 +3094,12 @@
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>En continu</t>
+          <t>Si le développement É.-U. passe par de la distribution locale</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>FY28 T4</t>
         </is>
       </c>
       <c r="M36" s="5" t="inlineStr">
@@ -3109,17 +3109,17 @@
       </c>
       <c r="N36" s="8" t="inlineStr">
         <is>
-          <t>Cible les jeunes entreprises en phase de démarrage dont le modèle repose sur la circularité. C'est du capital, pas de la subvention.</t>
+          <t>Vise les stratégies d'internationalisation complexes : entités, entrepôts, chaînes d'approvisionnement à l'étranger.</t>
         </is>
       </c>
       <c r="O36" s="8" t="inlineStr">
         <is>
-          <t>Les semences issues de la transformation de la soie et la gamme « Les Imparfaits » sont de la circularité réelle. À ne considérer que si l'ouverture du capital devient une option assumée.</t>
+          <t>Ne se justifie pas tant que les États-Unis sont servis par expédition directe depuis Québec.</t>
         </is>
       </c>
       <c r="P36" s="9" t="inlineStr">
         <is>
-          <t>https://www.fondaction.com/entreprise/fonds-economie-circulaire/</t>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-linternationalisation-des-entreprises</t>
         </is>
       </c>
     </row>
@@ -3129,163 +3129,239 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
+          <t>Fonds économie circulaire</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Fondaction</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Québec</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Capital (dilution)</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Dilution du capital</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>En continu</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>Élevé</t>
+        </is>
+      </c>
+      <c r="N37" s="8" t="inlineStr">
+        <is>
+          <t>Cible les jeunes entreprises en phase de démarrage dont le modèle repose sur la circularité. C'est du capital, pas de la subvention.</t>
+        </is>
+      </c>
+      <c r="O37" s="8" t="inlineStr">
+        <is>
+          <t>Les semences issues de la transformation de la soie et la gamme « Les Imparfaits » sont de la circularité réelle. À ne considérer que si l'ouverture du capital devient une option assumée.</t>
+        </is>
+      </c>
+      <c r="P37" s="9" t="inlineStr">
+        <is>
+          <t>https://www.fondaction.com/entreprise/fonds-economie-circulaire/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="58" customHeight="1">
+      <c r="A38" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
           <t>Programme canadien de l'innovation à l'international</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>Affaires mondiales Canada</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>Fédéral</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>Subvention</t>
         </is>
       </c>
-      <c r="F37" s="10" t="inlineStr">
+      <c r="F38" s="10" t="inlineStr">
         <is>
           <t>À valider</t>
         </is>
       </c>
-      <c r="G37" s="7" t="n">
+      <c r="G38" s="7" t="n">
         <v>15000</v>
       </c>
-      <c r="H37" s="7" t="n">
+      <c r="H38" s="7" t="n">
         <v>600000</v>
       </c>
-      <c r="I37" s="5" t="inlineStr">
+      <c r="I38" s="5" t="inlineStr">
         <is>
           <t>50 %</t>
         </is>
       </c>
-      <c r="J37" s="5" t="inlineStr">
+      <c r="J38" s="5" t="inlineStr">
         <is>
           <t>Dépôt ad hoc</t>
         </is>
       </c>
-      <c r="K37" s="5" t="inlineStr">
+      <c r="K38" s="5" t="inlineStr">
         <is>
           <t>Ad hoc</t>
         </is>
       </c>
-      <c r="L37" s="5" t="inlineStr">
+      <c r="L38" s="5" t="inlineStr">
         <is>
           <t>FY28</t>
         </is>
       </c>
-      <c r="M37" s="5" t="inlineStr">
+      <c r="M38" s="5" t="inlineStr">
         <is>
           <t>Élevé</t>
         </is>
       </c>
-      <c r="N37" s="8" t="inlineStr">
+      <c r="N38" s="8" t="inlineStr">
         <is>
           <t>Exige un partenaire de R-D au Brésil, en Chine, en Inde, en Israël ou en Corée du Sud.</t>
         </is>
       </c>
-      <c r="O37" s="8" t="inlineStr">
+      <c r="O38" s="8" t="inlineStr">
         <is>
           <t>La liste de pays ne recoupe pas la chaîne d'approvisionnement actuelle, qui passe par la Tunisie. À garder en veille seulement.</t>
         </is>
       </c>
-      <c r="P37" s="9" t="inlineStr">
+      <c r="P38" s="9" t="inlineStr">
         <is>
           <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/programmes-soutien/programme-canadien-innovation-international.html</t>
         </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>Potentiel total, verdict « Admissible » seulement</t>
-        </is>
-      </c>
-      <c r="G39" s="13">
-        <f>SUMIF($F$5:$F$37,"Admissible",G5:G37)</f>
-        <v>121550</v>
-      </c>
-      <c r="H39" s="13">
-        <f>SUMIF($F$5:$F$37,"Admissible",H5:H37)</f>
-        <v>465200</v>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="12" t="inlineStr">
         <is>
-          <t>Potentiel total, « Admissible » + « À valider »</t>
+          <t>Potentiel total, verdict « Admissible » seulement</t>
         </is>
       </c>
       <c r="G40" s="13">
-        <f>SUMIF($F$5:$F$37,"Admissible",G5:G37)+SUMIF($F$5:$F$37,"À valider",G5:G37)</f>
-        <v>421550</v>
+        <f>SUMIF($F$5:$F$38,"Admissible",G5:G38)</f>
+        <v>121550</v>
       </c>
       <c r="H40" s="13">
-        <f>SUMIF($F$5:$F$37,"Admissible",H5:H37)+SUMIF($F$5:$F$37,"À valider",H5:H37)</f>
-        <v>2875200</v>
+        <f>SUMIF($F$5:$F$38,"Admissible",H5:H38)</f>
+        <v>465200</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="12" t="inlineStr">
         <is>
+          <t>Potentiel total, « Admissible » + « À valider »</t>
+        </is>
+      </c>
+      <c r="G41" s="13">
+        <f>SUMIF($F$5:$F$38,"Admissible",G5:G38)+SUMIF($F$5:$F$38,"À valider",G5:G38)</f>
+        <v>436550</v>
+      </c>
+      <c r="H41" s="13">
+        <f>SUMIF($F$5:$F$38,"Admissible",H5:H38)+SUMIF($F$5:$F$38,"À valider",H5:H38)</f>
+        <v>2905200</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="12" t="inlineStr">
+        <is>
           <t>Dont admissible SANS aucune mise de fonds</t>
         </is>
       </c>
-      <c r="G41" s="13">
-        <f>SUMIFS(G5:G37,$F$5:$F$37,"Admissible",$I$5:$I$37,"Aucune")</f>
+      <c r="G42" s="13">
+        <f>SUMIFS(G5:G38,$F$5:$F$38,"Admissible",$I$5:$I$38,"Aucune")</f>
         <v>46400</v>
       </c>
-      <c r="H41" s="13">
-        <f>SUMIFS(H5:H37,$F$5:$F$37,"Admissible",$I$5:$I$37,"Aucune")</f>
+      <c r="H42" s="13">
+        <f>SUMIFS(H5:H38,$F$5:$F$38,"Admissible",$I$5:$I$38,"Aucune")</f>
         <v>74200</v>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="14" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>Notes de lecture</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="26" customHeight="1">
-      <c r="B44" s="15" t="inlineStr">
-        <is>
-          <t>• Montants min et max : fourchettes réalistes pour un dossier Lasclay, pas les plafonds théoriques des programmes. Ils servent à prioriser, pas à budgéter.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="26" customHeight="1">
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>• Verdicts : « Admissible » = tous les critères publiés sont rencontrés. « À valider » = un critère dépend d'un arbitrage, d'un cadrage ou d'une confirmation de l'organisme. « Reporté » = admissible sur papier, hors de portée financièrement aujourd'hui.</t>
+          <t>• Montants min et max : fourchettes réalistes pour un dossier Lasclay, pas les plafonds théoriques des programmes. Ils servent à prioriser, pas à budgéter. Cas particulier du rang 5 (IQPH) : l'organisme ne publie aucun montant. La fourchette de 15 à 30 k$ est INFÉRÉE de son objectif public — 48 entreprises et 12 M$ d'investissements générés sur 6 ans, avec un effet de levier annoncé jusqu'à 10 fois — et doit être confirmée auprès d'eux.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="26" customHeight="1">
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>• La contrainte dominante n'est pas l'admissibilité, c'est la mise de fonds : trésorerie de -2 060 $ et marge EDC utilisée à 94,8 %. D'où la priorité donnée aux crédits d'impôt et aux subventions salariales, qui remboursent des dépenses déjà engagées.</t>
+          <t>• Verdicts : « Admissible » = tous les critères publiés sont rencontrés. « À valider » = un critère dépend d'un arbitrage, d'un cadrage ou d'une confirmation de l'organisme. « Reporté » = admissible sur papier, hors de portée financièrement aujourd'hui.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="26" customHeight="1">
       <c r="B47" s="15" t="inlineStr">
         <is>
+          <t>• La contrainte dominante n'est pas l'admissibilité, c'est la mise de fonds : trésorerie de -2 060 $ et marge EDC utilisée à 94,8 %. D'où la priorité donnée aux crédits d'impôt et aux subventions salariales, qui remboursent des dépenses déjà engagées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
+      <c r="B48" s="15" t="inlineStr">
+        <is>
           <t>• Sources vérifiées le 5 août 2026 aux sites officiels des organismes. Les statuts de programme changent sans préavis : revalider avant tout dépôt.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:P37"/>
+  <autoFilter ref="A4:P38"/>
   <mergeCells count="6">
     <mergeCell ref="A1:P1"/>
-    <mergeCell ref="B44:H44"/>
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="B47:H47"/>
+    <mergeCell ref="B48:H48"/>
     <mergeCell ref="B45:H45"/>
     <mergeCell ref="B46:H46"/>
   </mergeCells>
@@ -3979,7 +4055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4165,20 +4241,24 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Demander un conseiller CTI et poser d'emblée la question de l'arbitrage avec la RS&amp;DE</t>
+          <t>Déposer la candidature : business model canvas, sommaire exécutif, extrait du registre des entreprises et CV, à candidature@iqph.org</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>PARI-CNRC</t>
+          <t>Prêt d'honneur IQPH</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Premier contact</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr"/>
+          <t>Dépôt en continu</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Sans intérêt et sans garantie — aucune autre source de la liste n'offre ça</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -4193,12 +4273,12 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Un seul appel à Services Québec pour couvrir les trois mesures (emploi, formation, GRH)</t>
+          <t>Demander un conseiller CTI et poser d'emblée la question de l'arbitrage avec la RS&amp;DE</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Services Québec</t>
+          <t>PARI-CNRC</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -4221,173 +4301,173 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Faire trancher par la Ville : l'enveloppe Capitale-Innovation est-elle disponible ou en attente du renouvellement de l'entente ?</t>
+          <t>Un seul appel à Services Québec pour couvrir les trois mesures (emploi, formation, GRH)</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Capitale-Innovation</t>
+          <t>Services Québec</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Vérification</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Un dossier de 500 k$ monté pour rien</t>
-        </is>
-      </c>
+          <t>Premier contact</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>~11 décembre 2026</t>
+          <t>Sept — nov 2026</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>FY2027 T2</t>
+          <t>FY2027 T1</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Déposer la demande pour l'été 2027</t>
+          <t>Faire trancher par la Ville : l'enveloppe Capitale-Innovation est-elle disponible ou en attente du renouvellement de l'entente ?</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Emplois d'été Canada</t>
+          <t>Capitale-Innovation</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Fermeture d'appel</t>
+          <t>Vérification</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Report d'un an complet</t>
+          <t>Un dossier de 500 k$ monté pour rien</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
+          <t>~11 décembre 2026</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>FY2027 T2</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Déposer la demande pour l'été 2027</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Emplois d'été Canada</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Fermeture d'appel</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Report d'un an complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
           <t>~4 février 2027</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>FY2027 T2</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Déposer dès les premiers jours : premier arrivé, premier servi</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>CanExport PME 2027-28</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Ouverture d'appel</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Épuisement de l'enveloppe en cours d'exercice</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>28 FÉVRIER 2027</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>FY2027 T2</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>DATE LIMITE ABSOLUE de production de la réclamation RS&amp;DE pour FY2025</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>RS&amp;DE FY2025</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>LIMITE FERME</t>
         </is>
       </c>
-      <c r="F14" s="17" t="inlineStr">
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>Perte définitive. L'ARC n'a aucun pouvoir discrétionnaire.</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Déc 2026 — fév 2027</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>FY2027 T2</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Déposer les subventions salariales de stage pour l'hiver et l'été</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>PSPE et Riipen</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Par trimestre</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr"/>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Mars — août 2027</t>
+          <t>Déc 2026 — fév 2027</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>FY2027 T3-T4</t>
+          <t>FY2027 T2</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Monter le dossier DEC Expansion en le cadrant comme manufacturier, pas comme commerce en ligne</t>
+          <t>Déposer les subventions salariales de stage pour l'hiver et l'été</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>CERI Expansion</t>
+          <t>PSPE et Riipen</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Dépôt en continu</t>
+          <t>Par trimestre</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr"/>
@@ -4400,17 +4480,17 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>FY2027 T3</t>
+          <t>FY2027 T3-T4</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Demander l'accompagnement technologique seul, sans le volet financement</t>
+          <t>Monter le dossier DEC Expansion en le cadrant comme manufacturier, pas comme commerce en ligne</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>grand V</t>
+          <t>CERI Expansion</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -4423,94 +4503,90 @@
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Mensuel, à partir de sept 2026</t>
+          <t>Mars — août 2027</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>FY2027 — continu</t>
+          <t>FY2027 T3</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Relancer le FAQDD au 418 692-5888 jusqu'à publication des modalités</t>
+          <t>Demander l'accompagnement technologique seul, sans le volet financement</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Écoleader Biodiversité</t>
+          <t>grand V</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Veille active</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Enveloppe de 5,7 M$ épuisée avant d'avoir déposé</t>
-        </is>
-      </c>
+          <t>Dépôt en continu</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr"/>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Mars — août 2027</t>
+          <t>Mensuel, à partir de sept 2026</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>FY2027 T3</t>
+          <t>FY2027 — continu</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Monter un stage de caractérisation de la fibre en laboratoire</t>
+          <t>Relancer le FAQDD au 418 692-5888 jusqu'à publication des modalités</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Mitacs</t>
+          <t>Écoleader Biodiversité</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Dépôt en continu</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr"/>
+          <t>Veille active</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Enveloppe de 5,7 M$ épuisée avant d'avoir déposé</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Sept — nov 2027</t>
+          <t>Mars — août 2027</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>FY2028 T1</t>
+          <t>FY2027 T3</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Produire la réclamation RS&amp;DE et CRIC de FY2027 dès la clôture</t>
+          <t>Monter un stage de caractérisation de la fibre en laboratoire</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>RS&amp;DE / CRIC</t>
+          <t>Mitacs</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Dépôt</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Le réflexe doit devenir annuel</t>
-        </is>
-      </c>
+          <t>Dépôt en continu</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr"/>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
@@ -4525,110 +4601,110 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Rouvrir le dossier IQ si FY2027 revient au positif : grand V, ESSOR volet 2</t>
+          <t>Produire la réclamation RS&amp;DE et CRIC de FY2027 dès la clôture</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>RS&amp;DE / CRIC</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Réévaluation</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr"/>
+          <t>Dépôt</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Le réflexe doit devenir annuel</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
+          <t>Sept — nov 2027</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>FY2028 T1</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Rouvrir le dossier IQ si FY2027 revient au positif : grand V, ESSOR volet 2</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Investissement Québec</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Réévaluation</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
           <t>~Février 2028</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>FY2028 T2</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Déposer sur un deuxième marché européen si le premier a produit des résultats</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>CanExport PME 2028-29</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>Ouverture d'appel</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr"/>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>28 FÉVRIER 2028</t>
         </is>
       </c>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>FY2028 T2</t>
         </is>
       </c>
-      <c r="C23" s="17" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>DATE LIMITE ABSOLUE de production de la réclamation RS&amp;DE pour FY2026</t>
         </is>
       </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>RS&amp;DE FY2026</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr">
+      <c r="E24" s="17" t="inlineStr">
         <is>
           <t>LIMITE FERME</t>
         </is>
       </c>
-      <c r="F23" s="17" t="inlineStr">
+      <c r="F24" s="17" t="inlineStr">
         <is>
           <t>Perte définitive de 45 k$ à 70 k$.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>Mars — août 2028</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>FY2028 T3</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Déposer Capitale-Innovation si l'entente est renouvelée et la trésorerie reconstituée</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Capitale-Innovation</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>Dépôt</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>C'est le dossier de fin de plan, pas de début</t>
         </is>
       </c>
     </row>
@@ -4645,45 +4721,49 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Financer les études de faisabilité en amont d'un projet d'équipement</t>
+          <t>Déposer Capitale-Innovation si l'entente est renouvelée et la trésorerie reconstituée</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>ESSOR volet 1</t>
+          <t>Capitale-Innovation</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Dépôt en continu</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="inlineStr"/>
+          <t>Dépôt</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>C'est le dossier de fin de plan, pas de début</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="32" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Août 2028</t>
+          <t>Mars — août 2028</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>FY2028 — clôture</t>
+          <t>FY2028 T3</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Revalider le seuil de 2 M$ : une catégorie entière de programmes fédéraux s'ouvre au-delà</t>
+          <t>Financer les études de faisabilité en amont d'un projet d'équipement</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Divers fédéral</t>
+          <t>ESSOR volet 1</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>Jalon</t>
+          <t>Dépôt en continu</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr"/>
@@ -4691,30 +4771,58 @@
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
+          <t>Août 2028</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>FY2028 — clôture</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Revalider le seuil de 2 M$ : une catégorie entière de programmes fédéraux s'ouvre au-delà</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Divers fédéral</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Jalon</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr"/>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
           <t>Janvier 2027, puis janvier 2028</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Annuel</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Rebalayer le répertoire Innoveici : 88 des 208 programmes étaient fermés au 5 août 2026</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>Veille</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
         <is>
           <t>Récurrent</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr"/>
+      <c r="F28" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5133,7 +5241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -5357,20 +5465,64 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>Initiative Québec Prêt d'Honneur (IQPH)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Territoire pilote Capitale-Nationale, phases admissibles, prêt sans intérêt ni garantie, sélection à deux niveaux, documents et adresse de dépôt.</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>https://www.iqph.org/l'organisme</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>CCIQ — annonce du partenariat IQPH</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Phase pilote dans la Capitale-Nationale, objectif de 48 entreprises et 12 M$ d'investissements générés sur 6 ans. Base de l'estimation du montant de prêt.</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>https://cciquebec.ca/la-chambre-de-commerce-et-dindustrie-de-quebec-appuie-une-initiative-novatrice-pour-propulser-ses-entrepreneurs-quebec-pret-dhonneur-iqph/</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
           <t>QuickBooks Online — Les Produits Lasclay Inc</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Tous les chiffres opposés aux critères : revenus, résultat, trésorerie, capitaux propres, dette, assiette R-D.</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>(accès interne via le Finance Proxy)</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>

</xml_diff>

<commit_message>
Reclasser le financement selon les quatre piliers, sans le manufacturier
Lasclay n'est plus manufacturier pour le moment. Le classement suit désormais
mission, ventes, international et R&D, avec une colonne Pilier.

Reculent : C3i, grand V accompagnement, Primo-adoptants, ESSOR et DEC Expansion,
qui reposaient sur l'achat d'équipement, la productivité d'usine ou le statut de
secteur manufacturier. Le conseil de cadrer le dossier DEC en manufacturier est
retiré.

Montent : CanExport et l'Écoleader Biodiversité entrent dans les six premiers,
Mitacs et Produits Naturels Canada dans les dix premiers.

Ajout du PSCE volet 2 d'Investissement Québec : 60 000 $ non remboursables pour
la diversification hors Québec, dont le seuil d'admissibilité de 1 M$ de chiffre
d'affaires vient d'être franchi avec FY2026. Fermé actuellement, mis en veille
trimestrielle.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UvYqHAWmt8Vm4vpbKQ1Pmv
</commit_message>
<xml_diff>
--- a/financement/Financement_Lasclay_2026.xlsx
+++ b/financement/Financement_Lasclay_2026.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan priorisé'!$A$4:$P$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan priorisé'!$A$4:$Q$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -574,25 +574,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="58" customWidth="1" min="14" max="14"/>
-    <col width="64" customWidth="1" min="15" max="15"/>
-    <col width="46" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="58" customWidth="1" min="15" max="15"/>
+    <col width="64" customWidth="1" min="16" max="16"/>
+    <col width="46" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -632,60 +633,65 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>Pilier</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>Type d'aide</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Montant min ($)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Montant max ($)</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Mise de fonds requise</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Statut au 5 août 2026</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Prochaine fenêtre / date clé</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Trimestre cible</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Effort</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Motif du verdict (validé)</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Angle Lasclay</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Lien</t>
         </is>
@@ -712,56 +718,61 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
           <t>Crédit d'impôt remboursable</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="H5" s="7" t="n">
         <v>30000</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="I5" s="7" t="n">
         <v>45000</v>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Aucune</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>Ouvert en continu</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>Limites FERMES : 28 fév 2027 (FY25), 28 fév 2028 (FY26)</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>FY27 T1</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="N5" s="8" t="inlineStr">
+      <c r="O5" s="8" t="inlineStr">
         <is>
           <t>103 364 $ de salaires portés au compte 6061 RSDE en FY2026, plus 7 112 $ de matériaux. SPCC : 35 % remboursable en argent.</t>
         </is>
       </c>
-      <c r="O5" s="8" t="inlineStr">
+      <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Argent comptant sur des salaires déjà payés, sans mise de fonds. Première action : confirmer avec le comptable si la réclamation FY2025 a été produite.</t>
         </is>
       </c>
-      <c r="P5" s="9" t="inlineStr">
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>https://www.canada.ca/fr/agence-revenu/services/impot/entreprises/sujets/recherche-scientifique-developpement-experimental-programme-encouragements-fiscaux.html</t>
         </is>
@@ -788,56 +799,61 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t>Crédit d'impôt remboursable</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="H6" s="7" t="n">
         <v>15000</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="I6" s="7" t="n">
         <v>25000</v>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Aucune</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>En vigueur (exercices ouverts après le 25 mars 2025)</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>Avec la déclaration fiscale annuelle</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>FY27 T1</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="N6" s="8" t="inlineStr">
+      <c r="O6" s="8" t="inlineStr">
         <is>
           <t>Remplace 8 anciens crédits québécois. 30 % sur le premier 1 M$ de dépenses admissibles. S'applique déjà à FY2026.</t>
         </is>
       </c>
-      <c r="O6" s="8" t="inlineStr">
+      <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Se réclame en tandem avec la RS&amp;DE fédérale. L'aide provinciale réduit l'assiette fédérale : faire modéliser le combiné, ne pas additionner naïvement.</t>
         </is>
       </c>
-      <c r="P6" s="9" t="inlineStr">
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>https://www.revenuquebec.ca/fr/entreprises/impots/impot-des-societes/credits-dimpot-des-societes/</t>
         </is>
@@ -849,73 +865,78 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>C3i — investissement et innovation</t>
+          <t>PARI-CNRC</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Revenu Québec</t>
+          <t>Conseil national de recherches Canada</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Crédit d'impôt remboursable</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>0</v>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Contribution non remboursable</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
+        </is>
       </c>
       <c r="H7" s="7" t="n">
-        <v>25000</v>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>L'achat d'équipement lui-même</t>
-        </is>
+        <v>20000</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>150000</v>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>En vigueur</t>
+          <t>20 % des salaires</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>Avec la déclaration fiscale annuelle</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>FY27-FY28</t>
+          <t>Demander un conseiller CTI dès maintenant</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
-        </is>
-      </c>
-      <c r="N7" s="8" t="inlineStr">
-        <is>
-          <t>15 % à 25 % du coût du matériel de fabrication et transformation (catégorie 53) et des logiciels de gestion, utilisé au Québec 730 jours consécutifs.</t>
+          <t>FY27 T1</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>187 487 $ d'immobilisations aux livres, dont 135 851 $ d'équipements. Ne se cumule PAS avec le CRIC sur la même dépense : arbitrer avec le comptable.</t>
-        </is>
-      </c>
-      <c r="P7" s="9" t="inlineStr">
-        <is>
-          <t>https://www.revenuquebec.ca/fr/entreprises/impots/impot-des-societes/credits-dimpot-des-societes/</t>
+          <t>PME canadienne de moins de 500 employés développant un produit ou procédé novateur. 80 % des salaires, 50 % des sous-traitants.</t>
+        </is>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>Matelassage d'une fibre volatile, inserts amovibles, gants isolés : projets défendables. ATTENTION : une contribution PARI réduit l'assiette RS&amp;DE sur les mêmes dollars.</t>
+        </is>
+      </c>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>https://nrc.canada.ca/fr/soutien-linnovation-technologique/propos-programme-daide-recherche-industrielle-cnrc</t>
         </is>
       </c>
     </row>
@@ -925,12 +946,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>PARI-CNRC</t>
+          <t>CanExport PME</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Conseil national de recherches Canada</t>
+          <t>Affaires mondiales Canada</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -940,58 +961,63 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Contribution non remboursable</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G8" s="7" t="n">
-        <v>20000</v>
-      </c>
       <c r="H8" s="7" t="n">
-        <v>150000</v>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>20 % des salaires</t>
-        </is>
+        <v>10000</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>50000</v>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>50 %</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>Demander un conseiller CTI dès maintenant</t>
+          <t>Ouvert jusqu'au 31 août 2026, 12 h</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>FY27 T1</t>
+          <t>Rouvre vers le 4 février 2027 pour l'exercice 2027-28</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
+          <t>FY27 T2</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="N8" s="8" t="inlineStr">
-        <is>
-          <t>PME canadienne de moins de 500 employés développant un produit ou procédé novateur. 80 % des salaires, 50 % des sous-traitants.</t>
-        </is>
-      </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>Matelassage d'une fibre volatile, inserts amovibles, gants isolés : projets défendables. ATTENTION : une contribution PARI réduit l'assiette RS&amp;DE sur les mêmes dollars.</t>
-        </is>
-      </c>
-      <c r="P8" s="9" t="inlineStr">
-        <is>
-          <t>https://nrc.canada.ca/fr/soutien-linnovation-technologique/propos-programme-daide-recherche-industrielle-cnrc</t>
+          <t>Enveloppe É.-U. de 3,1 M$ ENTIÈREMENT ALLOUÉE. Cible les marchés où l'entreprise a peu ou pas d'activités. 50 % des coûts, projet de 20 k$ à 100 k$.</t>
+        </is>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>Viser la France, la Belgique et les pays nordiques, où le récit du monarque se transpose. Pas les États-Unis. Bâtir le dossier d'ici février plutôt que d'improviser en 26 jours.</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/soutien-financier-expansion-commerciale-international/canexport-pme/nouveau-2026-2027.html</t>
         </is>
       </c>
     </row>
@@ -1016,56 +1042,61 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
+          <t>Mission et ventes</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
           <t>Prêt SANS INTÉRÊT ni garantie</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="G9" s="10" t="inlineStr">
         <is>
           <t>À valider</t>
         </is>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="H9" s="7" t="n">
         <v>15000</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="I9" s="7" t="n">
         <v>30000</v>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Aucune</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Ouvert — dépôt en continu</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="L9" s="5" t="inlineStr">
         <is>
           <t>Envoi des documents à candidature@iqph.org</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>FY27 T1</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="N9" s="8" t="inlineStr">
+      <c r="O9" s="8" t="inlineStr">
         <is>
           <t>Territoire pilote : agglomération de Québec — rempli. Phases admissibles : démarrage, CROISSANCE et repreneuriat. Prêt sans intérêt, sans frais de dossier et sans garantie personnelle. Sélection à deux niveaux : qualités entrepreneuriales et projet, puis productivité, innovation, commercialisation et développement durable. Montant fixé au cas par cas par le comité d'approbation — non publié.</t>
         </is>
       </c>
-      <c r="O9" s="8" t="inlineStr">
+      <c r="P9" s="8" t="inlineStr">
         <is>
           <t>Aucune mise de fonds et zéro intérêt : c'est le seul financement de la liste qui attaque directement les 53 074 $ d'intérêts. Organisme en phase pilote (objectif : 48 entreprises sur 6 ans) qui cherche des dossiers vitrines — la notoriété de Lasclay joue pour. DEUX RÉSERVES : le prêt vise à renforcer les fonds propres pour lever du financement institutionnel, or ils sont à -254 035 $, ce qui est autant l'argument que le risque devant le comité ; et l'accompagnement par un mentor est obligatoire pendant toute la durée du contrat. À CLARIFIER AVEC EUX : le prêt est-il consenti à l'entreprise ou à l'entrepreneur personnellement ?</t>
         </is>
       </c>
-      <c r="P9" s="9" t="inlineStr">
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>https://www.iqph.org/</t>
         </is>
@@ -1077,12 +1108,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Allonger les périodes d'emploi</t>
+          <t>Fonds Écoleader — Biodiversité</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Services Québec (MESS)</t>
+          <t>FAQDD / MELCCFP</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1092,58 +1123,63 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>3000</v>
+          <t>Mission</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Contribution non remboursable</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>13000</v>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>50 % du salaire</t>
-        </is>
+        <v>10000</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>40000</v>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Environ 25 %</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>Via un conseiller aux entreprises Services Québec</t>
+          <t>Modalités non publiées</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>FY27 T1</t>
+          <t>Annoncé pour le printemps 2026, en retard — relancer chaque mois au 418 692-5888</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
-        </is>
-      </c>
-      <c r="N10" s="8" t="inlineStr">
-        <is>
-          <t>50 % du salaire brut, maximum 6 500 $ par emploi par année. Le projet doit être récurrent et allonger la saison de travail.</t>
+          <t>FY27 T3</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>Taillé pour la saisonnalité hivernale de Lasclay. Le développement de la gamme été et plein air EST le projet de diversification que le programme finance.</t>
-        </is>
-      </c>
-      <c r="P10" s="9" t="inlineStr">
-        <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/allonger-periodes-emploi</t>
+          <t>Enveloppe de 5,7 M$, 2026-2028, Plan nature 2030. Entreprises de toutes tailles. Paie des experts pour intégrer la biodiversité.</t>
+        </is>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>Fit exceptionnel : la thèse d'affaires entière de Lasclay est de rendre l'asclépiade viable pour restaurer l'habitat du monarque.</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>https://faqdd.qc.ca/programmes/fonds-ecoleader-biodiversite/</t>
         </is>
       </c>
     </row>
@@ -1153,12 +1189,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Mesure de formation de la main-d'œuvre</t>
+          <t>PSCE — Volet 2 : diversification et consolidation hors Québec</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Services Québec</t>
+          <t>Investissement Québec</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1168,58 +1204,63 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="n">
-        <v>2000</v>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Contribution non remboursable</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
+        </is>
       </c>
       <c r="H11" s="7" t="n">
-        <v>15000</v>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
+        <v>20000</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>60000</v>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>25 % du coût total</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>Via le même conseiller</t>
+          <t>N'accepte pas les demandes</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>FY27 T1</t>
+          <t>Surveiller la réouverture — vérifier aussi s'il a été remplacé</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
-        </is>
-      </c>
-      <c r="N11" s="8" t="inlineStr">
-        <is>
-          <t>Couvre les frais de formateur et les salaires des employés pendant la formation, y compris pour la transformation numérique.</t>
+          <t>FY27-FY28</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>Équipe réduite à environ 2 personnes après le virage : la montée en compétences des restants tient les opérations.</t>
-        </is>
-      </c>
-      <c r="P11" s="9" t="inlineStr">
-        <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/former-main-oeuvre/developper-competences</t>
+          <t>SEUIL TOUT JUSTE FRANCHI : le programme exige un chiffre d'affaires supérieur à 1 M$ et inférieur ou égal à 50 M$. FY2025 était à 879 125 $, sous le seuil ; FY2026 clôture à 1 081 908 $, au-dessus. Exige aussi que plus de 40 % de la viabilité repose sur des revenus autonomes — largement rempli.</t>
+        </is>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>60 000 $ par entreprise par année, non remboursable, pour la diversification de marchés hors Québec. Aucune exigence de secteur manufacturier. C'est le meilleur complément à CanExport : le fédéral et le provincial financent le même effort d'export sans se cumuler sur la même dépense. À surveiller activement — le seuil de 1 M$ vient d'être franchi, ce qui rend Lasclay admissible pour la première fois.</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/programme-de-soutien-la-commercialisation-et-lexportation/psce-volet-2</t>
         </is>
       </c>
     </row>
@@ -1229,73 +1270,78 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Concertation pour l'emploi (GRH)</t>
+          <t>PARI — Programme emploi jeunesse</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Services Québec</t>
+          <t>Conseil national de recherches Canada</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Subvention salariale</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G12" s="7" t="n">
-        <v>2000</v>
-      </c>
       <c r="H12" s="7" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
+        <v>15000</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>30000</v>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Part du salaire</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>Via le même conseiller</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
+          <t>À déposer avec le dossier PARI principal</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
           <t>FY27 T1</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>Faible</t>
         </is>
       </c>
-      <c r="N12" s="8" t="inlineStr">
-        <is>
-          <t>Honoraires professionnels : diagnostic RH, mandat de consultation, coaching de gestion, accompagnement en gestion du changement.</t>
-        </is>
-      </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>Le virage manufacturier 2025-2026, avec mises à pied et redéfinition des rôles, est une gestion du changement documentée.</t>
-        </is>
-      </c>
-      <c r="P12" s="9" t="inlineStr">
-        <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/obtenir-conseils</t>
+          <t>Diplômé postsecondaire de 15 à 30 ans, 6 à 12 mois, minimum 30 h/semaine. Volets R-D, génie, multimédia ou étude de marché.</t>
+        </is>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>Le volet étude de marché couvre exactement le travail d'expansion américaine par régions réceptives.</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
+          <t>https://nrc.canada.ca/fr/soutien-linnovation-technologique/largent-pari-cnrc-embaucher-jeunes-diplomes</t>
         </is>
       </c>
     </row>
@@ -1305,73 +1351,78 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>PARI — Programme emploi jeunesse</t>
+          <t>Mitacs Accélération</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Conseil national de recherches Canada</t>
+          <t>Mitacs + MEIE</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Fédéral et Québec</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G13" s="7" t="n">
-        <v>15000</v>
-      </c>
       <c r="H13" s="7" t="n">
+        <v>7500</v>
+      </c>
+      <c r="I13" s="7" t="n">
         <v>30000</v>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>Part du salaire</t>
-        </is>
-      </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Environ 50 %</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>À déposer avec le dossier PARI principal</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>FY27 T1</t>
+          <t>Via un conseiller Mitacs en développement des affaires</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
-        </is>
-      </c>
-      <c r="N13" s="8" t="inlineStr">
-        <is>
-          <t>Diplômé postsecondaire de 15 à 30 ans, 6 à 12 mois, minimum 30 h/semaine. Volets R-D, génie, multimédia ou étude de marché.</t>
+          <t>FY27 T3</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>Le volet étude de marché couvre exactement le travail d'expansion américaine par régions réceptives.</t>
-        </is>
-      </c>
-      <c r="P13" s="9" t="inlineStr">
-        <is>
-          <t>https://nrc.canada.ca/fr/soutien-linnovation-technologique/largent-pari-cnrc-embaucher-jeunes-diplomes</t>
+          <t>Stagiaires universitaires, postdoctoraux et chercheurs intégrés à un projet d'innovation en entreprise. Financement partagé MEIE, entreprise, fédéral.</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="inlineStr">
+        <is>
+          <t>Le meilleur véhicule pour faire caractériser la fibre en laboratoire : conductivité thermique du produit fini, tenue à la compression, comportement à l'humidité.</t>
+        </is>
+      </c>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t>https://www.mitacs.ca/fr-ca/</t>
         </is>
       </c>
     </row>
@@ -1381,12 +1432,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Stages pratiques PSPE (Magnet, CTIC, TECHNATION, BioTalent)</t>
+          <t>Accès aux talents</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ESDC via partenaires sectoriels</t>
+          <t>Produits naturels Canada</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1396,58 +1447,63 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>5000</v>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
       </c>
       <c r="H14" s="7" t="n">
-        <v>15000</v>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>Salaire avancé, remboursé après</t>
-        </is>
+        <v>20000</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>75000</v>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Ouvert par trimestre scolaire</t>
+          <t>60 % du salaire</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>Premier arrivé, premier servi</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>FY27 T2</t>
+          <t>Demande à tout moment</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
-        </is>
-      </c>
-      <c r="N14" s="8" t="inlineStr">
-        <is>
-          <t>5 000 $ par stage d'étudiant postsecondaire. Postes à composante numérique ou technologique priorisés.</t>
+          <t>FY28 T1</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>Un poste en commerce électronique, automatisation ou données qualifie sans forcer. Déposer chez UN SEUL partenaire : c'est la même enveloppe fédérale.</t>
-        </is>
-      </c>
-      <c r="P14" s="9" t="inlineStr">
-        <is>
-          <t>https://swpprogram.ca/fr/</t>
+          <t>40 % du salaire d'un nouvel employé, maximum 75 000 $. Exige d'être membre de la grappe de l'innovation en produits naturels.</t>
+        </is>
+      </c>
+      <c r="P14" s="8" t="inlineStr">
+        <is>
+          <t>La définition de PNC — bioproduits et durabilité — couvre l'asclépiade. La collaboration cosmétique autour de l'huile de graine est le candidat naturel.</t>
+        </is>
+      </c>
+      <c r="Q14" s="9" t="inlineStr">
+        <is>
+          <t>https://www.naturalproductscanada.com/fr/programmes/programme-daccess-aux-talents/</t>
         </is>
       </c>
     </row>
@@ -1457,73 +1513,78 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Emplois d'été Canada</t>
+          <t>Allonger les périodes d'emploi</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Emploi et Développement social Canada</t>
+          <t>Services Québec (MESS)</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
           <t>Subvention salariale</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>3000</v>
       </c>
-      <c r="H15" s="7" t="n">
-        <v>8000</v>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>50 % du salaire minimum</t>
-        </is>
+      <c r="I15" s="7" t="n">
+        <v>13000</v>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Fermé — rouvre vers novembre 2026</t>
+          <t>50 % du salaire</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>Date limite attendue ~11 décembre 2026 pour l'été 2027</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>FY27 T2</t>
+          <t>Via un conseiller aux entreprises Services Québec</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
+          <t>FY27 T1</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
           <t>Faible</t>
         </is>
       </c>
-      <c r="N15" s="8" t="inlineStr">
-        <is>
-          <t>Secteur privé : jusqu'à 50 % du salaire minimum en vigueur. Jeunes de 15 à 30 ans, postes à temps plein.</t>
-        </is>
-      </c>
       <c r="O15" s="8" t="inlineStr">
         <is>
-          <t>Renfort d'atelier ou d'expédition pour la production estivale, en amont de la saison hivernale.</t>
-        </is>
-      </c>
-      <c r="P15" s="9" t="inlineStr">
-        <is>
-          <t>https://www.canada.ca/fr/emploi-developpement-social/services/financement/emplois-ete-canada.html</t>
+          <t>50 % du salaire brut, maximum 6 500 $ par emploi par année. Le projet doit être récurrent et allonger la saison de travail.</t>
+        </is>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>Toujours valable, mais l'argument se déplace : la saisonnalité qui reste à lisser est celle de l'expédition et du service client, pas celle de la production. Le développement de la gamme été demeure le projet de diversification que le programme finance.</t>
+        </is>
+      </c>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/allonger-periodes-emploi</t>
         </is>
       </c>
     </row>
@@ -1533,73 +1594,78 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Riipen — Level UP</t>
+          <t>Mesure de formation de la main-d'œuvre</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Riipen</t>
+          <t>Services Québec</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
           <t>Subvention</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G16" s="7" t="n">
-        <v>1400</v>
-      </c>
       <c r="H16" s="7" t="n">
-        <v>4200</v>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>Aucune</t>
-        </is>
+        <v>2000</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>15000</v>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Variable</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>Par semestre universitaire</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>FY27 T2</t>
+          <t>Via le même conseiller</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
+          <t>FY27 T1</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
           <t>Faible</t>
         </is>
       </c>
-      <c r="N16" s="8" t="inlineStr">
-        <is>
-          <t>1 400 $ par étudiant. Projets de 60 heures sur 2 à 8 semaines, encadrés par un enseignant.</t>
-        </is>
-      </c>
       <c r="O16" s="8" t="inlineStr">
         <is>
-          <t>Format parfait pour des mandats bornés : localisation des fiches produits pour les marchés américains, refonte du guide de plantation, analyse de saisonnalité.</t>
-        </is>
-      </c>
-      <c r="P16" s="9" t="inlineStr">
-        <is>
-          <t>https://fr.riipen.com/levelup/employers</t>
+          <t>Couvre les frais de formateur et les salaires des employés pendant la formation, y compris pour la transformation numérique.</t>
+        </is>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>Équipe réduite à environ 2 personnes après le virage : la montée en compétences des restants tient les opérations.</t>
+        </is>
+      </c>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/former-main-oeuvre/developper-competences</t>
         </is>
       </c>
     </row>
@@ -1609,73 +1675,78 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Mitacs Accélération</t>
+          <t>Concertation pour l'emploi (GRH)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Mitacs + MEIE</t>
+          <t>Services Québec</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Fédéral et Québec</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
           <t>Subvention</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G17" s="7" t="n">
-        <v>7500</v>
-      </c>
       <c r="H17" s="7" t="n">
-        <v>30000</v>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>Environ 50 %</t>
-        </is>
+        <v>2000</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>10000</v>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
           <t>Ouvert en continu</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>Via un conseiller Mitacs en développement des affaires</t>
-        </is>
-      </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>FY27 T3</t>
+          <t>Via le même conseiller</t>
         </is>
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="N17" s="8" t="inlineStr">
-        <is>
-          <t>Stagiaires universitaires, postdoctoraux et chercheurs intégrés à un projet d'innovation en entreprise. Financement partagé MEIE, entreprise, fédéral.</t>
+          <t>FY27 T1</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>Le meilleur véhicule pour faire caractériser la fibre en laboratoire : conductivité thermique du produit fini, tenue à la compression, comportement à l'humidité.</t>
-        </is>
-      </c>
-      <c r="P17" s="9" t="inlineStr">
-        <is>
-          <t>https://www.mitacs.ca/fr-ca/</t>
+          <t>Honoraires professionnels : diagnostic RH, mandat de consultation, coaching de gestion, accompagnement en gestion du changement.</t>
+        </is>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>Le virage manufacturier 2025-2026, avec mises à pied et redéfinition des rôles, est une gestion du changement documentée.</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/obtenir-conseils</t>
         </is>
       </c>
     </row>
@@ -1685,73 +1756,78 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>grand V — accompagnement technologique</t>
+          <t>Stages pratiques PSPE (Magnet, CTIC, TECHNATION, BioTalent)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>ESDC via partenaires sectoriels</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Service (sans dette)</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Subvention salariale</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G18" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="H18" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>Aucune</t>
-        </is>
+        <v>5000</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>15000</v>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Salaire avancé, remboursé après</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>En continu</t>
+          <t>Ouvert par trimestre scolaire</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>FY27 T3</t>
+          <t>Premier arrivé, premier servi</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
+          <t>FY27 T2</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
           <t>Faible</t>
         </is>
       </c>
-      <c r="N18" s="8" t="inlineStr">
-        <is>
-          <t>Jusqu'à 100 heures d'experts en innovation. Séparable du volet financement, qui lui est hors de portée.</t>
-        </is>
-      </c>
       <c r="O18" s="8" t="inlineStr">
         <is>
-          <t>Couvre le prototypage d'équipements sur mesure et la valorisation des résidus. Demander SANS le prêt de 250 000 $.</t>
-        </is>
-      </c>
-      <c r="P18" s="9" t="inlineStr">
-        <is>
-          <t>https://grandv.investquebec.com/</t>
+          <t>5 000 $ par stage d'étudiant postsecondaire. Postes à composante numérique ou technologique priorisés.</t>
+        </is>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>Un poste en commerce électronique, automatisation ou données qualifie sans forcer. Déposer chez UN SEUL partenaire : c'est la même enveloppe fédérale.</t>
+        </is>
+      </c>
+      <c r="Q18" s="9" t="inlineStr">
+        <is>
+          <t>https://swpprogram.ca/fr/</t>
         </is>
       </c>
     </row>
@@ -1761,73 +1837,78 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Fonds Écoleader — Biodiversité</t>
+          <t>Emplois d'été Canada</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>FAQDD / MELCCFP</t>
+          <t>Emploi et Développement social Canada</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Contribution non remboursable</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="n">
-        <v>10000</v>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Subvention salariale</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
+        </is>
       </c>
       <c r="H19" s="7" t="n">
-        <v>40000</v>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>Environ 25 %</t>
-        </is>
+        <v>3000</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>8000</v>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Modalités non publiées</t>
+          <t>50 % du salaire minimum</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>Annoncé pour le printemps 2026, en retard — relancer chaque mois au 418 692-5888</t>
+          <t>Fermé — rouvre vers novembre 2026</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>FY27 T3</t>
+          <t>Date limite attendue ~11 décembre 2026 pour l'été 2027</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="N19" s="8" t="inlineStr">
-        <is>
-          <t>Enveloppe de 5,7 M$, 2026-2028, Plan nature 2030. Entreprises de toutes tailles. Paie des experts pour intégrer la biodiversité.</t>
+          <t>FY27 T2</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O19" s="8" t="inlineStr">
         <is>
-          <t>Fit exceptionnel : la thèse d'affaires entière de Lasclay est de rendre l'asclépiade viable pour restaurer l'habitat du monarque.</t>
-        </is>
-      </c>
-      <c r="P19" s="9" t="inlineStr">
-        <is>
-          <t>https://faqdd.qc.ca/programmes/fonds-ecoleader-biodiversite/</t>
+          <t>Secteur privé : jusqu'à 50 % du salaire minimum en vigueur. Jeunes de 15 à 30 ans, postes à temps plein.</t>
+        </is>
+      </c>
+      <c r="P19" s="8" t="inlineStr">
+        <is>
+          <t>Renfort d'atelier ou d'expédition pour la production estivale, en amont de la saison hivernale.</t>
+        </is>
+      </c>
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/emploi-developpement-social/services/financement/emplois-ete-canada.html</t>
         </is>
       </c>
     </row>
@@ -1837,12 +1918,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>CanExport PME</t>
+          <t>Riipen — Level UP</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Affaires mondiales Canada</t>
+          <t>Riipen</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -1852,58 +1933,63 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
           <t>Subvention</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G20" s="7" t="n">
-        <v>10000</v>
-      </c>
       <c r="H20" s="7" t="n">
-        <v>50000</v>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>50 %</t>
-        </is>
+        <v>1400</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>4200</v>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Ouvert jusqu'au 31 août 2026, 12 h</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>Rouvre vers le 4 février 2027 pour l'exercice 2027-28</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
+          <t>Par semestre universitaire</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
           <t>FY27 T2</t>
         </is>
       </c>
-      <c r="M20" s="5" t="inlineStr">
-        <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="N20" s="8" t="inlineStr">
-        <is>
-          <t>Enveloppe É.-U. de 3,1 M$ ENTIÈREMENT ALLOUÉE. Cible les marchés où l'entreprise a peu ou pas d'activités. 50 % des coûts, projet de 20 k$ à 100 k$.</t>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O20" s="8" t="inlineStr">
         <is>
-          <t>Viser la France, la Belgique et les pays nordiques, où le récit du monarque se transpose. Pas les États-Unis. Bâtir le dossier d'ici février plutôt que d'improviser en 26 jours.</t>
-        </is>
-      </c>
-      <c r="P20" s="9" t="inlineStr">
-        <is>
-          <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/soutien-financier-expansion-commerciale-international/canexport-pme/nouveau-2026-2027.html</t>
+          <t>1 400 $ par étudiant. Projets de 60 heures sur 2 à 8 semaines, encadrés par un enseignant.</t>
+        </is>
+      </c>
+      <c r="P20" s="8" t="inlineStr">
+        <is>
+          <t>Format parfait pour des mandats bornés : localisation des fiches produits pour les marchés américains, refonte du guide de plantation, analyse de saisonnalité.</t>
+        </is>
+      </c>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>https://fr.riipen.com/levelup/employers</t>
         </is>
       </c>
     </row>
@@ -1913,73 +1999,78 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>CERI — Expansion des entreprises et productivité</t>
+          <t>Capitale-Innovation</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Développement économique Canada</t>
+          <t>Ville de Québec</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Municipal</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Contribution remboursable à 0 %</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Contribution non remboursable</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>À valider</t>
         </is>
       </c>
-      <c r="G21" s="7" t="n">
-        <v>25000</v>
-      </c>
       <c r="H21" s="7" t="n">
-        <v>250000</v>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>50 %</t>
-        </is>
+        <v>50000</v>
+      </c>
+      <c r="I21" s="7" t="n">
+        <v>500000</v>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>50 %, puis 60 % au-delà de 250 k$</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>En continu</t>
+          <t>Volet ouvert (page à jour le 8 juillet 2026)</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>FY27 T4</t>
+          <t>Enveloppe Vision Québec 2030 possiblement fermée depuis le 31 mars 2026 — à faire trancher</t>
         </is>
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
+          <t>FY28 T3</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
           <t>Élevé</t>
         </is>
       </c>
-      <c r="N21" s="8" t="inlineStr">
-        <is>
-          <t>Aucun seuil de revenus, contrairement à l'IRRT. Secteurs admissibles : manufacturier, transformation alimentaire, TIC, sciences de la vie. Commerce de détail EXPLICITEMENT EXCLU.</t>
-        </is>
-      </c>
       <c r="O21" s="8" t="inlineStr">
         <is>
-          <t>Le dossier doit se présenter comme manufacturier — atelier de Limoilou, transformation de l'isolant, code d'activité — et non comme du commerce en ligne. 0 % d'intérêt, remboursements 2 ans après la fin.</t>
-        </is>
-      </c>
-      <c r="P21" s="9" t="inlineStr">
-        <is>
-          <t>https://www.canada.ca/fr/developpement-economique-regions-quebec/financement-services/expansion-des-entreprises-et-productivite.html</t>
+          <t>Secteur « Manufacturier, matériaux, transformation industrielle » explicitement admissible. Siège dans l'agglomération de Québec : rempli (1286 av. de la Ronde).</t>
+        </is>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Le plus gros non remboursable accessible localement. Exige la preuve de détention de la PI. Cumul de toute aide publique plafonné à 70 %.</t>
+        </is>
+      </c>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/innovation/capitale-innovation.aspx</t>
         </is>
       </c>
     </row>
@@ -1989,73 +2080,78 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Capitale-Innovation</t>
+          <t>Validation de principe</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Ville de Québec</t>
+          <t>Produits naturels Canada</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Contribution non remboursable</t>
-        </is>
-      </c>
-      <c r="F22" s="10" t="inlineStr">
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Financement remboursable</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
         <is>
           <t>À valider</t>
         </is>
       </c>
-      <c r="G22" s="7" t="n">
+      <c r="H22" s="7" t="n">
         <v>50000</v>
       </c>
-      <c r="H22" s="7" t="n">
-        <v>500000</v>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>50 %, puis 60 % au-delà de 250 k$</t>
-        </is>
+      <c r="I22" s="7" t="n">
+        <v>250000</v>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Volet ouvert (page à jour le 8 juillet 2026)</t>
+          <t>60 %</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>Enveloppe Vision Québec 2030 possiblement fermée depuis le 31 mars 2026 — à faire trancher</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>FY28 T3</t>
+          <t>Demande à tout moment</t>
         </is>
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
+          <t>FY28 T4</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
           <t>Élevé</t>
         </is>
       </c>
-      <c r="N22" s="8" t="inlineStr">
-        <is>
-          <t>Secteur « Manufacturier, matériaux, transformation industrielle » explicitement admissible. Siège dans l'agglomération de Québec : rempli (1286 av. de la Ronde).</t>
-        </is>
-      </c>
       <c r="O22" s="8" t="inlineStr">
         <is>
-          <t>Le plus gros non remboursable accessible localement. Exige la preuve de détention de la PI. Cumul de toute aide publique plafonné à 70 %.</t>
-        </is>
-      </c>
-      <c r="P22" s="9" t="inlineStr">
-        <is>
-          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/innovation/capitale-innovation.aspx</t>
+          <t>40 % des coûts, maximum 250 000 $. PNC cherche un potentiel de 10 à 15 M$ de revenus annuels — un cran au-dessus de la trajectoire de Lasclay.</t>
+        </is>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Réserve sérieuse sur le critère de potentiel de revenus. À tenter seulement si le volet cosmétique prend de l'ampleur.</t>
+        </is>
+      </c>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>https://www.naturalproductscanada.com/fr/programmes/programme-validation-de-principe/</t>
         </is>
       </c>
     </row>
@@ -2065,73 +2161,78 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Programme Innovation — Volet 1</t>
+          <t>Bons d'accompagnement à la croissance</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>MEIE</t>
+          <t>Ville de Québec</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Municipal</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Reporté</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="n">
-        <v>50000</v>
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Contribution</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>500000</v>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>25 % en argent</t>
-        </is>
+        <v>5000</v>
+      </c>
+      <c r="I23" s="7" t="n">
+        <v>20000</v>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>N'accepte pas les demandes</t>
+          <t>Variable</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>Surveiller la réouverture</t>
+          <t>Ouvert, dépôt en continu</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>Aucune date de tombée</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
-        </is>
-      </c>
-      <c r="N23" s="8" t="inlineStr">
-        <is>
-          <t>Jusqu'à 500 000 $ par entreprise. Contribution privée EN ARGENT d'au moins 25 % des dépenses admissibles.</t>
+          <t>FY27 T4</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O23" s="8" t="inlineStr">
         <is>
-          <t>ABSENT du répertoire Innoveici : c'est un angle mort du premier tri. Pendant provincial de Capitale-Innovation, à surveiller activement.</t>
-        </is>
-      </c>
-      <c r="P23" s="9" t="inlineStr">
-        <is>
-          <t>https://www.economie.gouv.qc.ca/bibliotheques/programmes/aide-financiere/programme-innovation</t>
+          <t>Exclut explicitement les commerces opérant UNIQUEMENT en ligne.</t>
+        </is>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>L'atelier de Limoilou et la transformation de l'isolant sortent Lasclay de l'exclusion, mais il faut l'énoncer clairement dans la demande.</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/productivite/bons-accompagnement.aspx</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2242,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>ESSOR — Volet 1 (études préalables)</t>
+          <t>Panorama</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -2156,58 +2257,63 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="n">
-        <v>5000</v>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Prêt</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
+        </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>50000</v>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
+        <v>250000</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>1000000</v>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Capacité de crédit</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>Dépôt en continu</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>FY28 T3</t>
+          <t>Après retour à la rentabilité</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="N24" s="8" t="inlineStr">
-        <is>
-          <t>Études de faisabilité, diagnostic numérique, plan numérique. Entreprises de tous secteurs.</t>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>Élevé</t>
         </is>
       </c>
       <c r="O24" s="8" t="inlineStr">
         <is>
-          <t>Porte d'entrée à faible risque avant tout projet d'équipement financé par ESSOR volet 2.</t>
-        </is>
-      </c>
-      <c r="P24" s="9" t="inlineStr">
-        <is>
-          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-la-concretisation-de-projets-dinvestissement</t>
+          <t>Prêt de fonds de roulement export, moratoire de capital de 24 mois, SANS sûreté ni caution corporative ou personnelle. EXCLUT les États-Unis.</t>
+        </is>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Structure rare et attrayante, mais hors de portée avec un avoir de -254 035 $ et 584 320 $ de dette portant intérêt.</t>
+        </is>
+      </c>
+      <c r="Q24" s="9" t="inlineStr">
+        <is>
+          <t>https://exportation.investquebec.com/solutions</t>
         </is>
       </c>
     </row>
@@ -2217,73 +2323,78 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Bons d'accompagnement à la croissance</t>
+          <t>ESSOR — Volet 4 (internationalisation)</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Ville de Québec</t>
+          <t>Investissement Québec</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Contribution</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="n">
-        <v>5000</v>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Prêt ou garantie</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
+        </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>20000</v>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
+        <v>50000</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>500000</v>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Ouvert, dépôt en continu</t>
+          <t>Capacité de crédit</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>Aucune date de tombée</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>FY27 T4</t>
+          <t>Si le développement É.-U. passe par de la distribution locale</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
-        </is>
-      </c>
-      <c r="N25" s="8" t="inlineStr">
-        <is>
-          <t>Exclut explicitement les commerces opérant UNIQUEMENT en ligne.</t>
+          <t>FY28 T4</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Élevé</t>
         </is>
       </c>
       <c r="O25" s="8" t="inlineStr">
         <is>
-          <t>L'atelier de Limoilou et la transformation de l'isolant sortent Lasclay de l'exclusion, mais il faut l'énoncer clairement dans la demande.</t>
-        </is>
-      </c>
-      <c r="P25" s="9" t="inlineStr">
-        <is>
-          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/productivite/bons-accompagnement.aspx</t>
+          <t>Vise les stratégies d'internationalisation complexes : entités, entrepôts, chaînes d'approvisionnement à l'étranger.</t>
+        </is>
+      </c>
+      <c r="P25" s="8" t="inlineStr">
+        <is>
+          <t>Ne se justifie pas tant que les États-Unis sont servis par expédition directe depuis Québec.</t>
+        </is>
+      </c>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-linternationalisation-des-entreprises</t>
         </is>
       </c>
     </row>
@@ -2293,73 +2404,78 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Prêts aux entreprises</t>
+          <t>Programme Innovation — Volet 1</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Ville de Québec</t>
+          <t>MEIE</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Prêt</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>25000</v>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
+        </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>150000</v>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>Capacité de crédit</t>
-        </is>
+        <v>50000</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>500000</v>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>25 % en argent</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>En continu</t>
+          <t>N'accepte pas les demandes</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>FY28 T1</t>
+          <t>Surveiller la réouverture</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="N26" s="8" t="inlineStr">
-        <is>
-          <t>Quatre volets : démarrage, amélioration et transformation, croissance et expansion, relève.</t>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Élevé</t>
         </is>
       </c>
       <c r="O26" s="8" t="inlineStr">
         <is>
-          <t>Le volet « amélioration et transformation » colle au virage manufacturier. La capacité de crédit reste à démontrer avec un avoir négatif.</t>
-        </is>
-      </c>
-      <c r="P26" s="9" t="inlineStr">
-        <is>
-          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/autres/prets-aux-entreprises/index.aspx</t>
+          <t>Jusqu'à 500 000 $ par entreprise. Contribution privée EN ARGENT d'au moins 25 % des dépenses admissibles.</t>
+        </is>
+      </c>
+      <c r="P26" s="8" t="inlineStr">
+        <is>
+          <t>ABSENT du répertoire Innoveici : c'est un angle mort du premier tri. Pendant provincial de Capitale-Innovation, à surveiller activement.</t>
+        </is>
+      </c>
+      <c r="Q26" s="9" t="inlineStr">
+        <is>
+          <t>https://www.economie.gouv.qc.ca/bibliotheques/programmes/aide-financiere/programme-innovation</t>
         </is>
       </c>
     </row>
@@ -2369,73 +2485,78 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Primo-adoptants</t>
+          <t>Programme canadien de l'innovation à l'international</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>MEIE</t>
+          <t>Affaires mondiales Canada</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Subvention (versée au partenaire)</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="n">
-        <v>0</v>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>20 % en espèces</t>
-        </is>
+        <v>15000</v>
+      </c>
+      <c r="I27" s="7" t="n">
+        <v>600000</v>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Appel de projets</t>
+          <t>50 %</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>Surveiller les appels</t>
+          <t>Dépôt ad hoc</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>FY28 T3</t>
+          <t>Ad hoc</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="N27" s="8" t="inlineStr">
-        <is>
-          <t>Lasclay serait le primo-adoptant, pas le bénéficiaire. La contribution du gouvernement va à la startup ; le primo-adoptant met 20 % en espèces.</t>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>Élevé</t>
         </is>
       </c>
       <c r="O27" s="8" t="inlineStr">
         <is>
-          <t>Manière peu coûteuse de faire tester sur la fibre des équipements d'automatisation ou de vision par ordinateur pour le contrôle qualité.</t>
-        </is>
-      </c>
-      <c r="P27" s="9" t="inlineStr">
-        <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/liste-partielle-aide-financiere/appels-projets-innovation/appel-primo-adoptants</t>
+          <t>Exige un partenaire de R-D au Brésil, en Chine, en Inde, en Israël ou en Corée du Sud.</t>
+        </is>
+      </c>
+      <c r="P27" s="8" t="inlineStr">
+        <is>
+          <t>La liste de pays ne recoupe pas la chaîne d'approvisionnement actuelle, qui passe par la Tunisie. À garder en veille seulement.</t>
+        </is>
+      </c>
+      <c r="Q27" s="9" t="inlineStr">
+        <is>
+          <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/programmes-soutien/programme-canadien-innovation-international.html</t>
         </is>
       </c>
     </row>
@@ -2445,12 +2566,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Accès aux talents</t>
+          <t>CERI — Expansion des entreprises et productivité</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Produits naturels Canada</t>
+          <t>Développement économique Canada</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -2460,58 +2581,63 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
-        </is>
-      </c>
-      <c r="F28" s="10" t="inlineStr">
+          <t>Ventes</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Contribution remboursable à 0 %</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
         <is>
           <t>À valider</t>
         </is>
       </c>
-      <c r="G28" s="7" t="n">
-        <v>20000</v>
-      </c>
       <c r="H28" s="7" t="n">
-        <v>75000</v>
-      </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>60 % du salaire</t>
-        </is>
+        <v>25000</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>250000</v>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
+          <t>50 %</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
           <t>Ouvert en continu</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr">
-        <is>
-          <t>Demande à tout moment</t>
-        </is>
-      </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>FY28 T1</t>
+          <t>En continu</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="N28" s="8" t="inlineStr">
-        <is>
-          <t>40 % du salaire d'un nouvel employé, maximum 75 000 $. Exige d'être membre de la grappe de l'innovation en produits naturels.</t>
+          <t>FY27 T4</t>
+        </is>
+      </c>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>Élevé</t>
         </is>
       </c>
       <c r="O28" s="8" t="inlineStr">
         <is>
-          <t>La définition de PNC — bioproduits et durabilité — couvre l'asclépiade. La collaboration cosmétique autour de l'huile de graine est le candidat naturel.</t>
-        </is>
-      </c>
-      <c r="P28" s="9" t="inlineStr">
-        <is>
-          <t>https://www.naturalproductscanada.com/fr/programmes/programme-daccess-aux-talents/</t>
+          <t>Aucun seuil de revenus, contrairement à l'IRRT. Secteurs admissibles : manufacturier, transformation alimentaire, TIC, sciences de la vie. Commerce de détail EXPLICITEMENT EXCLU.</t>
+        </is>
+      </c>
+      <c r="P28" s="8" t="inlineStr">
+        <is>
+          <t>RÉTROGRADÉ. Je recommandais de cadrer le dossier en manufacturier ; ce n'est plus la posture de l'entreprise, et le commerce de détail est un secteur exclu par DEC. Le seul crochet honnête qui reste est la transformation de l'isolant, qui se poursuit au Québec (91 336 $ de salaires de production aux livres en FY2026). À ne tenter que si DEC confirme d'avance que cette activité suffit à qualifier. Le volet commercialisation et développement des marchés du programme reste, lui, parfaitement aligné.</t>
+        </is>
+      </c>
+      <c r="Q28" s="9" t="inlineStr">
+        <is>
+          <t>https://www.canada.ca/fr/developpement-economique-regions-quebec/financement-services/expansion-des-entreprises-et-productivite.html</t>
         </is>
       </c>
     </row>
@@ -2521,73 +2647,78 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Contrat d'intégration au travail</t>
+          <t>Prêts aux entreprises</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Services Québec</t>
+          <t>Ville de Québec</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Municipal</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="n">
-        <v>3000</v>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Prêt</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20000</v>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>Part du salaire</t>
-        </is>
+        <v>25000</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>150000</v>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Capacité de crédit</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
           <t>En continu</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr">
-        <is>
-          <t>FY28</t>
-        </is>
-      </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
-        </is>
-      </c>
-      <c r="N29" s="8" t="inlineStr">
-        <is>
-          <t>Soutien au salaire pour compenser un écart de productivité, plus couverture de l'adaptation du poste.</t>
+          <t>FY28 T1</t>
+        </is>
+      </c>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O29" s="8" t="inlineStr">
         <is>
-          <t>Pertinent pour l'assemblage, l'emballage de semences et l'expédition, où les tâches se découpent bien.</t>
-        </is>
-      </c>
-      <c r="P29" s="9" t="inlineStr">
-        <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/recruter/contrat-integration-travail</t>
+          <t>Quatre volets : démarrage, amélioration et transformation, croissance et expansion, relève.</t>
+        </is>
+      </c>
+      <c r="P29" s="8" t="inlineStr">
+        <is>
+          <t>Le volet « amélioration et transformation » colle au virage manufacturier. La capacité de crédit reste à démontrer avec un avoir négatif.</t>
+        </is>
+      </c>
+      <c r="Q29" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/autres/prets-aux-entreprises/index.aspx</t>
         </is>
       </c>
     </row>
@@ -2612,56 +2743,61 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
           <t>Service gratuit</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
-      </c>
-      <c r="G30" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="H30" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I30" s="5" t="inlineStr">
+      <c r="I30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
         <is>
           <t>Aucune</t>
         </is>
       </c>
-      <c r="J30" s="5" t="inlineStr">
+      <c r="K30" s="5" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
       </c>
-      <c r="K30" s="5" t="inlineStr">
+      <c r="L30" s="5" t="inlineStr">
         <is>
           <t>En continu</t>
         </is>
       </c>
-      <c r="L30" s="5" t="inlineStr">
+      <c r="M30" s="5" t="inlineStr">
         <is>
           <t>FY27 T1</t>
         </is>
       </c>
-      <c r="M30" s="5" t="inlineStr">
+      <c r="N30" s="5" t="inlineStr">
         <is>
           <t>Faible</t>
         </is>
       </c>
-      <c r="N30" s="8" t="inlineStr">
+      <c r="O30" s="8" t="inlineStr">
         <is>
           <t>Accès gratuit à des conseils RH et juridiques, à une bibliothèque de modèles et de politiques.</t>
         </is>
       </c>
-      <c r="O30" s="8" t="inlineStr">
+      <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Zéro dollar en jeu, mais utile pour sécuriser les contrats et les politiques après une réduction d'effectifs.</t>
         </is>
       </c>
-      <c r="P30" s="9" t="inlineStr">
+      <c r="Q30" s="9" t="inlineStr">
         <is>
           <t>https://pratiquesrh.com/</t>
         </is>
@@ -2673,12 +2809,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>ICI on recycle +</t>
+          <t>Contrat d'intégration au travail</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Recyc-Québec</t>
+          <t>Services Québec</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -2688,58 +2824,63 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Attestation (clé d'accès)</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Subvention salariale</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>Admissible</t>
         </is>
       </c>
-      <c r="G31" s="7" t="n">
-        <v>-350</v>
-      </c>
       <c r="H31" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>350 $ de frais d'inscription</t>
-        </is>
+        <v>3000</v>
+      </c>
+      <c r="I31" s="7" t="n">
+        <v>20000</v>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Part du salaire</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
+          <t>Ouvert en continu</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
           <t>En continu</t>
         </is>
       </c>
-      <c r="L31" s="5" t="inlineStr">
+      <c r="M31" s="5" t="inlineStr">
         <is>
           <t>FY28</t>
         </is>
       </c>
-      <c r="M31" s="5" t="inlineStr">
+      <c r="N31" s="5" t="inlineStr">
         <is>
           <t>Faible</t>
         </is>
       </c>
-      <c r="N31" s="8" t="inlineStr">
-        <is>
-          <t>N'octroie pas d'aide. Écocondition OBLIGATOIRE, au niveau « Mise en œuvre », pour le versement final de plusieurs aides de Recyc-Québec.</t>
-        </is>
-      </c>
       <c r="O31" s="8" t="inlineStr">
         <is>
-          <t>C'est une clé, pas une source. Environ 350 $ pour déverrouiller les enveloppes de Recyc-Québec et crédibiliser les appels d'offres corporatifs.</t>
-        </is>
-      </c>
-      <c r="P31" s="9" t="inlineStr">
-        <is>
-          <t>https://www.recyc-quebec.gouv.qc.ca/entreprises-organismes/performer/programme-ici-on-recycle-plus/</t>
+          <t>Soutien au salaire pour compenser un écart de productivité, plus couverture de l'adaptation du poste.</t>
+        </is>
+      </c>
+      <c r="P31" s="8" t="inlineStr">
+        <is>
+          <t>Pertinent pour l'assemblage, l'emballage de semences et l'expédition, où les tâches se découpent bien.</t>
+        </is>
+      </c>
+      <c r="Q31" s="9" t="inlineStr">
+        <is>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/recruter/contrat-integration-travail</t>
         </is>
       </c>
     </row>
@@ -2749,73 +2890,78 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Validation de principe</t>
+          <t>Fonds économie circulaire</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Produits naturels Canada</t>
+          <t>Fondaction</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Financement remboursable</t>
-        </is>
-      </c>
-      <c r="F32" s="10" t="inlineStr">
+          <t>Mission</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Capital (dilution)</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
         <is>
           <t>À valider</t>
         </is>
       </c>
-      <c r="G32" s="7" t="n">
-        <v>50000</v>
-      </c>
       <c r="H32" s="7" t="n">
-        <v>250000</v>
-      </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>60 %</t>
-        </is>
+        <v>100000</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>500000</v>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Dilution du capital</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>Demande à tout moment</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>FY28 T4</t>
+          <t>En continu</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
           <t>Élevé</t>
         </is>
       </c>
-      <c r="N32" s="8" t="inlineStr">
-        <is>
-          <t>40 % des coûts, maximum 250 000 $. PNC cherche un potentiel de 10 à 15 M$ de revenus annuels — un cran au-dessus de la trajectoire de Lasclay.</t>
-        </is>
-      </c>
       <c r="O32" s="8" t="inlineStr">
         <is>
-          <t>Réserve sérieuse sur le critère de potentiel de revenus. À tenter seulement si le volet cosmétique prend de l'ampleur.</t>
-        </is>
-      </c>
-      <c r="P32" s="9" t="inlineStr">
-        <is>
-          <t>https://www.naturalproductscanada.com/fr/programmes/programme-validation-de-principe/</t>
+          <t>Cible les jeunes entreprises en phase de démarrage dont le modèle repose sur la circularité. C'est du capital, pas de la subvention.</t>
+        </is>
+      </c>
+      <c r="P32" s="8" t="inlineStr">
+        <is>
+          <t>Les semences issues de la transformation de la soie et la gamme « Les Imparfaits » sont de la circularité réelle. À ne considérer que si l'ouverture du capital devient une option assumée.</t>
+        </is>
+      </c>
+      <c r="Q32" s="9" t="inlineStr">
+        <is>
+          <t>https://www.fondaction.com/entreprise/fonds-economie-circulaire/</t>
         </is>
       </c>
     </row>
@@ -2825,12 +2971,12 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Panorama</t>
+          <t>ICI on recycle +</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>Recyc-Québec</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -2840,58 +2986,63 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Prêt</t>
-        </is>
-      </c>
-      <c r="F33" s="11" t="inlineStr">
-        <is>
-          <t>Reporté</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="n">
-        <v>250000</v>
+          <t>Mission</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Attestation (clé d'accès)</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
+        </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>Capacité de crédit</t>
-        </is>
+        <v>-350</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
+          <t>350 $ de frais d'inscription</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
           <t>Ouvert</t>
         </is>
       </c>
-      <c r="K33" s="5" t="inlineStr">
-        <is>
-          <t>Après retour à la rentabilité</t>
-        </is>
-      </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
+          <t>En continu</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
           <t>FY28</t>
         </is>
       </c>
-      <c r="M33" s="5" t="inlineStr">
-        <is>
-          <t>Élevé</t>
-        </is>
-      </c>
-      <c r="N33" s="8" t="inlineStr">
-        <is>
-          <t>Prêt de fonds de roulement export, moratoire de capital de 24 mois, SANS sûreté ni caution corporative ou personnelle. EXCLUT les États-Unis.</t>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O33" s="8" t="inlineStr">
         <is>
-          <t>Structure rare et attrayante, mais hors de portée avec un avoir de -254 035 $ et 584 320 $ de dette portant intérêt.</t>
-        </is>
-      </c>
-      <c r="P33" s="9" t="inlineStr">
-        <is>
-          <t>https://exportation.investquebec.com/solutions</t>
+          <t>N'octroie pas d'aide. Écocondition OBLIGATOIRE, au niveau « Mise en œuvre », pour le versement final de plusieurs aides de Recyc-Québec.</t>
+        </is>
+      </c>
+      <c r="P33" s="8" t="inlineStr">
+        <is>
+          <t>C'est une clé, pas une source. Environ 350 $ pour déverrouiller les enveloppes de Recyc-Québec et crédibiliser les appels d'offres corporatifs.</t>
+        </is>
+      </c>
+      <c r="Q33" s="9" t="inlineStr">
+        <is>
+          <t>https://www.recyc-quebec.gouv.qc.ca/entreprises-organismes/performer/programme-ici-on-recycle-plus/</t>
         </is>
       </c>
     </row>
@@ -2901,7 +3052,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>ESSOR — Volet 2 (productivité et expansion)</t>
+          <t>grand V — accompagnement technologique</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -2916,58 +3067,63 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Contribution remboursable ou garantie</t>
-        </is>
-      </c>
-      <c r="F34" s="11" t="inlineStr">
-        <is>
-          <t>Reporté</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="n">
-        <v>50000</v>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Service (sans dette)</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
+        </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>500000</v>
-      </c>
-      <c r="I34" s="5" t="inlineStr">
-        <is>
-          <t>Capacité de crédit</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="I34" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
           <t>Ouvert en continu</t>
         </is>
       </c>
-      <c r="K34" s="5" t="inlineStr">
-        <is>
-          <t>Après un exercice FY2027 positif</t>
-        </is>
-      </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>FY28 T1</t>
+          <t>En continu</t>
         </is>
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
-        </is>
-      </c>
-      <c r="N34" s="8" t="inlineStr">
-        <is>
-          <t>Exige de démontrer un potentiel de hausse de rentabilité ou de masse salariale. Honoraires de gestion d'au moins 0,5 % du montant accordé.</t>
+          <t>FY27 T3</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O34" s="8" t="inlineStr">
         <is>
-          <t>Le raisonnement reste juste, il est prématuré d'un ou deux exercices. Rouvrir le dossier sur des états financiers montrant un redressement.</t>
-        </is>
-      </c>
-      <c r="P34" s="9" t="inlineStr">
-        <is>
-          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/essor-volet-2</t>
+          <t>Jusqu'à 100 heures d'experts en innovation. Séparable du volet financement, qui lui est hors de portée.</t>
+        </is>
+      </c>
+      <c r="P34" s="8" t="inlineStr">
+        <is>
+          <t>RÉTROGRADÉ : l'offre porte surtout sur la sélection d'équipements, la reconfiguration d'usine et le prototypage, qui ne sont plus des chantiers actifs. Reste utile pour l'amélioration de produits si un volet R&amp;D s'y prête.</t>
+        </is>
+      </c>
+      <c r="Q34" s="9" t="inlineStr">
+        <is>
+          <t>https://grandv.investquebec.com/</t>
         </is>
       </c>
     </row>
@@ -2977,7 +3133,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>grand V — financement</t>
+          <t>ESSOR — Volet 1 (études préalables)</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -2992,58 +3148,63 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Prêt à terme</t>
-        </is>
-      </c>
-      <c r="F35" s="11" t="inlineStr">
-        <is>
-          <t>Reporté</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="n">
-        <v>250000</v>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
+        </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>Capacité de crédit</t>
-        </is>
+        <v>5000</v>
+      </c>
+      <c r="I35" s="7" t="n">
+        <v>50000</v>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
           <t>Ouvert en continu</t>
         </is>
       </c>
-      <c r="K35" s="5" t="inlineStr">
-        <is>
-          <t>Après un exercice FY2027 positif</t>
-        </is>
-      </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>FY28 T1</t>
+          <t>Dépôt en continu</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
-        </is>
-      </c>
-      <c r="N35" s="8" t="inlineStr">
-        <is>
-          <t>Prêt MINIMUM de 250 000 $, moratoire de capital jusqu'à 48 mois. Devant -254 035 $ de capitaux propres et 584 320 $ de dette, l'analyse de crédit bloque.</t>
+          <t>FY28 T3</t>
+        </is>
+      </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O35" s="8" t="inlineStr">
         <is>
-          <t>C'était le levier identifié pour remplacer Merchant Growth et Shopify Capital. Il reste le bon levier, mais pas avant un redressement.</t>
-        </is>
-      </c>
-      <c r="P35" s="9" t="inlineStr">
-        <is>
-          <t>https://grandv.investquebec.com/</t>
+          <t>Études de faisabilité, diagnostic numérique, plan numérique. Entreprises de tous secteurs.</t>
+        </is>
+      </c>
+      <c r="P35" s="8" t="inlineStr">
+        <is>
+          <t>Porte d'entrée à faible risque avant tout projet d'équipement financé par ESSOR volet 2.</t>
+        </is>
+      </c>
+      <c r="Q35" s="9" t="inlineStr">
+        <is>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-la-concretisation-de-projets-dinvestissement</t>
         </is>
       </c>
     </row>
@@ -3053,12 +3214,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>ESSOR — Volet 4 (internationalisation)</t>
+          <t>C3i — investissement et innovation</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>Revenu Québec</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -3068,58 +3229,63 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Prêt ou garantie</t>
-        </is>
-      </c>
-      <c r="F36" s="11" t="inlineStr">
-        <is>
-          <t>Reporté</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="n">
-        <v>50000</v>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Crédit d'impôt remboursable</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>500000</v>
-      </c>
-      <c r="I36" s="5" t="inlineStr">
-        <is>
-          <t>Capacité de crédit</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>25000</v>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>L'achat d'équipement lui-même</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>Si le développement É.-U. passe par de la distribution locale</t>
+          <t>En vigueur</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>FY28 T4</t>
+          <t>Avec la déclaration fiscale annuelle</t>
         </is>
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
-        </is>
-      </c>
-      <c r="N36" s="8" t="inlineStr">
-        <is>
-          <t>Vise les stratégies d'internationalisation complexes : entités, entrepôts, chaînes d'approvisionnement à l'étranger.</t>
+          <t>FY27-FY28</t>
+        </is>
+      </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O36" s="8" t="inlineStr">
         <is>
-          <t>Ne se justifie pas tant que les États-Unis sont servis par expédition directe depuis Québec.</t>
-        </is>
-      </c>
-      <c r="P36" s="9" t="inlineStr">
-        <is>
-          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-linternationalisation-des-entreprises</t>
+          <t>15 % à 25 % du coût du matériel de fabrication et transformation (catégorie 53) et des logiciels de gestion, utilisé au Québec 730 jours consécutifs.</t>
+        </is>
+      </c>
+      <c r="P36" s="8" t="inlineStr">
+        <is>
+          <t>RÉTROGRADÉ : le crédit porte sur l'ACQUISITION de matériel de fabrication, et il n'y a plus de programme d'achat d'équipement. Ne se cumule pas avec le CRIC sur la même dépense. À réactiver seulement si un achat d'équipement revient au plan.</t>
+        </is>
+      </c>
+      <c r="Q36" s="9" t="inlineStr">
+        <is>
+          <t>https://www.revenuquebec.ca/fr/entreprises/impots/impot-des-societes/credits-dimpot-des-societes/</t>
         </is>
       </c>
     </row>
@@ -3129,12 +3295,12 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Fonds économie circulaire</t>
+          <t>Primo-adoptants</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Fondaction</t>
+          <t>MEIE</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -3144,58 +3310,63 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Capital (dilution)</t>
-        </is>
-      </c>
-      <c r="F37" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="n">
-        <v>100000</v>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Subvention (versée au partenaire)</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
+        </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>500000</v>
-      </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>Dilution du capital</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="I37" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>20 % en espèces</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>En continu</t>
+          <t>Appel de projets</t>
         </is>
       </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>Surveiller les appels</t>
         </is>
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
-        </is>
-      </c>
-      <c r="N37" s="8" t="inlineStr">
-        <is>
-          <t>Cible les jeunes entreprises en phase de démarrage dont le modèle repose sur la circularité. C'est du capital, pas de la subvention.</t>
+          <t>FY28 T3</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O37" s="8" t="inlineStr">
         <is>
-          <t>Les semences issues de la transformation de la soie et la gamme « Les Imparfaits » sont de la circularité réelle. À ne considérer que si l'ouverture du capital devient une option assumée.</t>
-        </is>
-      </c>
-      <c r="P37" s="9" t="inlineStr">
-        <is>
-          <t>https://www.fondaction.com/entreprise/fonds-economie-circulaire/</t>
+          <t>Lasclay serait le primo-adoptant, pas le bénéficiaire. La contribution du gouvernement va à la startup ; le primo-adoptant met 20 % en espèces.</t>
+        </is>
+      </c>
+      <c r="P37" s="8" t="inlineStr">
+        <is>
+          <t>Manière peu coûteuse de faire tester sur la fibre des équipements d'automatisation ou de vision par ordinateur pour le contrôle qualité.</t>
+        </is>
+      </c>
+      <c r="Q37" s="9" t="inlineStr">
+        <is>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/liste-partielle-aide-financiere/appels-projets-innovation/appel-primo-adoptants</t>
         </is>
       </c>
     </row>
@@ -3205,165 +3376,283 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Programme canadien de l'innovation à l'international</t>
+          <t>ESSOR — Volet 2 (productivité et expansion)</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Affaires mondiales Canada</t>
+          <t>Investissement Québec</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
-        </is>
-      </c>
-      <c r="F38" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="n">
-        <v>15000</v>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Contribution remboursable ou garantie</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
+        </is>
       </c>
       <c r="H38" s="7" t="n">
-        <v>600000</v>
-      </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>50 %</t>
-        </is>
+        <v>50000</v>
+      </c>
+      <c r="I38" s="7" t="n">
+        <v>500000</v>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>Dépôt ad hoc</t>
+          <t>Capacité de crédit</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>Ad hoc</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>Après un exercice FY2027 positif</t>
         </is>
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
+          <t>FY28 T1</t>
+        </is>
+      </c>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
           <t>Élevé</t>
         </is>
       </c>
-      <c r="N38" s="8" t="inlineStr">
-        <is>
-          <t>Exige un partenaire de R-D au Brésil, en Chine, en Inde, en Israël ou en Corée du Sud.</t>
-        </is>
-      </c>
       <c r="O38" s="8" t="inlineStr">
         <is>
-          <t>La liste de pays ne recoupe pas la chaîne d'approvisionnement actuelle, qui passe par la Tunisie. À garder en veille seulement.</t>
-        </is>
-      </c>
-      <c r="P38" s="9" t="inlineStr">
-        <is>
-          <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/programmes-soutien/programme-canadien-innovation-international.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>Potentiel total, verdict « Admissible » seulement</t>
-        </is>
-      </c>
-      <c r="G40" s="13">
-        <f>SUMIF($F$5:$F$38,"Admissible",G5:G38)</f>
-        <v>121550</v>
-      </c>
-      <c r="H40" s="13">
-        <f>SUMIF($F$5:$F$38,"Admissible",H5:H38)</f>
-        <v>465200</v>
+          <t>Exige de démontrer un potentiel de hausse de rentabilité ou de masse salariale. Honoraires de gestion d'au moins 0,5 % du montant accordé.</t>
+        </is>
+      </c>
+      <c r="P38" s="8" t="inlineStr">
+        <is>
+          <t>Le raisonnement reste juste, il est prématuré d'un ou deux exercices. Rouvrir le dossier sur des états financiers montrant un redressement.</t>
+        </is>
+      </c>
+      <c r="Q38" s="9" t="inlineStr">
+        <is>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/essor-volet-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="58" customHeight="1">
+      <c r="A39" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>grand V — financement</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Investissement Québec</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Québec</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Prêt à terme</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="n">
+        <v>250000</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>Capacité de crédit</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>Ouvert en continu</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>Après un exercice FY2027 positif</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>FY28 T1</t>
+        </is>
+      </c>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>Élevé</t>
+        </is>
+      </c>
+      <c r="O39" s="8" t="inlineStr">
+        <is>
+          <t>Prêt MINIMUM de 250 000 $, moratoire de capital jusqu'à 48 mois. Devant -254 035 $ de capitaux propres et 584 320 $ de dette, l'analyse de crédit bloque.</t>
+        </is>
+      </c>
+      <c r="P39" s="8" t="inlineStr">
+        <is>
+          <t>C'était le levier identifié pour remplacer Merchant Growth et Shopify Capital. Il reste le bon levier, mais pas avant un redressement.</t>
+        </is>
+      </c>
+      <c r="Q39" s="9" t="inlineStr">
+        <is>
+          <t>https://grandv.investquebec.com/</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>Potentiel total, « Admissible » + « À valider »</t>
-        </is>
-      </c>
-      <c r="G41" s="13">
-        <f>SUMIF($F$5:$F$38,"Admissible",G5:G38)+SUMIF($F$5:$F$38,"À valider",G5:G38)</f>
-        <v>436550</v>
+          <t>Potentiel total, verdict « Admissible » seulement</t>
+        </is>
       </c>
       <c r="H41" s="13">
-        <f>SUMIF($F$5:$F$38,"Admissible",H5:H38)+SUMIF($F$5:$F$38,"À valider",H5:H38)</f>
-        <v>2905200</v>
+        <f>SUMIF($G$5:$G$39,"Admissible",H5:H39)</f>
+        <v>121550</v>
+      </c>
+      <c r="I41" s="13">
+        <f>SUMIF($G$5:$G$39,"Admissible",I5:I39)</f>
+        <v>465200</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="12" t="inlineStr">
         <is>
+          <t>Potentiel total, « Admissible » + « À valider »</t>
+        </is>
+      </c>
+      <c r="H42" s="13">
+        <f>SUMIF($G$5:$G$39,"Admissible",H5:H39)+SUMIF($G$5:$G$39,"À valider",H5:H39)</f>
+        <v>436550</v>
+      </c>
+      <c r="I42" s="13">
+        <f>SUMIF($G$5:$G$39,"Admissible",I5:I39)+SUMIF($G$5:$G$39,"À valider",I5:I39)</f>
+        <v>2905200</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
           <t>Dont admissible SANS aucune mise de fonds</t>
         </is>
       </c>
-      <c r="G42" s="13">
-        <f>SUMIFS(G5:G38,$F$5:$F$38,"Admissible",$I$5:$I$38,"Aucune")</f>
+      <c r="H43" s="13">
+        <f>SUMIFS(H5:H39,$G$5:$G$39,"Admissible",$J$5:$J$39,"Aucune")</f>
         <v>46400</v>
       </c>
-      <c r="H42" s="13">
-        <f>SUMIFS(H5:H38,$F$5:$F$38,"Admissible",$I$5:$I$38,"Aucune")</f>
+      <c r="I43" s="13">
+        <f>SUMIFS(I5:I39,$G$5:$G$39,"Admissible",$J$5:$J$39,"Aucune")</f>
         <v>74200</v>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="14" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>Notes de lecture</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="26" customHeight="1">
-      <c r="B45" s="15" t="inlineStr">
-        <is>
-          <t>• Montants min et max : fourchettes réalistes pour un dossier Lasclay, pas les plafonds théoriques des programmes. Ils servent à prioriser, pas à budgéter. Cas particulier du rang 5 (IQPH) : l'organisme ne publie aucun montant. La fourchette de 15 à 30 k$ est INFÉRÉE de son objectif public — 48 entreprises et 12 M$ d'investissements générés sur 6 ans, avec un effet de levier annoncé jusqu'à 10 fois — et doit être confirmée auprès d'eux.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="26" customHeight="1">
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>• Verdicts : « Admissible » = tous les critères publiés sont rencontrés. « À valider » = un critère dépend d'un arbitrage, d'un cadrage ou d'une confirmation de l'organisme. « Reporté » = admissible sur papier, hors de portée financièrement aujourd'hui.</t>
+          <t>• Montants min et max : fourchettes réalistes pour un dossier Lasclay, pas les plafonds théoriques des programmes. Ils servent à prioriser, pas à budgéter. Cas particulier du rang 5 (IQPH) : l'organisme ne publie aucun montant. La fourchette de 15 à 30 k$ est INFÉRÉE de son objectif public — 48 entreprises et 12 M$ d'investissements générés sur 6 ans, avec un effet de levier annoncé jusqu'à 10 fois — et doit être confirmée auprès d'eux.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="26" customHeight="1">
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>• La contrainte dominante n'est pas l'admissibilité, c'est la mise de fonds : trésorerie de -2 060 $ et marge EDC utilisée à 94,8 %. D'où la priorité donnée aux crédits d'impôt et aux subventions salariales, qui remboursent des dépenses déjà engagées.</t>
+          <t>• Verdicts : « Admissible » = tous les critères publiés sont rencontrés. « À valider » = un critère dépend d'un arbitrage, d'un cadrage ou d'une confirmation de l'organisme. « Reporté » = admissible sur papier, hors de portée financièrement aujourd'hui.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="26" customHeight="1">
       <c r="B48" s="15" t="inlineStr">
         <is>
+          <t>• La contrainte dominante n'est pas l'admissibilité, c'est la mise de fonds : trésorerie de -2 060 $ et marge EDC utilisée à 94,8 %. D'où la priorité donnée aux crédits d'impôt et aux subventions salariales, qui remboursent des dépenses déjà engagées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1">
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>• Colonne Pilier : le classement suit les quatre priorités de l'entreprise — mission, ventes, international, R&amp;D. Lasclay n'est plus manufacturier pour le moment, ce qui fait reculer tout ce qui repose sur l'achat d'équipement, la productivité d'usine ou le statut de secteur manufacturier : C3i, ESSOR, grand V, Primo-adoptants et DEC Expansion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="26" customHeight="1">
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>• Nuance à tenir : les livres portent encore 91 336 $ de salaires de production et 135 851 $ d'équipements en FY2026. Ne pas se déclarer manufacturier devant un programme et s'en réclamer devant un autre — choisir une version et la tenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>• Colonne Pilier : le classement suit les quatre priorités de l'entreprise, soit mission, ventes, international et R&amp;D. Lasclay n'est plus manufacturier pour le moment, ce qui fait reculer tout ce qui repose sur l'achat d'équipement, la productivité d'usine ou le statut de secteur manufacturier : C3i, ESSOR, grand V, Primo-adoptants et DEC Expansion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="26" customHeight="1">
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>• Nuance à tenir : les livres portent encore 91 336 $ de salaires de production et 135 851 $ d'équipements en FY2026. Ne pas se déclarer non manufacturier devant un programme et s'en réclamer devant un autre. Choisir une version et la tenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="B53" s="15" t="inlineStr">
+        <is>
           <t>• Sources vérifiées le 5 août 2026 aux sites officiels des organismes. Les statuts de programme changent sans préavis : revalider avant tout dépôt.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:P38"/>
-  <mergeCells count="6">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="B47:H47"/>
-    <mergeCell ref="B48:H48"/>
-    <mergeCell ref="B45:H45"/>
-    <mergeCell ref="B46:H46"/>
+  <autoFilter ref="A4:Q39"/>
+  <mergeCells count="10">
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="B52:I52"/>
+    <mergeCell ref="B48:I48"/>
+    <mergeCell ref="B53:I53"/>
+    <mergeCell ref="B47:I47"/>
+    <mergeCell ref="B51:I51"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="B50:I50"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4055,7 +4344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4799,30 +5088,94 @@
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
+          <t>Trimestriel, dès sept 2026</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>FY2027 — continu</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Vérifier la réouverture du PSCE volet 2, et s'il a été remplacé par un autre véhicule d'aide à l'export</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>PSCE volet 2</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Veille active</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>60 000 $ non remboursables ; Lasclay vient tout juste de franchir le seuil de 1 M$</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Trimestriel, dès sept 2026</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>FY2027 — continu</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Vérifier la réouverture du PSCE volet 2, et s'il a été remplacé par un autre véhicule d'aide à l'export</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>PSCE volet 2</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Veille active</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>60 000 $ non remboursables ; le seuil de 1 M$ vient tout juste d'être franchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
           <t>Janvier 2027, puis janvier 2028</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Annuel</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Rebalayer le répertoire Innoveici : 88 des 208 programmes étaient fermés au 5 août 2026</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D30" s="8" t="inlineStr">
         <is>
           <t>Veille</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>Récurrent</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr"/>
+      <c r="F30" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5241,7 +5594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -5509,20 +5862,64 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
+          <t>Investissement Québec — PSCE volet 2</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Seuil d'admissibilité : chiffre d'affaires supérieur à 1 M$ et jusqu'à 50 M$. Aide maximale de 60 000 $ par entreprise par année, non remboursable. Statut fermé au 5 août 2026.</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/programme-de-soutien-la-commercialisation-et-lexportation/psce-volet-2</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Investissement Québec — PSCE volet 2</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Seuil d'admissibilité : chiffre d'affaires supérieur à 1 M$ et jusqu'à 50 M$. Aide maximale de 60 000 $ par entreprise par année, non remboursable. Statut fermé au 5 août 2026.</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/programme-de-soutien-la-commercialisation-et-lexportation/psce-volet-2</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>QuickBooks Online — Les Produits Lasclay Inc</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Tous les chiffres opposés aux critères : revenus, résultat, trésorerie, capitaux propres, dette, assiette R-D.</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>(accès interne via le Finance Proxy)</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>

</xml_diff>

<commit_message>
Ajouter les concours et bourses, absents des répertoires publics
Nouvel onglet « Concours et bourses » : TELUS AidonsNosPME, Défi OSEntreprendre
volet Réussite inc., Mercuriades, Phénix de l'environnement, Ascension JCCQ,
La Ruche, Dans l'Oeil du Dragon et FedEx BackingSmall.

TELUS entre au rang 4 du plan : l'édition 2026 ferme le 2 septembre, Lasclay a
déjà gagné une édition, aucune mise de fonds n'est exigée et les prix vont
jusqu'à 125 000 $. Ajouté au calendrier comme limite ferme.

Deux dossiers de concours déjà ouverts sont repérés dans la boîte Missive et
attendent une décision : La Ruche et Dans l'Oeil du Dragon.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UvYqHAWmt8Vm4vpbKQ1Pmv
</commit_message>
<xml_diff>
--- a/financement/Financement_Lasclay_2026.xlsx
+++ b/financement/Financement_Lasclay_2026.xlsx
@@ -12,9 +12,10 @@
     <sheet name="Calendrier 24 mois" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Diagnostic QBO" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Concours et bourses" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan priorisé'!$A$4:$Q$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan priorisé'!$A$4:$Q$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -154,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -209,6 +210,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -574,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:Q54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -946,27 +950,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>CanExport PME</t>
+          <t>TELUS #AidonsNosPME — 5e édition</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Affaires mondiales Canada</t>
+          <t>TELUS Affaires</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Fédéral (privé)</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>International</t>
+          <t>Mission et ventes</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
+          <t>Concours — bourse non remboursable</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -978,46 +982,46 @@
         <v>10000</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>50000</v>
+        <v>125000</v>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>50 %</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>Ouvert jusqu'au 31 août 2026, 12 h</t>
+          <t>OUVERT — ferme le 2 septembre 2026 à 23 h 59</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Rouvre vers le 4 février 2027 pour l'exercice 2027-28</t>
+          <t>Dépôt d'ici le 2 septembre 2026. Lauréats annoncés vers le 24 septembre.</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>FY27 T2</t>
+          <t>FY2026 — CE MOIS-CI</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>Enveloppe É.-U. de 3,1 M$ ENTIÈREMENT ALLOUÉE. Cible les marchés où l'entreprise a peu ou pas d'activités. 50 % des coûts, projet de 20 k$ à 100 k$.</t>
+          <t>Entreprise canadienne en activité, légalement enregistrée, générant des revenus, 100 employés ou moins. Rempli. Édition 2026 : 3 grands prix jusqu'à 125 000 $, 6 prix communautaires de 10 000 $, 1 prix du public de 25 000 $ par vote. Plus de 1 M$ au total. Aucune clause excluant les anciens lauréats dans le règlement consulté — à faire confirmer par TELUS.</t>
         </is>
       </c>
       <c r="P8" s="8" t="inlineStr">
         <is>
-          <t>Viser la France, la Belgique et les pays nordiques, où le récit du monarque se transpose. Pas les États-Unis. Bâtir le dossier d'ici février plutôt que d'improviser en 26 jours.</t>
+          <t>LE SEUL ARGENT SUR LA TABLE CE MOIS-CI. Lasclay a déjà gagné une édition : le dossier existe, le récit convainc ce jury, et l'effort de redéposer est faible. C'est une loterie — une dizaine de gagnants pour des milliers de candidatures — mais une loterie à coût quasi nul, sans mise de fonds, avec un prix du public qui récompense une communauté engagée. C'est exactement l'actif de Lasclay.</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/soutien-financier-expansion-commerciale-international/canexport-pme/nouveau-2026-2027.html</t>
+          <t>https://www.telus.com/fr/business/small/campaigns/stand-with-owners</t>
         </is>
       </c>
     </row>
@@ -1027,58 +1031,58 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Prêt d'honneur IQPH</t>
+          <t>CanExport PME</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Initiative Québec Prêt d'Honneur</t>
+          <t>Affaires mondiales Canada</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Québec (Capitale-Nationale)</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Mission et ventes</t>
+          <t>International</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Prêt SANS INTÉRÊT ni garantie</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>30000</v>
+        <v>50000</v>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Aucune</t>
+          <t>50 %</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>Ouvert — dépôt en continu</t>
+          <t>Ouvert jusqu'au 31 août 2026, 12 h</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Envoi des documents à candidature@iqph.org</t>
+          <t>Rouvre vers le 4 février 2027 pour l'exercice 2027-28</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>FY27 T1</t>
+          <t>FY27 T2</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
@@ -1088,17 +1092,17 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>Territoire pilote : agglomération de Québec — rempli. Phases admissibles : démarrage, CROISSANCE et repreneuriat. Prêt sans intérêt, sans frais de dossier et sans garantie personnelle. Sélection à deux niveaux : qualités entrepreneuriales et projet, puis productivité, innovation, commercialisation et développement durable. Montant fixé au cas par cas par le comité d'approbation — non publié.</t>
+          <t>Enveloppe É.-U. de 3,1 M$ ENTIÈREMENT ALLOUÉE. Cible les marchés où l'entreprise a peu ou pas d'activités. 50 % des coûts, projet de 20 k$ à 100 k$.</t>
         </is>
       </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
-          <t>Aucune mise de fonds et zéro intérêt : c'est le seul financement de la liste qui attaque directement les 53 074 $ d'intérêts. Organisme en phase pilote (objectif : 48 entreprises sur 6 ans) qui cherche des dossiers vitrines — la notoriété de Lasclay joue pour. DEUX RÉSERVES : le prêt vise à renforcer les fonds propres pour lever du financement institutionnel, or ils sont à -254 035 $, ce qui est autant l'argument que le risque devant le comité ; et l'accompagnement par un mentor est obligatoire pendant toute la durée du contrat. À CLARIFIER AVEC EUX : le prêt est-il consenti à l'entreprise ou à l'entrepreneur personnellement ?</t>
+          <t>Viser la France, la Belgique et les pays nordiques, où le récit du monarque se transpose. Pas les États-Unis. Bâtir le dossier d'ici février plutôt que d'improviser en 26 jours.</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>https://www.iqph.org/</t>
+          <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/soutien-financier-expansion-commerciale-international/canexport-pme/nouveau-2026-2027.html</t>
         </is>
       </c>
     </row>
@@ -1108,27 +1112,27 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Fonds Écoleader — Biodiversité</t>
+          <t>Prêt d'honneur IQPH</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>FAQDD / MELCCFP</t>
+          <t>Initiative Québec Prêt d'Honneur</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Québec (Capitale-Nationale)</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Mission</t>
+          <t>Mission et ventes</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Contribution non remboursable</t>
+          <t>Prêt SANS INTÉRÊT ni garantie</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -1137,29 +1141,29 @@
         </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>40000</v>
+        <v>30000</v>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Environ 25 %</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>Modalités non publiées</t>
+          <t>Ouvert — dépôt en continu</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Annoncé pour le printemps 2026, en retard — relancer chaque mois au 418 692-5888</t>
+          <t>Envoi des documents à candidature@iqph.org</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>FY27 T3</t>
+          <t>FY27 T1</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
@@ -1169,17 +1173,17 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>Enveloppe de 5,7 M$, 2026-2028, Plan nature 2030. Entreprises de toutes tailles. Paie des experts pour intégrer la biodiversité.</t>
+          <t>Territoire pilote : agglomération de Québec — rempli. Phases admissibles : démarrage, CROISSANCE et repreneuriat. Prêt sans intérêt, sans frais de dossier et sans garantie personnelle. Sélection à deux niveaux : qualités entrepreneuriales et projet, puis productivité, innovation, commercialisation et développement durable. Montant fixé au cas par cas par le comité d'approbation — non publié.</t>
         </is>
       </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
-          <t>Fit exceptionnel : la thèse d'affaires entière de Lasclay est de rendre l'asclépiade viable pour restaurer l'habitat du monarque.</t>
+          <t>Aucune mise de fonds et zéro intérêt : c'est le seul financement de la liste qui attaque directement les 53 074 $ d'intérêts. Organisme en phase pilote (objectif : 48 entreprises sur 6 ans) qui cherche des dossiers vitrines — la notoriété de Lasclay joue pour. DEUX RÉSERVES : le prêt vise à renforcer les fonds propres pour lever du financement institutionnel, or ils sont à -254 035 $, ce qui est autant l'argument que le risque devant le comité ; et l'accompagnement par un mentor est obligatoire pendant toute la durée du contrat. À CLARIFIER AVEC EUX : le prêt est-il consenti à l'entreprise ou à l'entrepreneur personnellement ?</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>https://faqdd.qc.ca/programmes/fonds-ecoleader-biodiversite/</t>
+          <t>https://www.iqph.org/</t>
         </is>
       </c>
     </row>
@@ -1189,12 +1193,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>PSCE — Volet 2 : diversification et consolidation hors Québec</t>
+          <t>Fonds Écoleader — Biodiversité</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>FAQDD / MELCCFP</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1204,7 +1208,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>International</t>
+          <t>Mission</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1212,35 +1216,35 @@
           <t>Contribution non remboursable</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>Reporté</t>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>60000</v>
+        <v>40000</v>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>25 % du coût total</t>
+          <t>Environ 25 %</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>N'accepte pas les demandes</t>
+          <t>Modalités non publiées</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>Surveiller la réouverture — vérifier aussi s'il a été remplacé</t>
+          <t>Annoncé pour le printemps 2026, en retard — relancer chaque mois au 418 692-5888</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>FY27-FY28</t>
+          <t>FY27 T3</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
@@ -1250,17 +1254,17 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>SEUIL TOUT JUSTE FRANCHI : le programme exige un chiffre d'affaires supérieur à 1 M$ et inférieur ou égal à 50 M$. FY2025 était à 879 125 $, sous le seuil ; FY2026 clôture à 1 081 908 $, au-dessus. Exige aussi que plus de 40 % de la viabilité repose sur des revenus autonomes — largement rempli.</t>
+          <t>Enveloppe de 5,7 M$, 2026-2028, Plan nature 2030. Entreprises de toutes tailles. Paie des experts pour intégrer la biodiversité.</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>60 000 $ par entreprise par année, non remboursable, pour la diversification de marchés hors Québec. Aucune exigence de secteur manufacturier. C'est le meilleur complément à CanExport : le fédéral et le provincial financent le même effort d'export sans se cumuler sur la même dépense. À surveiller activement — le seuil de 1 M$ vient d'être franchi, ce qui rend Lasclay admissible pour la première fois.</t>
+          <t>Fit exceptionnel : la thèse d'affaires entière de Lasclay est de rendre l'asclépiade viable pour restaurer l'habitat du monarque.</t>
         </is>
       </c>
       <c r="Q11" s="9" t="inlineStr">
         <is>
-          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/programme-de-soutien-la-commercialisation-et-lexportation/psce-volet-2</t>
+          <t>https://faqdd.qc.ca/programmes/fonds-ecoleader-biodiversite/</t>
         </is>
       </c>
     </row>
@@ -1270,78 +1274,78 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>PARI — Programme emploi jeunesse</t>
+          <t>PSCE — Volet 2 : diversification et consolidation hors Québec</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Conseil national de recherches Canada</t>
+          <t>Investissement Québec</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>International</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
+          <t>Contribution non remboursable</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Part du salaire</t>
+          <t>25 % du coût total</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>N'accepte pas les demandes</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>À déposer avec le dossier PARI principal</t>
+          <t>Surveiller la réouverture — vérifier aussi s'il a été remplacé</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>FY27 T1</t>
+          <t>FY27-FY28</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>Diplômé postsecondaire de 15 à 30 ans, 6 à 12 mois, minimum 30 h/semaine. Volets R-D, génie, multimédia ou étude de marché.</t>
+          <t>SEUIL TOUT JUSTE FRANCHI : le programme exige un chiffre d'affaires supérieur à 1 M$ et inférieur ou égal à 50 M$. FY2025 était à 879 125 $, sous le seuil ; FY2026 clôture à 1 081 908 $, au-dessus. Exige aussi que plus de 40 % de la viabilité repose sur des revenus autonomes — largement rempli.</t>
         </is>
       </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
-          <t>Le volet étude de marché couvre exactement le travail d'expansion américaine par régions réceptives.</t>
+          <t>60 000 $ par entreprise par année, non remboursable, pour la diversification de marchés hors Québec. Aucune exigence de secteur manufacturier. C'est le meilleur complément à CanExport : le fédéral et le provincial financent le même effort d'export sans se cumuler sur la même dépense. À surveiller activement — le seuil de 1 M$ vient d'être franchi, ce qui rend Lasclay admissible pour la première fois.</t>
         </is>
       </c>
       <c r="Q12" s="9" t="inlineStr">
         <is>
-          <t>https://nrc.canada.ca/fr/soutien-linnovation-technologique/largent-pari-cnrc-embaucher-jeunes-diplomes</t>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/programme-de-soutien-la-commercialisation-et-lexportation/psce-volet-2</t>
         </is>
       </c>
     </row>
@@ -1351,17 +1355,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Mitacs Accélération</t>
+          <t>PARI — Programme emploi jeunesse</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Mitacs + MEIE</t>
+          <t>Conseil national de recherches Canada</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Fédéral et Québec</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1371,7 +1375,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
+          <t>Subvention salariale</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -1380,49 +1384,49 @@
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>7500</v>
+        <v>15000</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>30000</v>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Environ 50 %</t>
+          <t>Part du salaire</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>Via un conseiller Mitacs en développement des affaires</t>
+          <t>À déposer avec le dossier PARI principal</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>FY27 T3</t>
+          <t>FY27 T1</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>Stagiaires universitaires, postdoctoraux et chercheurs intégrés à un projet d'innovation en entreprise. Financement partagé MEIE, entreprise, fédéral.</t>
+          <t>Diplômé postsecondaire de 15 à 30 ans, 6 à 12 mois, minimum 30 h/semaine. Volets R-D, génie, multimédia ou étude de marché.</t>
         </is>
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>Le meilleur véhicule pour faire caractériser la fibre en laboratoire : conductivité thermique du produit fini, tenue à la compression, comportement à l'humidité.</t>
+          <t>Le volet étude de marché couvre exactement le travail d'expansion américaine par régions réceptives.</t>
         </is>
       </c>
       <c r="Q13" s="9" t="inlineStr">
         <is>
-          <t>https://www.mitacs.ca/fr-ca/</t>
+          <t>https://nrc.canada.ca/fr/soutien-linnovation-technologique/largent-pari-cnrc-embaucher-jeunes-diplomes</t>
         </is>
       </c>
     </row>
@@ -1432,17 +1436,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Accès aux talents</t>
+          <t>Mitacs Accélération</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Produits naturels Canada</t>
+          <t>Mitacs + MEIE</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Fédéral et Québec</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1455,20 +1459,20 @@
           <t>Subvention</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
-        <v>20000</v>
+        <v>7500</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>75000</v>
+        <v>30000</v>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>60 % du salaire</t>
+          <t>Environ 50 %</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -1478,12 +1482,12 @@
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Demande à tout moment</t>
+          <t>Via un conseiller Mitacs en développement des affaires</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>FY28 T1</t>
+          <t>FY27 T3</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -1493,17 +1497,17 @@
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>40 % du salaire d'un nouvel employé, maximum 75 000 $. Exige d'être membre de la grappe de l'innovation en produits naturels.</t>
+          <t>Stagiaires universitaires, postdoctoraux et chercheurs intégrés à un projet d'innovation en entreprise. Financement partagé MEIE, entreprise, fédéral.</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
         <is>
-          <t>La définition de PNC — bioproduits et durabilité — couvre l'asclépiade. La collaboration cosmétique autour de l'huile de graine est le candidat naturel.</t>
+          <t>Le meilleur véhicule pour faire caractériser la fibre en laboratoire : conductivité thermique du produit fini, tenue à la compression, comportement à l'humidité.</t>
         </is>
       </c>
       <c r="Q14" s="9" t="inlineStr">
         <is>
-          <t>https://www.naturalproductscanada.com/fr/programmes/programme-daccess-aux-talents/</t>
+          <t>https://www.mitacs.ca/fr-ca/</t>
         </is>
       </c>
     </row>
@@ -1513,43 +1517,43 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Allonger les périodes d'emploi</t>
+          <t>Accès aux talents</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Services Québec (MESS)</t>
+          <t>Produits naturels Canada</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Hors piliers</t>
+          <t>R&amp;D</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>3000</v>
+        <v>20000</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>13000</v>
+        <v>75000</v>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>50 % du salaire</t>
+          <t>60 % du salaire</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -1559,32 +1563,32 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>Via un conseiller aux entreprises Services Québec</t>
+          <t>Demande à tout moment</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>FY27 T1</t>
+          <t>FY28 T1</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
         <is>
-          <t>50 % du salaire brut, maximum 6 500 $ par emploi par année. Le projet doit être récurrent et allonger la saison de travail.</t>
+          <t>40 % du salaire d'un nouvel employé, maximum 75 000 $. Exige d'être membre de la grappe de l'innovation en produits naturels.</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
-          <t>Toujours valable, mais l'argument se déplace : la saisonnalité qui reste à lisser est celle de l'expédition et du service client, pas celle de la production. Le développement de la gamme été demeure le projet de diversification que le programme finance.</t>
+          <t>La définition de PNC — bioproduits et durabilité — couvre l'asclépiade. La collaboration cosmétique autour de l'huile de graine est le candidat naturel.</t>
         </is>
       </c>
       <c r="Q15" s="9" t="inlineStr">
         <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/allonger-periodes-emploi</t>
+          <t>https://www.naturalproductscanada.com/fr/programmes/programme-daccess-aux-talents/</t>
         </is>
       </c>
     </row>
@@ -1594,12 +1598,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Mesure de formation de la main-d'œuvre</t>
+          <t>Allonger les périodes d'emploi</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Services Québec</t>
+          <t>Services Québec (MESS)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1614,7 +1618,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
+          <t>Subvention salariale</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1623,14 +1627,14 @@
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>15000</v>
+        <v>13000</v>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Variable</t>
+          <t>50 % du salaire</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -1640,7 +1644,7 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>Via le même conseiller</t>
+          <t>Via un conseiller aux entreprises Services Québec</t>
         </is>
       </c>
       <c r="M16" s="5" t="inlineStr">
@@ -1655,17 +1659,17 @@
       </c>
       <c r="O16" s="8" t="inlineStr">
         <is>
-          <t>Couvre les frais de formateur et les salaires des employés pendant la formation, y compris pour la transformation numérique.</t>
+          <t>50 % du salaire brut, maximum 6 500 $ par emploi par année. Le projet doit être récurrent et allonger la saison de travail.</t>
         </is>
       </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>Équipe réduite à environ 2 personnes après le virage : la montée en compétences des restants tient les opérations.</t>
+          <t>Toujours valable, mais l'argument se déplace : la saisonnalité qui reste à lisser est celle de l'expédition et du service client, pas celle de la production. Le développement de la gamme été demeure le projet de diversification que le programme finance.</t>
         </is>
       </c>
       <c r="Q16" s="9" t="inlineStr">
         <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/former-main-oeuvre/developper-competences</t>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/allonger-periodes-emploi</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1679,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Concertation pour l'emploi (GRH)</t>
+          <t>Mesure de formation de la main-d'œuvre</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1707,7 +1711,7 @@
         <v>2000</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
@@ -1736,17 +1740,17 @@
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>Honoraires professionnels : diagnostic RH, mandat de consultation, coaching de gestion, accompagnement en gestion du changement.</t>
+          <t>Couvre les frais de formateur et les salaires des employés pendant la formation, y compris pour la transformation numérique.</t>
         </is>
       </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
-          <t>Le virage manufacturier 2025-2026, avec mises à pied et redéfinition des rôles, est une gestion du changement documentée.</t>
+          <t>Équipe réduite à environ 2 personnes après le virage : la montée en compétences des restants tient les opérations.</t>
         </is>
       </c>
       <c r="Q17" s="9" t="inlineStr">
         <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/obtenir-conseils</t>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/former-main-oeuvre/developper-competences</t>
         </is>
       </c>
     </row>
@@ -1756,27 +1760,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Stages pratiques PSPE (Magnet, CTIC, TECHNATION, BioTalent)</t>
+          <t>Concertation pour l'emploi (GRH)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>ESDC via partenaires sectoriels</t>
+          <t>Services Québec</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Ventes</t>
+          <t>Hors piliers</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
+          <t>Subvention</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1785,29 +1789,29 @@
         </is>
       </c>
       <c r="H18" s="7" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Salaire avancé, remboursé après</t>
+          <t>Variable</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>Ouvert par trimestre scolaire</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>Premier arrivé, premier servi</t>
+          <t>Via le même conseiller</t>
         </is>
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>FY27 T2</t>
+          <t>FY27 T1</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
@@ -1817,17 +1821,17 @@
       </c>
       <c r="O18" s="8" t="inlineStr">
         <is>
-          <t>5 000 $ par stage d'étudiant postsecondaire. Postes à composante numérique ou technologique priorisés.</t>
+          <t>Honoraires professionnels : diagnostic RH, mandat de consultation, coaching de gestion, accompagnement en gestion du changement.</t>
         </is>
       </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
-          <t>Un poste en commerce électronique, automatisation ou données qualifie sans forcer. Déposer chez UN SEUL partenaire : c'est la même enveloppe fédérale.</t>
+          <t>Le virage manufacturier 2025-2026, avec mises à pied et redéfinition des rôles, est une gestion du changement documentée.</t>
         </is>
       </c>
       <c r="Q18" s="9" t="inlineStr">
         <is>
-          <t>https://swpprogram.ca/fr/</t>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/aide-gestion-ressources-humaines/obtenir-conseils</t>
         </is>
       </c>
     </row>
@@ -1837,12 +1841,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Emplois d'été Canada</t>
+          <t>Stages pratiques PSPE (Magnet, CTIC, TECHNATION, BioTalent)</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Emploi et Développement social Canada</t>
+          <t>ESDC via partenaires sectoriels</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1852,7 +1856,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Hors piliers</t>
+          <t>Ventes</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -1866,24 +1870,24 @@
         </is>
       </c>
       <c r="H19" s="7" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>50 % du salaire minimum</t>
+          <t>Salaire avancé, remboursé après</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>Fermé — rouvre vers novembre 2026</t>
+          <t>Ouvert par trimestre scolaire</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>Date limite attendue ~11 décembre 2026 pour l'été 2027</t>
+          <t>Premier arrivé, premier servi</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
@@ -1898,17 +1902,17 @@
       </c>
       <c r="O19" s="8" t="inlineStr">
         <is>
-          <t>Secteur privé : jusqu'à 50 % du salaire minimum en vigueur. Jeunes de 15 à 30 ans, postes à temps plein.</t>
+          <t>5 000 $ par stage d'étudiant postsecondaire. Postes à composante numérique ou technologique priorisés.</t>
         </is>
       </c>
       <c r="P19" s="8" t="inlineStr">
         <is>
-          <t>Renfort d'atelier ou d'expédition pour la production estivale, en amont de la saison hivernale.</t>
+          <t>Un poste en commerce électronique, automatisation ou données qualifie sans forcer. Déposer chez UN SEUL partenaire : c'est la même enveloppe fédérale.</t>
         </is>
       </c>
       <c r="Q19" s="9" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/emploi-developpement-social/services/financement/emplois-ete-canada.html</t>
+          <t>https://swpprogram.ca/fr/</t>
         </is>
       </c>
     </row>
@@ -1918,12 +1922,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Riipen — Level UP</t>
+          <t>Emplois d'été Canada</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Riipen</t>
+          <t>Emploi et Développement social Canada</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -1933,12 +1937,12 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Ventes</t>
+          <t>Hors piliers</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
+          <t>Subvention salariale</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1947,24 +1951,24 @@
         </is>
       </c>
       <c r="H20" s="7" t="n">
-        <v>1400</v>
+        <v>3000</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>4200</v>
+        <v>8000</v>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Aucune</t>
+          <t>50 % du salaire minimum</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Fermé — rouvre vers novembre 2026</t>
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>Par semestre universitaire</t>
+          <t>Date limite attendue ~11 décembre 2026 pour l'été 2027</t>
         </is>
       </c>
       <c r="M20" s="5" t="inlineStr">
@@ -1979,17 +1983,17 @@
       </c>
       <c r="O20" s="8" t="inlineStr">
         <is>
-          <t>1 400 $ par étudiant. Projets de 60 heures sur 2 à 8 semaines, encadrés par un enseignant.</t>
+          <t>Secteur privé : jusqu'à 50 % du salaire minimum en vigueur. Jeunes de 15 à 30 ans, postes à temps plein.</t>
         </is>
       </c>
       <c r="P20" s="8" t="inlineStr">
         <is>
-          <t>Format parfait pour des mandats bornés : localisation des fiches produits pour les marchés américains, refonte du guide de plantation, analyse de saisonnalité.</t>
+          <t>Renfort d'atelier ou d'expédition pour la production estivale, en amont de la saison hivernale.</t>
         </is>
       </c>
       <c r="Q20" s="9" t="inlineStr">
         <is>
-          <t>https://fr.riipen.com/levelup/employers</t>
+          <t>https://www.canada.ca/fr/emploi-developpement-social/services/financement/emplois-ete-canada.html</t>
         </is>
       </c>
     </row>
@@ -1999,78 +2003,78 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Capitale-Innovation</t>
+          <t>Riipen — Level UP</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Ville de Québec</t>
+          <t>Riipen</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>International</t>
+          <t>Ventes</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Contribution non remboursable</t>
-        </is>
-      </c>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
-        <v>50000</v>
+        <v>1400</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>500000</v>
+        <v>4200</v>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>50 %, puis 60 % au-delà de 250 k$</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>Volet ouvert (page à jour le 8 juillet 2026)</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>Enveloppe Vision Québec 2030 possiblement fermée depuis le 31 mars 2026 — à faire trancher</t>
+          <t>Par semestre universitaire</t>
         </is>
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>FY28 T3</t>
+          <t>FY27 T2</t>
         </is>
       </c>
       <c r="N21" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O21" s="8" t="inlineStr">
         <is>
-          <t>Secteur « Manufacturier, matériaux, transformation industrielle » explicitement admissible. Siège dans l'agglomération de Québec : rempli (1286 av. de la Ronde).</t>
+          <t>1 400 $ par étudiant. Projets de 60 heures sur 2 à 8 semaines, encadrés par un enseignant.</t>
         </is>
       </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
-          <t>Le plus gros non remboursable accessible localement. Exige la preuve de détention de la PI. Cumul de toute aide publique plafonné à 70 %.</t>
+          <t>Format parfait pour des mandats bornés : localisation des fiches produits pour les marchés américains, refonte du guide de plantation, analyse de saisonnalité.</t>
         </is>
       </c>
       <c r="Q21" s="9" t="inlineStr">
         <is>
-          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/innovation/capitale-innovation.aspx</t>
+          <t>https://fr.riipen.com/levelup/employers</t>
         </is>
       </c>
     </row>
@@ -2080,27 +2084,27 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Validation de principe</t>
+          <t>Capitale-Innovation</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Produits naturels Canada</t>
+          <t>Ville de Québec</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Municipal</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>International</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Financement remboursable</t>
+          <t>Contribution non remboursable</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -2112,26 +2116,26 @@
         <v>50000</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>250000</v>
+        <v>500000</v>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>60 %</t>
+          <t>50 %, puis 60 % au-delà de 250 k$</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Volet ouvert (page à jour le 8 juillet 2026)</t>
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>Demande à tout moment</t>
+          <t>Enveloppe Vision Québec 2030 possiblement fermée depuis le 31 mars 2026 — à faire trancher</t>
         </is>
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>FY28 T4</t>
+          <t>FY28 T3</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
@@ -2141,17 +2145,17 @@
       </c>
       <c r="O22" s="8" t="inlineStr">
         <is>
-          <t>40 % des coûts, maximum 250 000 $. PNC cherche un potentiel de 10 à 15 M$ de revenus annuels — un cran au-dessus de la trajectoire de Lasclay.</t>
+          <t>Secteur « Manufacturier, matériaux, transformation industrielle » explicitement admissible. Siège dans l'agglomération de Québec : rempli (1286 av. de la Ronde).</t>
         </is>
       </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
-          <t>Réserve sérieuse sur le critère de potentiel de revenus. À tenter seulement si le volet cosmétique prend de l'ampleur.</t>
+          <t>Le plus gros non remboursable accessible localement. Exige la preuve de détention de la PI. Cumul de toute aide publique plafonné à 70 %.</t>
         </is>
       </c>
       <c r="Q22" s="9" t="inlineStr">
         <is>
-          <t>https://www.naturalproductscanada.com/fr/programmes/programme-validation-de-principe/</t>
+          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/innovation/capitale-innovation.aspx</t>
         </is>
       </c>
     </row>
@@ -2161,27 +2165,27 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Bons d'accompagnement à la croissance</t>
+          <t>Validation de principe</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Ville de Québec</t>
+          <t>Produits naturels Canada</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Ventes</t>
+          <t>R&amp;D</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Contribution</t>
+          <t>Financement remboursable</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -2190,49 +2194,49 @@
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>5000</v>
+        <v>50000</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>20000</v>
+        <v>250000</v>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Variable</t>
+          <t>60 %</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>Ouvert, dépôt en continu</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>Aucune date de tombée</t>
+          <t>Demande à tout moment</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>FY27 T4</t>
+          <t>FY28 T4</t>
         </is>
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Élevé</t>
         </is>
       </c>
       <c r="O23" s="8" t="inlineStr">
         <is>
-          <t>Exclut explicitement les commerces opérant UNIQUEMENT en ligne.</t>
+          <t>40 % des coûts, maximum 250 000 $. PNC cherche un potentiel de 10 à 15 M$ de revenus annuels — un cran au-dessus de la trajectoire de Lasclay.</t>
         </is>
       </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
-          <t>L'atelier de Limoilou et la transformation de l'isolant sortent Lasclay de l'exclusion, mais il faut l'énoncer clairement dans la demande.</t>
+          <t>Réserve sérieuse sur le critère de potentiel de revenus. À tenter seulement si le volet cosmétique prend de l'ampleur.</t>
         </is>
       </c>
       <c r="Q23" s="9" t="inlineStr">
         <is>
-          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/productivite/bons-accompagnement.aspx</t>
+          <t>https://www.naturalproductscanada.com/fr/programmes/programme-validation-de-principe/</t>
         </is>
       </c>
     </row>
@@ -2242,78 +2246,78 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Panorama</t>
+          <t>Bons d'accompagnement à la croissance</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>Ville de Québec</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Municipal</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>International</t>
+          <t>Ventes</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Prêt</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="inlineStr">
-        <is>
-          <t>Reporté</t>
+          <t>Contribution</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>250000</v>
+        <v>5000</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>1000000</v>
+        <v>20000</v>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Capacité de crédit</t>
+          <t>Variable</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Ouvert, dépôt en continu</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>Après retour à la rentabilité</t>
+          <t>Aucune date de tombée</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>FY27 T4</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O24" s="8" t="inlineStr">
         <is>
-          <t>Prêt de fonds de roulement export, moratoire de capital de 24 mois, SANS sûreté ni caution corporative ou personnelle. EXCLUT les États-Unis.</t>
+          <t>Exclut explicitement les commerces opérant UNIQUEMENT en ligne.</t>
         </is>
       </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
-          <t>Structure rare et attrayante, mais hors de portée avec un avoir de -254 035 $ et 584 320 $ de dette portant intérêt.</t>
+          <t>L'atelier de Limoilou et la transformation de l'isolant sortent Lasclay de l'exclusion, mais il faut l'énoncer clairement dans la demande.</t>
         </is>
       </c>
       <c r="Q24" s="9" t="inlineStr">
         <is>
-          <t>https://exportation.investquebec.com/solutions</t>
+          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/productivite/bons-accompagnement.aspx</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2327,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>ESSOR — Volet 4 (internationalisation)</t>
+          <t>Panorama</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -2343,7 +2347,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Prêt ou garantie</t>
+          <t>Prêt</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
@@ -2352,10 +2356,10 @@
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>50000</v>
+        <v>250000</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>500000</v>
+        <v>1000000</v>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
@@ -2369,12 +2373,12 @@
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>Si le développement É.-U. passe par de la distribution locale</t>
+          <t>Après retour à la rentabilité</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>FY28 T4</t>
+          <t>FY28</t>
         </is>
       </c>
       <c r="N25" s="5" t="inlineStr">
@@ -2384,17 +2388,17 @@
       </c>
       <c r="O25" s="8" t="inlineStr">
         <is>
-          <t>Vise les stratégies d'internationalisation complexes : entités, entrepôts, chaînes d'approvisionnement à l'étranger.</t>
+          <t>Prêt de fonds de roulement export, moratoire de capital de 24 mois, SANS sûreté ni caution corporative ou personnelle. EXCLUT les États-Unis.</t>
         </is>
       </c>
       <c r="P25" s="8" t="inlineStr">
         <is>
-          <t>Ne se justifie pas tant que les États-Unis sont servis par expédition directe depuis Québec.</t>
+          <t>Structure rare et attrayante, mais hors de portée avec un avoir de -254 035 $ et 584 320 $ de dette portant intérêt.</t>
         </is>
       </c>
       <c r="Q25" s="9" t="inlineStr">
         <is>
-          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-linternationalisation-des-entreprises</t>
+          <t>https://exportation.investquebec.com/solutions</t>
         </is>
       </c>
     </row>
@@ -2404,12 +2408,12 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Programme Innovation — Volet 1</t>
+          <t>ESSOR — Volet 4 (internationalisation)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>MEIE</t>
+          <t>Investissement Québec</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -2419,12 +2423,12 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>International</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
+          <t>Prêt ou garantie</t>
         </is>
       </c>
       <c r="G26" s="11" t="inlineStr">
@@ -2440,22 +2444,22 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>25 % en argent</t>
+          <t>Capacité de crédit</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>N'accepte pas les demandes</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>Surveiller la réouverture</t>
+          <t>Si le développement É.-U. passe par de la distribution locale</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>FY28 T4</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
@@ -2465,17 +2469,17 @@
       </c>
       <c r="O26" s="8" t="inlineStr">
         <is>
-          <t>Jusqu'à 500 000 $ par entreprise. Contribution privée EN ARGENT d'au moins 25 % des dépenses admissibles.</t>
+          <t>Vise les stratégies d'internationalisation complexes : entités, entrepôts, chaînes d'approvisionnement à l'étranger.</t>
         </is>
       </c>
       <c r="P26" s="8" t="inlineStr">
         <is>
-          <t>ABSENT du répertoire Innoveici : c'est un angle mort du premier tri. Pendant provincial de Capitale-Innovation, à surveiller activement.</t>
+          <t>Ne se justifie pas tant que les États-Unis sont servis par expédition directe depuis Québec.</t>
         </is>
       </c>
       <c r="Q26" s="9" t="inlineStr">
         <is>
-          <t>https://www.economie.gouv.qc.ca/bibliotheques/programmes/aide-financiere/programme-innovation</t>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-linternationalisation-des-entreprises</t>
         </is>
       </c>
     </row>
@@ -2485,17 +2489,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Programme canadien de l'innovation à l'international</t>
+          <t>Programme Innovation — Volet 1</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Affaires mondiales Canada</t>
+          <t>MEIE</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Fédéral</t>
+          <t>Québec</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -2508,30 +2512,30 @@
           <t>Subvention</t>
         </is>
       </c>
-      <c r="G27" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>15000</v>
+        <v>50000</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>600000</v>
+        <v>500000</v>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>50 %</t>
+          <t>25 % en argent</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>Dépôt ad hoc</t>
+          <t>N'accepte pas les demandes</t>
         </is>
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>Ad hoc</t>
+          <t>Surveiller la réouverture</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
@@ -2546,17 +2550,17 @@
       </c>
       <c r="O27" s="8" t="inlineStr">
         <is>
-          <t>Exige un partenaire de R-D au Brésil, en Chine, en Inde, en Israël ou en Corée du Sud.</t>
+          <t>Jusqu'à 500 000 $ par entreprise. Contribution privée EN ARGENT d'au moins 25 % des dépenses admissibles.</t>
         </is>
       </c>
       <c r="P27" s="8" t="inlineStr">
         <is>
-          <t>La liste de pays ne recoupe pas la chaîne d'approvisionnement actuelle, qui passe par la Tunisie. À garder en veille seulement.</t>
+          <t>ABSENT du répertoire Innoveici : c'est un angle mort du premier tri. Pendant provincial de Capitale-Innovation, à surveiller activement.</t>
         </is>
       </c>
       <c r="Q27" s="9" t="inlineStr">
         <is>
-          <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/programmes-soutien/programme-canadien-innovation-international.html</t>
+          <t>https://www.economie.gouv.qc.ca/bibliotheques/programmes/aide-financiere/programme-innovation</t>
         </is>
       </c>
     </row>
@@ -2566,12 +2570,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>CERI — Expansion des entreprises et productivité</t>
+          <t>Programme canadien de l'innovation à l'international</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Développement économique Canada</t>
+          <t>Affaires mondiales Canada</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -2581,12 +2585,12 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Ventes</t>
+          <t>R&amp;D</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Contribution remboursable à 0 %</t>
+          <t>Subvention</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
@@ -2595,10 +2599,10 @@
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>250000</v>
+        <v>600000</v>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
@@ -2607,17 +2611,17 @@
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Dépôt ad hoc</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>En continu</t>
+          <t>Ad hoc</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>FY27 T4</t>
+          <t>FY28</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
@@ -2627,17 +2631,17 @@
       </c>
       <c r="O28" s="8" t="inlineStr">
         <is>
-          <t>Aucun seuil de revenus, contrairement à l'IRRT. Secteurs admissibles : manufacturier, transformation alimentaire, TIC, sciences de la vie. Commerce de détail EXPLICITEMENT EXCLU.</t>
+          <t>Exige un partenaire de R-D au Brésil, en Chine, en Inde, en Israël ou en Corée du Sud.</t>
         </is>
       </c>
       <c r="P28" s="8" t="inlineStr">
         <is>
-          <t>RÉTROGRADÉ. Je recommandais de cadrer le dossier en manufacturier ; ce n'est plus la posture de l'entreprise, et le commerce de détail est un secteur exclu par DEC. Le seul crochet honnête qui reste est la transformation de l'isolant, qui se poursuit au Québec (91 336 $ de salaires de production aux livres en FY2026). À ne tenter que si DEC confirme d'avance que cette activité suffit à qualifier. Le volet commercialisation et développement des marchés du programme reste, lui, parfaitement aligné.</t>
+          <t>La liste de pays ne recoupe pas la chaîne d'approvisionnement actuelle, qui passe par la Tunisie. À garder en veille seulement.</t>
         </is>
       </c>
       <c r="Q28" s="9" t="inlineStr">
         <is>
-          <t>https://www.canada.ca/fr/developpement-economique-regions-quebec/financement-services/expansion-des-entreprises-et-productivite.html</t>
+          <t>https://www.deleguescommerciaux.gc.ca/fr/nos-solutions/programmes-soutien/programme-canadien-innovation-international.html</t>
         </is>
       </c>
     </row>
@@ -2647,27 +2651,27 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Prêts aux entreprises</t>
+          <t>CERI — Expansion des entreprises et productivité</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Ville de Québec</t>
+          <t>Développement économique Canada</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Municipal</t>
+          <t>Fédéral</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Hors piliers</t>
+          <t>Ventes</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Prêt</t>
+          <t>Contribution remboursable à 0 %</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
@@ -2679,16 +2683,16 @@
         <v>25000</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>150000</v>
+        <v>250000</v>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Capacité de crédit</t>
+          <t>50 %</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L29" s="5" t="inlineStr">
@@ -2698,27 +2702,27 @@
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>FY28 T1</t>
+          <t>FY27 T4</t>
         </is>
       </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Élevé</t>
         </is>
       </c>
       <c r="O29" s="8" t="inlineStr">
         <is>
-          <t>Quatre volets : démarrage, amélioration et transformation, croissance et expansion, relève.</t>
+          <t>Aucun seuil de revenus, contrairement à l'IRRT. Secteurs admissibles : manufacturier, transformation alimentaire, TIC, sciences de la vie. Commerce de détail EXPLICITEMENT EXCLU.</t>
         </is>
       </c>
       <c r="P29" s="8" t="inlineStr">
         <is>
-          <t>Le volet « amélioration et transformation » colle au virage manufacturier. La capacité de crédit reste à démontrer avec un avoir négatif.</t>
+          <t>RÉTROGRADÉ. Je recommandais de cadrer le dossier en manufacturier ; ce n'est plus la posture de l'entreprise, et le commerce de détail est un secteur exclu par DEC. Le seul crochet honnête qui reste est la transformation de l'isolant, qui se poursuit au Québec (91 336 $ de salaires de production aux livres en FY2026). À ne tenter que si DEC confirme d'avance que cette activité suffit à qualifier. Le volet commercialisation et développement des marchés du programme reste, lui, parfaitement aligné.</t>
         </is>
       </c>
       <c r="Q29" s="9" t="inlineStr">
         <is>
-          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/autres/prets-aux-entreprises/index.aspx</t>
+          <t>https://www.canada.ca/fr/developpement-economique-regions-quebec/financement-services/expansion-des-entreprises-et-productivite.html</t>
         </is>
       </c>
     </row>
@@ -2728,17 +2732,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Pratiques RH (FCCQ) et RH éclair! (FCEI)</t>
+          <t>Prêts aux entreprises</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>FCCQ / FCEI</t>
+          <t>Ville de Québec</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Québec et fédéral</t>
+          <t>Municipal</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -2748,23 +2752,23 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Service gratuit</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
+          <t>Prêt</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>Aucune</t>
+          <t>Capacité de crédit</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -2779,27 +2783,27 @@
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>FY27 T1</t>
+          <t>FY28 T1</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O30" s="8" t="inlineStr">
         <is>
-          <t>Accès gratuit à des conseils RH et juridiques, à une bibliothèque de modèles et de politiques.</t>
+          <t>Quatre volets : démarrage, amélioration et transformation, croissance et expansion, relève.</t>
         </is>
       </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
-          <t>Zéro dollar en jeu, mais utile pour sécuriser les contrats et les politiques après une réduction d'effectifs.</t>
+          <t>Le volet « amélioration et transformation » colle au virage manufacturier. La capacité de crédit reste à démontrer avec un avoir négatif.</t>
         </is>
       </c>
       <c r="Q30" s="9" t="inlineStr">
         <is>
-          <t>https://pratiquesrh.com/</t>
+          <t>https://www.ville.quebec.qc.ca/gens_affaires/financement/autres/prets-aux-entreprises/index.aspx</t>
         </is>
       </c>
     </row>
@@ -2809,17 +2813,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Contrat d'intégration au travail</t>
+          <t>Pratiques RH (FCCQ) et RH éclair! (FCEI)</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Services Québec</t>
+          <t>FCCQ / FCEI</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Québec</t>
+          <t>Québec et fédéral</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -2829,7 +2833,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Subvention salariale</t>
+          <t>Service gratuit</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -2838,19 +2842,19 @@
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Part du salaire</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="L31" s="5" t="inlineStr">
@@ -2860,7 +2864,7 @@
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>FY28</t>
+          <t>FY27 T1</t>
         </is>
       </c>
       <c r="N31" s="5" t="inlineStr">
@@ -2870,17 +2874,17 @@
       </c>
       <c r="O31" s="8" t="inlineStr">
         <is>
-          <t>Soutien au salaire pour compenser un écart de productivité, plus couverture de l'adaptation du poste.</t>
+          <t>Accès gratuit à des conseils RH et juridiques, à une bibliothèque de modèles et de politiques.</t>
         </is>
       </c>
       <c r="P31" s="8" t="inlineStr">
         <is>
-          <t>Pertinent pour l'assemblage, l'emballage de semences et l'expédition, où les tâches se découpent bien.</t>
+          <t>Zéro dollar en jeu, mais utile pour sécuriser les contrats et les politiques après une réduction d'effectifs.</t>
         </is>
       </c>
       <c r="Q31" s="9" t="inlineStr">
         <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/recruter/contrat-integration-travail</t>
+          <t>https://pratiquesrh.com/</t>
         </is>
       </c>
     </row>
@@ -2890,12 +2894,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Fonds économie circulaire</t>
+          <t>Contrat d'intégration au travail</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Fondaction</t>
+          <t>Services Québec</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -2905,33 +2909,33 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Mission</t>
+          <t>Hors piliers</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Capital (dilution)</t>
-        </is>
-      </c>
-      <c r="G32" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+          <t>Subvention salariale</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>100000</v>
+        <v>3000</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>500000</v>
+        <v>20000</v>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>Dilution du capital</t>
+          <t>Part du salaire</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>Ouvert</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
@@ -2946,22 +2950,22 @@
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O32" s="8" t="inlineStr">
         <is>
-          <t>Cible les jeunes entreprises en phase de démarrage dont le modèle repose sur la circularité. C'est du capital, pas de la subvention.</t>
+          <t>Soutien au salaire pour compenser un écart de productivité, plus couverture de l'adaptation du poste.</t>
         </is>
       </c>
       <c r="P32" s="8" t="inlineStr">
         <is>
-          <t>Les semences issues de la transformation de la soie et la gamme « Les Imparfaits » sont de la circularité réelle. À ne considérer que si l'ouverture du capital devient une option assumée.</t>
+          <t>Pertinent pour l'assemblage, l'emballage de semences et l'expédition, où les tâches se découpent bien.</t>
         </is>
       </c>
       <c r="Q32" s="9" t="inlineStr">
         <is>
-          <t>https://www.fondaction.com/entreprise/fonds-economie-circulaire/</t>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/administrer-gerer/embauche-gestion-personnel/recruter/contrat-integration-travail</t>
         </is>
       </c>
     </row>
@@ -2971,12 +2975,12 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>ICI on recycle +</t>
+          <t>Fonds économie circulaire</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Recyc-Québec</t>
+          <t>Fondaction</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -2991,23 +2995,23 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Attestation (clé d'accès)</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
+          <t>Capital (dilution)</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>-350</v>
+        <v>100000</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>350 $ de frais d'inscription</t>
+          <t>Dilution du capital</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
@@ -3027,22 +3031,22 @@
       </c>
       <c r="N33" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Élevé</t>
         </is>
       </c>
       <c r="O33" s="8" t="inlineStr">
         <is>
-          <t>N'octroie pas d'aide. Écocondition OBLIGATOIRE, au niveau « Mise en œuvre », pour le versement final de plusieurs aides de Recyc-Québec.</t>
+          <t>Cible les jeunes entreprises en phase de démarrage dont le modèle repose sur la circularité. C'est du capital, pas de la subvention.</t>
         </is>
       </c>
       <c r="P33" s="8" t="inlineStr">
         <is>
-          <t>C'est une clé, pas une source. Environ 350 $ pour déverrouiller les enveloppes de Recyc-Québec et crédibiliser les appels d'offres corporatifs.</t>
+          <t>Les semences issues de la transformation de la soie et la gamme « Les Imparfaits » sont de la circularité réelle. À ne considérer que si l'ouverture du capital devient une option assumée.</t>
         </is>
       </c>
       <c r="Q33" s="9" t="inlineStr">
         <is>
-          <t>https://www.recyc-quebec.gouv.qc.ca/entreprises-organismes/performer/programme-ici-on-recycle-plus/</t>
+          <t>https://www.fondaction.com/entreprise/fonds-economie-circulaire/</t>
         </is>
       </c>
     </row>
@@ -3052,12 +3056,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>grand V — accompagnement technologique</t>
+          <t>ICI on recycle +</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>Recyc-Québec</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -3067,12 +3071,12 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Hors piliers</t>
+          <t>Mission</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Service (sans dette)</t>
+          <t>Attestation (clé d'accès)</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -3081,19 +3085,19 @@
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>0</v>
+        <v>-350</v>
       </c>
       <c r="I34" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Aucune</t>
+          <t>350 $ de frais d'inscription</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Ouvert</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
@@ -3103,7 +3107,7 @@
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>FY27 T3</t>
+          <t>FY28</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
@@ -3113,17 +3117,17 @@
       </c>
       <c r="O34" s="8" t="inlineStr">
         <is>
-          <t>Jusqu'à 100 heures d'experts en innovation. Séparable du volet financement, qui lui est hors de portée.</t>
+          <t>N'octroie pas d'aide. Écocondition OBLIGATOIRE, au niveau « Mise en œuvre », pour le versement final de plusieurs aides de Recyc-Québec.</t>
         </is>
       </c>
       <c r="P34" s="8" t="inlineStr">
         <is>
-          <t>RÉTROGRADÉ : l'offre porte surtout sur la sélection d'équipements, la reconfiguration d'usine et le prototypage, qui ne sont plus des chantiers actifs. Reste utile pour l'amélioration de produits si un volet R&amp;D s'y prête.</t>
+          <t>C'est une clé, pas une source. Environ 350 $ pour déverrouiller les enveloppes de Recyc-Québec et crédibiliser les appels d'offres corporatifs.</t>
         </is>
       </c>
       <c r="Q34" s="9" t="inlineStr">
         <is>
-          <t>https://grandv.investquebec.com/</t>
+          <t>https://www.recyc-quebec.gouv.qc.ca/entreprises-organismes/performer/programme-ici-on-recycle-plus/</t>
         </is>
       </c>
     </row>
@@ -3133,7 +3137,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>ESSOR — Volet 1 (études préalables)</t>
+          <t>grand V — accompagnement technologique</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -3153,7 +3157,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Subvention</t>
+          <t>Service (sans dette)</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -3162,14 +3166,14 @@
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>Variable</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
@@ -3179,32 +3183,32 @@
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>Dépôt en continu</t>
+          <t>En continu</t>
         </is>
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>FY28 T3</t>
+          <t>FY27 T3</t>
         </is>
       </c>
       <c r="N35" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O35" s="8" t="inlineStr">
         <is>
-          <t>Études de faisabilité, diagnostic numérique, plan numérique. Entreprises de tous secteurs.</t>
+          <t>Jusqu'à 100 heures d'experts en innovation. Séparable du volet financement, qui lui est hors de portée.</t>
         </is>
       </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
-          <t>Porte d'entrée à faible risque avant tout projet d'équipement financé par ESSOR volet 2.</t>
+          <t>RÉTROGRADÉ : l'offre porte surtout sur la sélection d'équipements, la reconfiguration d'usine et le prototypage, qui ne sont plus des chantiers actifs. Reste utile pour l'amélioration de produits si un volet R&amp;D s'y prête.</t>
         </is>
       </c>
       <c r="Q35" s="9" t="inlineStr">
         <is>
-          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-la-concretisation-de-projets-dinvestissement</t>
+          <t>https://grandv.investquebec.com/</t>
         </is>
       </c>
     </row>
@@ -3214,12 +3218,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>C3i — investissement et innovation</t>
+          <t>ESSOR — Volet 1 (études préalables)</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Revenu Québec</t>
+          <t>Investissement Québec</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -3234,58 +3238,58 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Crédit d'impôt remboursable</t>
-        </is>
-      </c>
-      <c r="G36" s="10" t="inlineStr">
-        <is>
-          <t>À valider</t>
+          <t>Subvention</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>25000</v>
+        <v>50000</v>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>L'achat d'équipement lui-même</t>
+          <t>Variable</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>En vigueur</t>
+          <t>Ouvert en continu</t>
         </is>
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>Avec la déclaration fiscale annuelle</t>
+          <t>Dépôt en continu</t>
         </is>
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>FY27-FY28</t>
+          <t>FY28 T3</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O36" s="8" t="inlineStr">
         <is>
-          <t>15 % à 25 % du coût du matériel de fabrication et transformation (catégorie 53) et des logiciels de gestion, utilisé au Québec 730 jours consécutifs.</t>
+          <t>Études de faisabilité, diagnostic numérique, plan numérique. Entreprises de tous secteurs.</t>
         </is>
       </c>
       <c r="P36" s="8" t="inlineStr">
         <is>
-          <t>RÉTROGRADÉ : le crédit porte sur l'ACQUISITION de matériel de fabrication, et il n'y a plus de programme d'achat d'équipement. Ne se cumule pas avec le CRIC sur la même dépense. À réactiver seulement si un achat d'équipement revient au plan.</t>
+          <t>Porte d'entrée à faible risque avant tout projet d'équipement financé par ESSOR volet 2.</t>
         </is>
       </c>
       <c r="Q36" s="9" t="inlineStr">
         <is>
-          <t>https://www.revenuquebec.ca/fr/entreprises/impots/impot-des-societes/credits-dimpot-des-societes/</t>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/appui-la-concretisation-de-projets-dinvestissement</t>
         </is>
       </c>
     </row>
@@ -3295,12 +3299,12 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Primo-adoptants</t>
+          <t>C3i — investissement et innovation</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>MEIE</t>
+          <t>Revenu Québec</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -3315,58 +3319,58 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Subvention (versée au partenaire)</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>Admissible</t>
+          <t>Crédit d'impôt remboursable</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>20 % en espèces</t>
+          <t>L'achat d'équipement lui-même</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>Appel de projets</t>
+          <t>En vigueur</t>
         </is>
       </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>Surveiller les appels</t>
+          <t>Avec la déclaration fiscale annuelle</t>
         </is>
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>FY28 T3</t>
+          <t>FY27-FY28</t>
         </is>
       </c>
       <c r="N37" s="5" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="O37" s="8" t="inlineStr">
         <is>
-          <t>Lasclay serait le primo-adoptant, pas le bénéficiaire. La contribution du gouvernement va à la startup ; le primo-adoptant met 20 % en espèces.</t>
+          <t>15 % à 25 % du coût du matériel de fabrication et transformation (catégorie 53) et des logiciels de gestion, utilisé au Québec 730 jours consécutifs.</t>
         </is>
       </c>
       <c r="P37" s="8" t="inlineStr">
         <is>
-          <t>Manière peu coûteuse de faire tester sur la fibre des équipements d'automatisation ou de vision par ordinateur pour le contrôle qualité.</t>
+          <t>RÉTROGRADÉ : le crédit porte sur l'ACQUISITION de matériel de fabrication, et il n'y a plus de programme d'achat d'équipement. Ne se cumule pas avec le CRIC sur la même dépense. À réactiver seulement si un achat d'équipement revient au plan.</t>
         </is>
       </c>
       <c r="Q37" s="9" t="inlineStr">
         <is>
-          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/liste-partielle-aide-financiere/appels-projets-innovation/appel-primo-adoptants</t>
+          <t>https://www.revenuquebec.ca/fr/entreprises/impots/impot-des-societes/credits-dimpot-des-societes/</t>
         </is>
       </c>
     </row>
@@ -3376,12 +3380,12 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>ESSOR — Volet 2 (productivité et expansion)</t>
+          <t>Primo-adoptants</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>MEIE</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -3396,58 +3400,58 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Contribution remboursable ou garantie</t>
-        </is>
-      </c>
-      <c r="G38" s="11" t="inlineStr">
-        <is>
-          <t>Reporté</t>
+          <t>Subvention (versée au partenaire)</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>500000</v>
+        <v>0</v>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>Capacité de crédit</t>
+          <t>20 % en espèces</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>Ouvert en continu</t>
+          <t>Appel de projets</t>
         </is>
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>Après un exercice FY2027 positif</t>
+          <t>Surveiller les appels</t>
         </is>
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>FY28 T1</t>
+          <t>FY28 T3</t>
         </is>
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>Élevé</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="O38" s="8" t="inlineStr">
         <is>
-          <t>Exige de démontrer un potentiel de hausse de rentabilité ou de masse salariale. Honoraires de gestion d'au moins 0,5 % du montant accordé.</t>
+          <t>Lasclay serait le primo-adoptant, pas le bénéficiaire. La contribution du gouvernement va à la startup ; le primo-adoptant met 20 % en espèces.</t>
         </is>
       </c>
       <c r="P38" s="8" t="inlineStr">
         <is>
-          <t>Le raisonnement reste juste, il est prématuré d'un ou deux exercices. Rouvrir le dossier sur des états financiers montrant un redressement.</t>
+          <t>Manière peu coûteuse de faire tester sur la fibre des équipements d'automatisation ou de vision par ordinateur pour le contrôle qualité.</t>
         </is>
       </c>
       <c r="Q38" s="9" t="inlineStr">
         <is>
-          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/essor-volet-2</t>
+          <t>https://www.quebec.ca/entreprises-et-travailleurs-autonomes/liste-partielle-aide-financiere/appels-projets-innovation/appel-primo-adoptants</t>
         </is>
       </c>
     </row>
@@ -3457,201 +3461,282 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
+          <t>ESSOR — Volet 2 (productivité et expansion)</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Investissement Québec</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Québec</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Hors piliers</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Contribution remboursable ou garantie</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>Reporté</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>Capacité de crédit</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>Ouvert en continu</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>Après un exercice FY2027 positif</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>FY28 T1</t>
+        </is>
+      </c>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>Élevé</t>
+        </is>
+      </c>
+      <c r="O39" s="8" t="inlineStr">
+        <is>
+          <t>Exige de démontrer un potentiel de hausse de rentabilité ou de masse salariale. Honoraires de gestion d'au moins 0,5 % du montant accordé.</t>
+        </is>
+      </c>
+      <c r="P39" s="8" t="inlineStr">
+        <is>
+          <t>Le raisonnement reste juste, il est prématuré d'un ou deux exercices. Rouvrir le dossier sur des états financiers montrant un redressement.</t>
+        </is>
+      </c>
+      <c r="Q39" s="9" t="inlineStr">
+        <is>
+          <t>https://www.investquebec.com/fr/financement/programmes-gouvernementaux/essor/essor-volet-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="58" customHeight="1">
+      <c r="A40" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
           <t>grand V — financement</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>Investissement Québec</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>Québec</t>
         </is>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>Hors piliers</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t>Prêt à terme</t>
         </is>
       </c>
-      <c r="G39" s="11" t="inlineStr">
+      <c r="G40" s="11" t="inlineStr">
         <is>
           <t>Reporté</t>
         </is>
       </c>
-      <c r="H39" s="7" t="n">
+      <c r="H40" s="7" t="n">
         <v>250000</v>
       </c>
-      <c r="I39" s="7" t="n">
+      <c r="I40" s="7" t="n">
         <v>1000000</v>
       </c>
-      <c r="J39" s="5" t="inlineStr">
+      <c r="J40" s="5" t="inlineStr">
         <is>
           <t>Capacité de crédit</t>
         </is>
       </c>
-      <c r="K39" s="5" t="inlineStr">
+      <c r="K40" s="5" t="inlineStr">
         <is>
           <t>Ouvert en continu</t>
         </is>
       </c>
-      <c r="L39" s="5" t="inlineStr">
+      <c r="L40" s="5" t="inlineStr">
         <is>
           <t>Après un exercice FY2027 positif</t>
         </is>
       </c>
-      <c r="M39" s="5" t="inlineStr">
+      <c r="M40" s="5" t="inlineStr">
         <is>
           <t>FY28 T1</t>
         </is>
       </c>
-      <c r="N39" s="5" t="inlineStr">
+      <c r="N40" s="5" t="inlineStr">
         <is>
           <t>Élevé</t>
         </is>
       </c>
-      <c r="O39" s="8" t="inlineStr">
+      <c r="O40" s="8" t="inlineStr">
         <is>
           <t>Prêt MINIMUM de 250 000 $, moratoire de capital jusqu'à 48 mois. Devant -254 035 $ de capitaux propres et 584 320 $ de dette, l'analyse de crédit bloque.</t>
         </is>
       </c>
-      <c r="P39" s="8" t="inlineStr">
+      <c r="P40" s="8" t="inlineStr">
         <is>
           <t>C'était le levier identifié pour remplacer Merchant Growth et Shopify Capital. Il reste le bon levier, mais pas avant un redressement.</t>
         </is>
       </c>
-      <c r="Q39" s="9" t="inlineStr">
+      <c r="Q40" s="9" t="inlineStr">
         <is>
           <t>https://grandv.investquebec.com/</t>
         </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>Potentiel total, verdict « Admissible » seulement</t>
-        </is>
-      </c>
-      <c r="H41" s="13">
-        <f>SUMIF($G$5:$G$39,"Admissible",H5:H39)</f>
-        <v>121550</v>
-      </c>
-      <c r="I41" s="13">
-        <f>SUMIF($G$5:$G$39,"Admissible",I5:I39)</f>
-        <v>465200</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>Potentiel total, « Admissible » + « À valider »</t>
+          <t>Potentiel total, verdict « Admissible » seulement</t>
         </is>
       </c>
       <c r="H42" s="13">
-        <f>SUMIF($G$5:$G$39,"Admissible",H5:H39)+SUMIF($G$5:$G$39,"À valider",H5:H39)</f>
-        <v>436550</v>
+        <f>SUMIF($G$5:$G$40,"Admissible",H5:H40)</f>
+        <v>131550</v>
       </c>
       <c r="I42" s="13">
-        <f>SUMIF($G$5:$G$39,"Admissible",I5:I39)+SUMIF($G$5:$G$39,"À valider",I5:I39)</f>
-        <v>2905200</v>
+        <f>SUMIF($G$5:$G$40,"Admissible",I5:I40)</f>
+        <v>590200</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="12" t="inlineStr">
         <is>
+          <t>Potentiel total, « Admissible » + « À valider »</t>
+        </is>
+      </c>
+      <c r="H43" s="13">
+        <f>SUMIF($G$5:$G$40,"Admissible",H5:H40)+SUMIF($G$5:$G$40,"À valider",H5:H40)</f>
+        <v>446550</v>
+      </c>
+      <c r="I43" s="13">
+        <f>SUMIF($G$5:$G$40,"Admissible",I5:I40)+SUMIF($G$5:$G$40,"À valider",I5:I40)</f>
+        <v>3030200</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
           <t>Dont admissible SANS aucune mise de fonds</t>
         </is>
       </c>
-      <c r="H43" s="13">
-        <f>SUMIFS(H5:H39,$G$5:$G$39,"Admissible",$J$5:$J$39,"Aucune")</f>
-        <v>46400</v>
-      </c>
-      <c r="I43" s="13">
-        <f>SUMIFS(I5:I39,$G$5:$G$39,"Admissible",$J$5:$J$39,"Aucune")</f>
-        <v>74200</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="14" t="inlineStr">
+      <c r="H44" s="13">
+        <f>SUMIFS(H5:H40,$G$5:$G$40,"Admissible",$J$5:$J$40,"Aucune")</f>
+        <v>56400</v>
+      </c>
+      <c r="I44" s="13">
+        <f>SUMIFS(I5:I40,$G$5:$G$40,"Admissible",$J$5:$J$40,"Aucune")</f>
+        <v>199200</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>Notes de lecture</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="26" customHeight="1">
-      <c r="B46" s="15" t="inlineStr">
-        <is>
-          <t>• Montants min et max : fourchettes réalistes pour un dossier Lasclay, pas les plafonds théoriques des programmes. Ils servent à prioriser, pas à budgéter. Cas particulier du rang 5 (IQPH) : l'organisme ne publie aucun montant. La fourchette de 15 à 30 k$ est INFÉRÉE de son objectif public — 48 entreprises et 12 M$ d'investissements générés sur 6 ans, avec un effet de levier annoncé jusqu'à 10 fois — et doit être confirmée auprès d'eux.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="26" customHeight="1">
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>• Verdicts : « Admissible » = tous les critères publiés sont rencontrés. « À valider » = un critère dépend d'un arbitrage, d'un cadrage ou d'une confirmation de l'organisme. « Reporté » = admissible sur papier, hors de portée financièrement aujourd'hui.</t>
+          <t>• Montants min et max : fourchettes réalistes pour un dossier Lasclay, pas les plafonds théoriques des programmes. Ils servent à prioriser, pas à budgéter. Cas particulier du rang 5 (IQPH) : l'organisme ne publie aucun montant. La fourchette de 15 à 30 k$ est INFÉRÉE de son objectif public — 48 entreprises et 12 M$ d'investissements générés sur 6 ans, avec un effet de levier annoncé jusqu'à 10 fois — et doit être confirmée auprès d'eux.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="26" customHeight="1">
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>• La contrainte dominante n'est pas l'admissibilité, c'est la mise de fonds : trésorerie de -2 060 $ et marge EDC utilisée à 94,8 %. D'où la priorité donnée aux crédits d'impôt et aux subventions salariales, qui remboursent des dépenses déjà engagées.</t>
+          <t>• Verdicts : « Admissible » = tous les critères publiés sont rencontrés. « À valider » = un critère dépend d'un arbitrage, d'un cadrage ou d'une confirmation de l'organisme. « Reporté » = admissible sur papier, hors de portée financièrement aujourd'hui.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="26" customHeight="1">
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>• Colonne Pilier : le classement suit les quatre priorités de l'entreprise — mission, ventes, international, R&amp;D. Lasclay n'est plus manufacturier pour le moment, ce qui fait reculer tout ce qui repose sur l'achat d'équipement, la productivité d'usine ou le statut de secteur manufacturier : C3i, ESSOR, grand V, Primo-adoptants et DEC Expansion.</t>
+          <t>• La contrainte dominante n'est pas l'admissibilité, c'est la mise de fonds : trésorerie de -2 060 $ et marge EDC utilisée à 94,8 %. D'où la priorité donnée aux crédits d'impôt et aux subventions salariales, qui remboursent des dépenses déjà engagées.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="26" customHeight="1">
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>• Nuance à tenir : les livres portent encore 91 336 $ de salaires de production et 135 851 $ d'équipements en FY2026. Ne pas se déclarer manufacturier devant un programme et s'en réclamer devant un autre — choisir une version et la tenir.</t>
+          <t>• Colonne Pilier : le classement suit les quatre priorités de l'entreprise — mission, ventes, international, R&amp;D. Lasclay n'est plus manufacturier pour le moment, ce qui fait reculer tout ce qui repose sur l'achat d'équipement, la productivité d'usine ou le statut de secteur manufacturier : C3i, ESSOR, grand V, Primo-adoptants et DEC Expansion.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="26" customHeight="1">
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>• Colonne Pilier : le classement suit les quatre priorités de l'entreprise, soit mission, ventes, international et R&amp;D. Lasclay n'est plus manufacturier pour le moment, ce qui fait reculer tout ce qui repose sur l'achat d'équipement, la productivité d'usine ou le statut de secteur manufacturier : C3i, ESSOR, grand V, Primo-adoptants et DEC Expansion.</t>
+          <t>• Nuance à tenir : les livres portent encore 91 336 $ de salaires de production et 135 851 $ d'équipements en FY2026. Ne pas se déclarer manufacturier devant un programme et s'en réclamer devant un autre — choisir une version et la tenir.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="26" customHeight="1">
       <c r="B52" s="15" t="inlineStr">
         <is>
-          <t>• Nuance à tenir : les livres portent encore 91 336 $ de salaires de production et 135 851 $ d'équipements en FY2026. Ne pas se déclarer non manufacturier devant un programme et s'en réclamer devant un autre. Choisir une version et la tenir.</t>
+          <t>• Colonne Pilier : le classement suit les quatre priorités de l'entreprise, soit mission, ventes, international et R&amp;D. Lasclay n'est plus manufacturier pour le moment, ce qui fait reculer tout ce qui repose sur l'achat d'équipement, la productivité d'usine ou le statut de secteur manufacturier : C3i, ESSOR, grand V, Primo-adoptants et DEC Expansion.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="26" customHeight="1">
       <c r="B53" s="15" t="inlineStr">
         <is>
+          <t>• Nuance à tenir : les livres portent encore 91 336 $ de salaires de production et 135 851 $ d'équipements en FY2026. Ne pas se déclarer non manufacturier devant un programme et s'en réclamer devant un autre. Choisir une version et la tenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="26" customHeight="1">
+      <c r="B54" s="15" t="inlineStr">
+        <is>
           <t>• Sources vérifiées le 5 août 2026 aux sites officiels des organismes. Les statuts de programme changent sans préavis : revalider avant tout dépôt.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q39"/>
+  <autoFilter ref="A4:Q40"/>
   <mergeCells count="10">
-    <mergeCell ref="B49:I49"/>
     <mergeCell ref="B52:I52"/>
+    <mergeCell ref="B53:I53"/>
     <mergeCell ref="B48:I48"/>
-    <mergeCell ref="B53:I53"/>
     <mergeCell ref="B47:I47"/>
     <mergeCell ref="B51:I51"/>
+    <mergeCell ref="B54:I54"/>
     <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="B46:I46"/>
     <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="B49:I49"/>
     <mergeCell ref="B50:I50"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4344,7 +4429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4402,37 +4487,41 @@
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>31 août 2026, 12 h</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>2 SEPTEMBRE 2026, 23 h 59</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>FY2026 — clôture</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Décider : déposer CanExport PME maintenant pour un marché européen, ou bâtir le dossier pour février 2027</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>CanExport PME</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Fermeture d'appel</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr"/>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Redéposer la candidature TELUS #AidonsNosPME. Le dossier gagnant existe déjà, l'effort est faible et il n'y a aucune mise de fonds</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>TELUS #AidonsNosPME</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>LIMITE FERME</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>Prochaine édition dans un an. Jusqu'à 125 000 $ et un prix du public de 25 000 $ par vote.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>31 août 2026</t>
+          <t>31 août 2026, 12 h</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -4442,17 +4531,17 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Clôture de l'exercice FY2026</t>
+          <t>Décider : déposer CanExport PME maintenant pour un marché européen, ou bâtir le dossier pour février 2027</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CanExport PME</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Comptable</t>
+          <t>Fermeture d'appel</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr"/>
@@ -4460,49 +4549,45 @@
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Août 2026</t>
+          <t>31 août 2026</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Immédiat</t>
+          <t>FY2026 — clôture</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Confirmer avec le comptable si la réclamation RS&amp;DE de FY2025 a été produite</t>
+          <t>Clôture de l'exercice FY2026</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>RS&amp;DE / CRIC</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Vérification</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Perte définitive du crédit après le 28 février 2027</t>
-        </is>
-      </c>
+          <t>Comptable</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr"/>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Sept — nov 2026</t>
+          <t>Août 2026</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>FY2027 T1</t>
+          <t>Immédiat</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Produire la réclamation RS&amp;DE et CRIC de FY2026 dans la foulée des états financiers</t>
+          <t>Confirmer avec le comptable si la réclamation RS&amp;DE de FY2025 a été produite</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -4512,10 +4597,14 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Dépôt</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr"/>
+          <t>Vérification</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Perte définitive du crédit après le 28 février 2027</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
@@ -4530,24 +4619,20 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Déposer la candidature : business model canvas, sommaire exécutif, extrait du registre des entreprises et CV, à candidature@iqph.org</t>
+          <t>Produire la réclamation RS&amp;DE et CRIC de FY2026 dans la foulée des états financiers</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Prêt d'honneur IQPH</t>
+          <t>RS&amp;DE / CRIC</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Dépôt en continu</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Sans intérêt et sans garantie — aucune autre source de la liste n'offre ça</t>
-        </is>
-      </c>
+          <t>Dépôt</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr"/>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -4562,20 +4647,24 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Demander un conseiller CTI et poser d'emblée la question de l'arbitrage avec la RS&amp;DE</t>
+          <t>Déposer la candidature : business model canvas, sommaire exécutif, extrait du registre des entreprises et CV, à candidature@iqph.org</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>PARI-CNRC</t>
+          <t>Prêt d'honneur IQPH</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Premier contact</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr"/>
+          <t>Dépôt en continu</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Sans intérêt et sans garantie — aucune autre source de la liste n'offre ça</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
@@ -4590,12 +4679,12 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Un seul appel à Services Québec pour couvrir les trois mesures (emploi, formation, GRH)</t>
+          <t>Demander un conseiller CTI et poser d'emblée la question de l'arbitrage avec la RS&amp;DE</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Services Québec</t>
+          <t>PARI-CNRC</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -4618,125 +4707,121 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Faire trancher par la Ville : l'enveloppe Capitale-Innovation est-elle disponible ou en attente du renouvellement de l'entente ?</t>
+          <t>Un seul appel à Services Québec pour couvrir les trois mesures (emploi, formation, GRH)</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Capitale-Innovation</t>
+          <t>Services Québec</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Vérification</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Un dossier de 500 k$ monté pour rien</t>
-        </is>
-      </c>
+          <t>Premier contact</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr"/>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>~11 décembre 2026</t>
+          <t>Sept — nov 2026</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>FY2027 T2</t>
+          <t>FY2027 T1</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Déposer la demande pour l'été 2027</t>
+          <t>Faire trancher par la Ville : l'enveloppe Capitale-Innovation est-elle disponible ou en attente du renouvellement de l'entente ?</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Emplois d'été Canada</t>
+          <t>Capitale-Innovation</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Fermeture d'appel</t>
+          <t>Vérification</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Report d'un an complet</t>
+          <t>Un dossier de 500 k$ monté pour rien</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>~4 février 2027</t>
+          <t>~11 mars 2027</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
+          <t>FY2027 T3</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Déposer au volet Réussite inc. — prix national de 25 000 $ — et aux Phénix de l'environnement, dépôt avant le 8 mars</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>OSEntreprendre et Phénix</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Fermeture d'appel</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Cycle annuel ; report d'un an</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>~11 décembre 2026</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
           <t>FY2027 T2</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Déposer dès les premiers jours : premier arrivé, premier servi</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>CanExport PME 2027-28</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Ouverture d'appel</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Épuisement de l'enveloppe en cours d'exercice</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>28 FÉVRIER 2027</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>FY2027 T2</t>
-        </is>
-      </c>
-      <c r="C15" s="17" t="inlineStr">
-        <is>
-          <t>DATE LIMITE ABSOLUE de production de la réclamation RS&amp;DE pour FY2025</t>
-        </is>
-      </c>
-      <c r="D15" s="17" t="inlineStr">
-        <is>
-          <t>RS&amp;DE FY2025</t>
-        </is>
-      </c>
-      <c r="E15" s="17" t="inlineStr">
-        <is>
-          <t>LIMITE FERME</t>
-        </is>
-      </c>
-      <c r="F15" s="17" t="inlineStr">
-        <is>
-          <t>Perte définitive. L'ARC n'a aucun pouvoir discrétionnaire.</t>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Déposer la demande pour l'été 2027</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Emplois d'été Canada</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Fermeture d'appel</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Report d'un an complet</t>
         </is>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Déc 2026 — fév 2027</t>
+          <t>~4 février 2027</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -4746,73 +4831,81 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Déposer les subventions salariales de stage pour l'hiver et l'été</t>
+          <t>Déposer dès les premiers jours : premier arrivé, premier servi</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>PSPE et Riipen</t>
+          <t>CanExport PME 2027-28</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Par trimestre</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr"/>
+          <t>Ouverture d'appel</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Épuisement de l'enveloppe en cours d'exercice</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Mars — août 2027</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>FY2027 T3-T4</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Monter le dossier DEC Expansion en le cadrant comme manufacturier, pas comme commerce en ligne</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>CERI Expansion</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Dépôt en continu</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr"/>
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>28 FÉVRIER 2027</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>FY2027 T2</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>DATE LIMITE ABSOLUE de production de la réclamation RS&amp;DE pour FY2025</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>RS&amp;DE FY2025</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>LIMITE FERME</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>Perte définitive. L'ARC n'a aucun pouvoir discrétionnaire.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Mars — août 2027</t>
+          <t>Déc 2026 — fév 2027</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>FY2027 T3</t>
+          <t>FY2027 T2</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Demander l'accompagnement technologique seul, sans le volet financement</t>
+          <t>Déposer les subventions salariales de stage pour l'hiver et l'été</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>grand V</t>
+          <t>PSPE et Riipen</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Dépôt en continu</t>
+          <t>Par trimestre</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr"/>
@@ -4820,34 +4913,30 @@
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Mensuel, à partir de sept 2026</t>
+          <t>Mars — août 2027</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>FY2027 — continu</t>
+          <t>FY2027 T3-T4</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Relancer le FAQDD au 418 692-5888 jusqu'à publication des modalités</t>
+          <t>Monter le dossier DEC Expansion en le cadrant comme manufacturier, pas comme commerce en ligne</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Écoleader Biodiversité</t>
+          <t>CERI Expansion</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Veille active</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Enveloppe de 5,7 M$ épuisée avant d'avoir déposé</t>
-        </is>
-      </c>
+          <t>Dépôt en continu</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr"/>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -4862,12 +4951,12 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Monter un stage de caractérisation de la fibre en laboratoire</t>
+          <t>Demander l'accompagnement technologique seul, sans le volet financement</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Mitacs</t>
+          <t>grand V</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -4880,59 +4969,59 @@
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Sept — nov 2027</t>
+          <t>Mensuel, à partir de sept 2026</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>FY2028 T1</t>
+          <t>FY2027 — continu</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Produire la réclamation RS&amp;DE et CRIC de FY2027 dès la clôture</t>
+          <t>Relancer le FAQDD au 418 692-5888 jusqu'à publication des modalités</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>RS&amp;DE / CRIC</t>
+          <t>Écoleader Biodiversité</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Dépôt</t>
+          <t>Veille active</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Le réflexe doit devenir annuel</t>
+          <t>Enveloppe de 5,7 M$ épuisée avant d'avoir déposé</t>
         </is>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Sept — nov 2027</t>
+          <t>Mars — août 2027</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>FY2028 T1</t>
+          <t>FY2027 T3</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Rouvrir le dossier IQ si FY2027 revient au positif : grand V, ESSOR volet 2</t>
+          <t>Monter un stage de caractérisation de la fibre en laboratoire</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Investissement Québec</t>
+          <t>Mitacs</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Réévaluation</t>
+          <t>Dépôt en continu</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr"/>
@@ -4940,242 +5029,302 @@
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>~Février 2028</t>
+          <t>Sept — nov 2027</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>FY2028 T2</t>
+          <t>FY2028 T1</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Déposer sur un deuxième marché européen si le premier a produit des résultats</t>
+          <t>Produire la réclamation RS&amp;DE et CRIC de FY2027 dès la clôture</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>CanExport PME 2028-29</t>
+          <t>RS&amp;DE / CRIC</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Ouverture d'appel</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr"/>
+          <t>Dépôt</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Le réflexe doit devenir annuel</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>28 FÉVRIER 2028</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="inlineStr">
-        <is>
-          <t>FY2028 T2</t>
-        </is>
-      </c>
-      <c r="C24" s="17" t="inlineStr">
-        <is>
-          <t>DATE LIMITE ABSOLUE de production de la réclamation RS&amp;DE pour FY2026</t>
-        </is>
-      </c>
-      <c r="D24" s="17" t="inlineStr">
-        <is>
-          <t>RS&amp;DE FY2026</t>
-        </is>
-      </c>
-      <c r="E24" s="17" t="inlineStr">
-        <is>
-          <t>LIMITE FERME</t>
-        </is>
-      </c>
-      <c r="F24" s="17" t="inlineStr">
-        <is>
-          <t>Perte définitive de 45 k$ à 70 k$.</t>
-        </is>
-      </c>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Sept — nov 2027</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>FY2028 T1</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Rouvrir le dossier IQ si FY2027 revient au positif : grand V, ESSOR volet 2</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Investissement Québec</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Réévaluation</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr"/>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Mars — août 2028</t>
+          <t>~Février 2028</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>FY2028 T3</t>
+          <t>FY2028 T2</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Déposer Capitale-Innovation si l'entente est renouvelée et la trésorerie reconstituée</t>
+          <t>Déposer sur un deuxième marché européen si le premier a produit des résultats</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Capitale-Innovation</t>
+          <t>CanExport PME 2028-29</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Dépôt</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>C'est le dossier de fin de plan, pas de début</t>
-        </is>
-      </c>
+          <t>Ouverture d'appel</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr"/>
     </row>
     <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>Mars — août 2028</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>FY2028 T3</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Financer les études de faisabilité en amont d'un projet d'équipement</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>ESSOR volet 1</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>Dépôt en continu</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="inlineStr"/>
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>28 FÉVRIER 2028</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>FY2028 T2</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>DATE LIMITE ABSOLUE de production de la réclamation RS&amp;DE pour FY2026</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>RS&amp;DE FY2026</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>LIMITE FERME</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Perte définitive de 45 k$ à 70 k$.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Août 2028</t>
+          <t>Mars — août 2028</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>FY2028 — clôture</t>
+          <t>FY2028 T3</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Revalider le seuil de 2 M$ : une catégorie entière de programmes fédéraux s'ouvre au-delà</t>
+          <t>Déposer Capitale-Innovation si l'entente est renouvelée et la trésorerie reconstituée</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Divers fédéral</t>
+          <t>Capitale-Innovation</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>Jalon</t>
-        </is>
-      </c>
-      <c r="F27" s="8" t="inlineStr"/>
+          <t>Dépôt</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>C'est le dossier de fin de plan, pas de début</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Trimestriel, dès sept 2026</t>
+          <t>Mars — août 2028</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>FY2027 — continu</t>
+          <t>FY2028 T3</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Vérifier la réouverture du PSCE volet 2, et s'il a été remplacé par un autre véhicule d'aide à l'export</t>
+          <t>Financer les études de faisabilité en amont d'un projet d'équipement</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>PSCE volet 2</t>
+          <t>ESSOR volet 1</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Veille active</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>60 000 $ non remboursables ; Lasclay vient tout juste de franchir le seuil de 1 M$</t>
-        </is>
-      </c>
+          <t>Dépôt en continu</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr"/>
     </row>
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Trimestriel, dès sept 2026</t>
+          <t>Août 2028</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>FY2027 — continu</t>
+          <t>FY2028 — clôture</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Vérifier la réouverture du PSCE volet 2, et s'il a été remplacé par un autre véhicule d'aide à l'export</t>
+          <t>Revalider le seuil de 2 M$ : une catégorie entière de programmes fédéraux s'ouvre au-delà</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>PSCE volet 2</t>
+          <t>Divers fédéral</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>Veille active</t>
-        </is>
-      </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>60 000 $ non remboursables ; le seuil de 1 M$ vient tout juste d'être franchi</t>
-        </is>
-      </c>
+          <t>Jalon</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr"/>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
+          <t>Trimestriel, dès sept 2026</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>FY2027 — continu</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Vérifier la réouverture du PSCE volet 2, et s'il a été remplacé par un autre véhicule d'aide à l'export</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>PSCE volet 2</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>Veille active</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>60 000 $ non remboursables ; Lasclay vient tout juste de franchir le seuil de 1 M$</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Trimestriel, dès sept 2026</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>FY2027 — continu</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Vérifier la réouverture du PSCE volet 2, et s'il a été remplacé par un autre véhicule d'aide à l'export</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>PSCE volet 2</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Veille active</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>60 000 $ non remboursables ; le seuil de 1 M$ vient tout juste d'être franchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
           <t>Janvier 2027, puis janvier 2028</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Annuel</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Rebalayer le répertoire Innoveici : 88 des 208 programmes étaient fermés au 5 août 2026</t>
         </is>
       </c>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="D32" s="8" t="inlineStr">
         <is>
           <t>Veille</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E32" s="8" t="inlineStr">
         <is>
           <t>Récurrent</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr"/>
+      <c r="F32" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5594,7 +5743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -5906,20 +6055,64 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>TELUS — règlement #AidonsNosPME 2026</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Fenêtre du 2 juin au 2 septembre 2026, structure des prix, critère des 100 employés ou moins, absence de clause excluant les anciens lauréats.</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>https://www.telus.com/fr/business/small/campaigns/stand-with-owners-content-rules</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Boîte Missive de Lasclay</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Deux dossiers de concours déjà ouverts : La Ruche et Dans l'Œil du Dragon.</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>(accès interne via le proxy Missive)</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
           <t>QuickBooks Online — Les Produits Lasclay Inc</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Tous les chiffres opposés aux critères : revenus, résultat, trésorerie, capitaux propres, dette, assiette R-D.</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>(accès interne via le Finance Proxy)</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
@@ -5932,4 +6125,410 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="74" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Concours et bourses — la catégorie que les répertoires publics ignorent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Innoveici et les portails gouvernementaux ne recensent que des programmes. Les concours sont ailleurs, n'exigent aucune mise de fonds, et Lasclay en a déjà gagné un.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Concours</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Organisateur</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Prix</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Cycle et date limite</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Ce qu'il faut savoir</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Lien</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>TELUS #AidonsNosPME</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>TELUS Affaires</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>3 grands prix jusqu'à 125 000 $ · 6 prix communautaires de 10 000 $ · 1 prix du public de 25 000 $</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>Annuel · édition 2026 ouverte du 2 juin au 2 SEPTEMBRE 2026</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>DÉJÀ GAGNÉ par Lasclay. Le dossier existe et le récit convainc ce jury. Entreprise canadienne en activité, 100 employés ou moins : rempli. Aucune clause excluant les anciens lauréats dans le règlement consulté, mais à faire confirmer par TELUS avant d'investir du temps. Lauréats annoncés vers le 24 septembre. Le prix du public se gagne par vote — c'est précisément là que la communauté de Lasclay vaut de l'or.</t>
+        </is>
+      </c>
+      <c r="G5" s="24" t="inlineStr">
+        <is>
+          <t>https://www.telus.com/fr/business/small/campaigns/stand-with-owners</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Défi OSEntreprendre — volet Réussite inc.</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>OSEntreprendre / Desjardins</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Prix national de 25 000 $ au Gala des Grands Prix Desjardins</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Annuel · cycle novembre à juin · date limite autour du 11 mars</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Admissible</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Le volet Réussite inc. s'adresse aux entreprises qui reviennent plus de 5 ans après leur première participation, pour raconter leur parcours. Lasclay, fondée en 2020 et passée par un virage manufacturier public, a exactement le récit que ce volet cherche. Pas de sélection locale : la candidature monte directement au régional. Un prix Coup de cœur Développement durable existe aussi.</t>
+        </is>
+      </c>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>https://www.osentreprendre.quebec/defi-osentreprendre/volet/reussite-inc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Les Mercuriades</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Fédération des chambres de commerce du Québec</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>13 catégories + Entreprise de l'année Hydro-Québec. Prestige et visibilité, peu d'argent</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Annuel · gala en mai · candidatures à l'automne</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Le concours d'affaires le plus prestigieux du Québec, 46e édition. Catégories pertinentes : développement durable, innovation, exportation. La valeur est la visibilité et la crédibilité auprès des bailleurs, pas le chèque. Un lauréat ou finaliste Mercuriades pèse dans un dossier IQ ou DEC déposé l'année suivante.</t>
+        </is>
+      </c>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>https://mercuriades.ca/le-concours-admissibilite-et-categories/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="78" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Phénix de l'environnement</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>MELCCFP, Éco Entreprises Québec, Fondation québécoise en environnement</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Prestige, pas de bourse significative</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Annuel · dépôt avant le 8 mars</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Le fit de mission le plus pur de toute la liste : une entreprise qui bâtit une filière économique pour restaurer l'habitat du monarque. Aucun argent direct, mais c'est la reconnaissance qui crédibilise le dossier Écoleader Biodiversité et tout discours d'impact devant un comité. À déposer la même année que la candidature Écoleader.</t>
+        </is>
+      </c>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>https://www.environnement.gouv.qc.ca/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="78" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Concours Ascension</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Jeune Chambre de commerce de Québec / Desjardins Entreprises</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Bourse de plus de 60 000 $ en biens et services, 6 lauréats</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Annuel · finalistes annoncés en janvier · gala en mai</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Concours de pitch réservé aux MEMBRES de la JCCQ dirigeant une jeune entreprise. Deux vérifications avant d'investir : l'adhésion à la JCCQ, et si une entreprise de 6 ans entre encore dans la définition de « jeune entreprise ». La bourse est en biens et services, pas en argent — utile surtout pour des honoraires professionnels.</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>https://www.jccq.qc.ca/concours-ascension</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>La Ruche — sociofinancement</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>La Ruche Québec</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Selon la campagne, avec effet de levier de partenaires qui doublent parfois les mises</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>En continu</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>DOSSIER DÉJÀ OUVERT : un fil de la boîte Missive demande « Souhaitez-vous arrêter vos démarches de financement sur La Ruche ? ». À trancher, dans un sens ou dans l'autre. Le sociofinancement est le véhicule qui exploite le mieux une communauté engagée, et c'est l'actif le plus sous-utilisé de Lasclay après les crédits d'impôt.</t>
+        </is>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>https://laruchequebec.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="78" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Dans l'Œil du Dragon</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Radio-Canada</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Investissement contre participation au capital</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Par saison · appel de candidatures annuel</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>CANDIDATURE DÉJÀ DÉPOSÉE : un fil « Dans l'Œil du Dragon — Suivi de candidature » existe dans la boîte Missive. Ce n'est pas une bourse mais un investissement dilutif, et la valeur réelle est l'exposition télévisuelle nationale. À traiter comme un canal de vente, pas comme du financement.</t>
+        </is>
+      </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>https://ici.radio-canada.ca/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="78" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>FedEx #BackingSmall Canada</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>FedEx Canada</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Environ 100 000 $ répartis entre plusieurs lauréats canadiens</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Irrégulier · édition 2025 tenue, statut 2026 à confirmer</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>À valider</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Le programme américain FedEx Small Business Grants est retiré depuis 2024, mais le volet canadien #BackingSmall a tenu une édition en 2025. À vérifier directement sur fedex.ca : si l'édition 2026 a lieu, le profil de Lasclay — produit physique, expédition, récit fort — est exactement leur cible.</t>
+        </is>
+      </c>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>https://www.fedex.com/en-ca/small-business/backing-small.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>• Les concours n'exigent aucune mise de fonds et ne se remboursent pas. Dans la situation de trésorerie actuelle, c'est leur principal mérite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>• Ce sont des loteries : une dizaine de gagnants pour des milliers de candidatures. Le calcul tient parce que l'effort de dépôt est faible et que Lasclay part avec un avantage réel — un récit qui a déjà converti chez TELUS, une communauté qui vote, et une mission vérifiable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>• Deux dossiers sont déjà ouverts et attendent une décision : La Ruche et Dans l'Œil du Dragon. Les deux apparaissent dans la boîte Missive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>• Ceux qui ne donnent pas d'argent — Mercuriades, Phénix — se déposent quand même : un titre de finaliste change la lecture d'un dossier devant un comité d'IQ, de DEC ou de l'IQPH l'année suivante.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>